<commit_message>
data: datos matinal 2026-05-26 para deploy inicial en Render
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{894F898A-6F88-4188-8FA7-BF1A6BA51B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92AF494B-D70D-4702-B3ED-6579DAB6C4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -580,7 +580,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
@@ -665,28 +666,28 @@
         <v>22</v>
       </c>
       <c r="H2">
-        <v>10868000</v>
+        <v>11232000</v>
       </c>
       <c r="I2">
-        <v>301735.19</v>
+        <v>2580714.09</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2413881.54</v>
+        <v>2884327.51</v>
       </c>
       <c r="L2">
-        <v>22.21</v>
+        <v>25.68</v>
       </c>
       <c r="M2">
-        <v>100578.4</v>
+        <v>151806.71</v>
       </c>
       <c r="N2">
-        <v>503155.47</v>
+        <v>4325642.95</v>
       </c>
       <c r="O2">
-        <v>158486.94</v>
+        <v>-14607.99</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -718,31 +719,31 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>46332000</v>
+        <v>42768000</v>
       </c>
       <c r="I3">
-        <v>16712863.210000001</v>
+        <v>37411681</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>133702905.72</v>
+        <v>41813055.240000002</v>
       </c>
       <c r="L3">
-        <v>288.58</v>
+        <v>97.77</v>
       </c>
       <c r="M3">
-        <v>5570954.4000000004</v>
+        <v>2200687.12</v>
       </c>
       <c r="N3">
-        <v>1410435.09</v>
+        <v>2678159.5</v>
       </c>
       <c r="O3">
-        <v>1909654.48</v>
+        <v>194881.91</v>
       </c>
       <c r="P3">
-        <v>126726.92</v>
+        <v>559362.31999999995</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -771,31 +772,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>107210400</v>
+        <v>103664000</v>
       </c>
       <c r="I4">
-        <v>4388957.41</v>
+        <v>116254731.12</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>35111659.280000001</v>
+        <v>129931758.31</v>
       </c>
       <c r="L4">
-        <v>32.75</v>
+        <v>125.34</v>
       </c>
       <c r="M4">
-        <v>1462985.8</v>
+        <v>6838513.5999999996</v>
       </c>
       <c r="N4">
-        <v>4896259.17</v>
+        <v>-6295365.5599999996</v>
       </c>
       <c r="O4">
-        <v>768296.67</v>
+        <v>1855821.89</v>
       </c>
       <c r="P4">
-        <v>-1051979.74</v>
+        <v>722387.37</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,31 +825,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>6001600</v>
+        <v>8184000</v>
       </c>
       <c r="I5">
-        <v>71108.75</v>
+        <v>11698505.460000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>568869.98</v>
+        <v>13074800.220000001</v>
       </c>
       <c r="L5">
-        <v>9.48</v>
+        <v>159.76</v>
       </c>
       <c r="M5">
-        <v>23702.92</v>
+        <v>688147.38</v>
       </c>
       <c r="N5">
-        <v>282404.34999999998</v>
+        <v>-1757252.73</v>
       </c>
       <c r="O5">
-        <v>98496.57</v>
+        <v>2170700.08</v>
       </c>
       <c r="P5">
-        <v>238871.74</v>
+        <v>3174736.56</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,31 +878,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>60561600</v>
+        <v>40920000</v>
       </c>
       <c r="I6">
-        <v>798687.69</v>
+        <v>24857954.370000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>6389501.54</v>
+        <v>27782419.579999998</v>
       </c>
       <c r="L6">
-        <v>10.55</v>
+        <v>67.89</v>
       </c>
       <c r="M6">
-        <v>266229.23</v>
+        <v>1462232.61</v>
       </c>
       <c r="N6">
-        <v>2845852.97</v>
+        <v>8031022.8200000003</v>
       </c>
       <c r="O6">
-        <v>112369.12</v>
+        <v>2199718.59</v>
       </c>
       <c r="P6">
-        <v>2900325.67</v>
+        <v>203892.01</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -930,31 +931,31 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>55924000</v>
+        <v>79112000</v>
       </c>
       <c r="I7">
-        <v>4218410.37</v>
+        <v>58073722.159999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>33747282.969999999</v>
+        <v>64905924.759999998</v>
       </c>
       <c r="L7">
-        <v>60.34</v>
+        <v>82.04</v>
       </c>
       <c r="M7">
-        <v>1406136.79</v>
+        <v>3416101.3</v>
       </c>
       <c r="N7">
-        <v>2462170.9300000002</v>
+        <v>10519138.92</v>
       </c>
       <c r="O7">
-        <v>422979.15</v>
+        <v>6952588.4199999999</v>
       </c>
       <c r="P7">
-        <v>893324.54</v>
+        <v>1200087.51</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,31 +984,31 @@
         <v>22</v>
       </c>
       <c r="H8">
-        <v>43102400</v>
+        <v>40920000</v>
       </c>
       <c r="I8">
-        <v>7806975.1399999997</v>
+        <v>39577067.18</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>62455801.109999999</v>
+        <v>44233192.740000002</v>
       </c>
       <c r="L8">
-        <v>144.9</v>
+        <v>108.1</v>
       </c>
       <c r="M8">
-        <v>2602325.0499999998</v>
+        <v>2328062.7799999998</v>
       </c>
       <c r="N8">
-        <v>1680734.52</v>
+        <v>671466.41</v>
       </c>
       <c r="O8">
-        <v>36492.080000000002</v>
+        <v>1967561.5</v>
       </c>
       <c r="P8">
-        <v>881013.83</v>
+        <v>230847.97</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1089,10 +1090,10 @@
         <v>41</v>
       </c>
       <c r="H2">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="I2">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1118,10 +1119,10 @@
         <v>41</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I3">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1147,7 +1148,7 @@
         <v>41</v>
       </c>
       <c r="H4">
-        <v>3.3</v>
+        <v>1.5</v>
       </c>
       <c r="I4">
         <v>0.5</v>
@@ -1176,7 +1177,7 @@
         <v>41</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1205,7 +1206,7 @@
         <v>41</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>17.8</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1234,10 +1235,10 @@
         <v>41</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1263,7 +1264,7 @@
         <v>41</v>
       </c>
       <c r="H8">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1292,10 +1293,10 @@
         <v>43</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1321,10 +1322,10 @@
         <v>43</v>
       </c>
       <c r="H10">
-        <v>0.8</v>
+        <v>5.4</v>
       </c>
       <c r="I10">
-        <v>1.1000000000000001</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: datasets 27/05/2026 + fix legacy PorcCambio opcional
- LEGACY/orbit_matinal_v42.py: PorcCambio ahora opcional en hoja Rechazos
  (resultado.xlsx actual no la tiene; se inicializa en 0.0 si falta)
- 01_INPUTS/ventas.csv + resultado.xlsx: datos del 27/05/2026
- 04_DATASETS_ORBIT/: 14 CSVs regenerados (fecha_ejecucion 2026-05-27, dia_objetivo Ju)
- 02_HISTORY/historial_ventas_cliente.csv: actualizado

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92AF494B-D70D-4702-B3ED-6579DAB6C4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A6F2076-669B-4AF3-A2D3-E3A5DF99B0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>PorcRechazo</t>
-  </si>
-  <si>
-    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -230,12 +227,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
-  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -244,7 +241,6 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -669,28 +665,28 @@
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>2580714.09</v>
+        <v>2570601.64</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2884327.51</v>
+        <v>2937830.44</v>
       </c>
       <c r="L2">
-        <v>25.68</v>
+        <v>26.16</v>
       </c>
       <c r="M2">
-        <v>151806.71</v>
+        <v>122409.60000000001</v>
       </c>
       <c r="N2">
-        <v>4325642.95</v>
+        <v>2887132.79</v>
       </c>
       <c r="O2">
-        <v>-14607.99</v>
+        <v>327165.53999999998</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>632530.74</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -722,28 +718,28 @@
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>37411681</v>
+        <v>38288667.280000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>41813055.240000002</v>
+        <v>43758476.890000001</v>
       </c>
       <c r="L3">
-        <v>97.77</v>
+        <v>102.32</v>
       </c>
       <c r="M3">
-        <v>2200687.12</v>
+        <v>1823269.87</v>
       </c>
       <c r="N3">
-        <v>2678159.5</v>
+        <v>1493110.91</v>
       </c>
       <c r="O3">
-        <v>194881.91</v>
+        <v>1404850.69</v>
       </c>
       <c r="P3">
-        <v>559362.31999999995</v>
+        <v>303136.03000000003</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -775,28 +771,28 @@
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>116254731.12</v>
+        <v>117143104.38</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>129931758.31</v>
+        <v>133877833.58</v>
       </c>
       <c r="L4">
-        <v>125.34</v>
+        <v>129.15</v>
       </c>
       <c r="M4">
-        <v>6838513.5999999996</v>
+        <v>5578243.0700000003</v>
       </c>
       <c r="N4">
-        <v>-6295365.5599999996</v>
+        <v>-4493034.79</v>
       </c>
       <c r="O4">
-        <v>1855821.89</v>
+        <v>1157286.6499999999</v>
       </c>
       <c r="P4">
-        <v>722387.37</v>
+        <v>63608373.039999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -828,28 +824,28 @@
         <v>8184000</v>
       </c>
       <c r="I5">
-        <v>11698505.460000001</v>
+        <v>11891165.26</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>13074800.220000001</v>
+        <v>13589903.15</v>
       </c>
       <c r="L5">
-        <v>159.76</v>
+        <v>166.05</v>
       </c>
       <c r="M5">
-        <v>688147.38</v>
+        <v>566245.96</v>
       </c>
       <c r="N5">
-        <v>-1757252.73</v>
+        <v>-1235721.75</v>
       </c>
       <c r="O5">
-        <v>2170700.08</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>3174736.56</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -881,28 +877,28 @@
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>24857954.370000001</v>
+        <v>24879507.510000002</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>27782419.579999998</v>
+        <v>28433722.870000001</v>
       </c>
       <c r="L6">
-        <v>67.89</v>
+        <v>69.489999999999995</v>
       </c>
       <c r="M6">
-        <v>1462232.61</v>
+        <v>1184738.45</v>
       </c>
       <c r="N6">
-        <v>8031022.8200000003</v>
+        <v>5346830.83</v>
       </c>
       <c r="O6">
-        <v>2199718.59</v>
+        <v>79729.490000000005</v>
       </c>
       <c r="P6">
-        <v>203892.01</v>
+        <v>232400.11</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -934,28 +930,28 @@
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>58073722.159999996</v>
+        <v>64280548.909999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>64905924.759999998</v>
+        <v>73463484.469999999</v>
       </c>
       <c r="L7">
-        <v>82.04</v>
+        <v>92.86</v>
       </c>
       <c r="M7">
-        <v>3416101.3</v>
+        <v>3060978.52</v>
       </c>
       <c r="N7">
-        <v>10519138.92</v>
+        <v>4943817.03</v>
       </c>
       <c r="O7">
-        <v>6952588.4199999999</v>
+        <v>765026.58</v>
       </c>
       <c r="P7">
-        <v>1200087.51</v>
+        <v>717385.05</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -987,28 +983,28 @@
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>39577067.18</v>
+        <v>40746542.399999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>44233192.740000002</v>
+        <v>46567477.030000001</v>
       </c>
       <c r="L8">
-        <v>108.1</v>
+        <v>113.8</v>
       </c>
       <c r="M8">
-        <v>2328062.7799999998</v>
+        <v>1940311.54</v>
       </c>
       <c r="N8">
-        <v>671466.41</v>
+        <v>57819.199999999997</v>
       </c>
       <c r="O8">
-        <v>1967561.5</v>
+        <v>501173.74</v>
       </c>
       <c r="P8">
-        <v>230847.97</v>
+        <v>417411.89</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1016,16 +1012,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1035,10 +1031,9 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1063,11 +1058,8 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1087,16 +1079,13 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H2">
         <v>0.9</v>
       </c>
-      <c r="I2">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1116,16 +1105,13 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3">
         <v>0.4</v>
       </c>
-      <c r="I3">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1145,16 +1131,13 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>1.5</v>
-      </c>
-      <c r="I4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1174,16 +1157,13 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>2.1</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1203,16 +1183,13 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>17.8</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>17.600000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1232,16 +1209,13 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7">
-        <v>0.5</v>
-      </c>
-      <c r="I7">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1261,16 +1235,13 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8">
-        <v>0.9</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1287,19 +1258,16 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
         <v>42</v>
       </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
       <c r="H9">
-        <v>0.6</v>
-      </c>
-      <c r="I9">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1316,23 +1284,20 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
       <c r="H10">
-        <v>5.4</v>
-      </c>
-      <c r="I10">
-        <v>0.5</v>
+        <v>5.3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: regeneracion completa 2026-05-29 — todos los datasets actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A6F2076-669B-4AF3-A2D3-E3A5DF99B0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEA745CE-4110-408C-9C00-952E9E51130D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>PorcRechazo</t>
+  </si>
+  <si>
+    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -227,12 +230,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
+  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="8">
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -241,6 +244,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -665,28 +669,28 @@
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>2570601.64</v>
+        <v>2868375.87</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2937830.44</v>
+        <v>2993087.87</v>
       </c>
       <c r="L2">
-        <v>26.16</v>
+        <v>26.65</v>
       </c>
       <c r="M2">
-        <v>122409.60000000001</v>
+        <v>124711.99</v>
       </c>
       <c r="N2">
-        <v>2887132.79</v>
+        <v>8363624.1299999999</v>
       </c>
       <c r="O2">
-        <v>327165.53999999998</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>632530.74</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -718,28 +722,28 @@
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>38288667.280000001</v>
+        <v>40474173.079999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>43758476.890000001</v>
+        <v>42233919.740000002</v>
       </c>
       <c r="L3">
-        <v>102.32</v>
+        <v>98.75</v>
       </c>
       <c r="M3">
-        <v>1823269.87</v>
+        <v>1759746.66</v>
       </c>
       <c r="N3">
-        <v>1493110.91</v>
+        <v>2293826.92</v>
       </c>
       <c r="O3">
-        <v>1404850.69</v>
+        <v>945695.68</v>
       </c>
       <c r="P3">
-        <v>303136.03000000003</v>
+        <v>623068.23</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -771,28 +775,28 @@
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>117143104.38</v>
+        <v>118357765.34999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>133877833.58</v>
+        <v>123503755.14</v>
       </c>
       <c r="L4">
-        <v>129.15</v>
+        <v>119.14</v>
       </c>
       <c r="M4">
-        <v>5578243.0700000003</v>
+        <v>5145989.8</v>
       </c>
       <c r="N4">
-        <v>-4493034.79</v>
+        <v>-14693765.35</v>
       </c>
       <c r="O4">
-        <v>1157286.6499999999</v>
+        <v>173189.14</v>
       </c>
       <c r="P4">
-        <v>63608373.039999999</v>
+        <v>488926.39</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,28 +828,28 @@
         <v>8184000</v>
       </c>
       <c r="I5">
-        <v>11891165.26</v>
+        <v>11927690.050000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>13589903.15</v>
+        <v>12446285.27</v>
       </c>
       <c r="L5">
-        <v>166.05</v>
+        <v>152.08000000000001</v>
       </c>
       <c r="M5">
-        <v>566245.96</v>
+        <v>518595.22</v>
       </c>
       <c r="N5">
-        <v>-1235721.75</v>
+        <v>-3743690.05</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>197788.91</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>14623.46</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,28 +881,28 @@
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>24879507.510000002</v>
+        <v>29712880.890000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>28433722.870000001</v>
+        <v>31004745.280000001</v>
       </c>
       <c r="L6">
-        <v>69.489999999999995</v>
+        <v>75.77</v>
       </c>
       <c r="M6">
-        <v>1184738.45</v>
+        <v>1291864.3899999999</v>
       </c>
       <c r="N6">
-        <v>5346830.83</v>
+        <v>11207119.109999999</v>
       </c>
       <c r="O6">
-        <v>79729.490000000005</v>
+        <v>961667.35</v>
       </c>
       <c r="P6">
-        <v>232400.11</v>
+        <v>185467.97</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -930,28 +934,28 @@
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>64280548.909999996</v>
+        <v>64792765.579999998</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>73463484.469999999</v>
+        <v>67609842.340000004</v>
       </c>
       <c r="L7">
-        <v>92.86</v>
+        <v>85.46</v>
       </c>
       <c r="M7">
-        <v>3060978.52</v>
+        <v>2817076.76</v>
       </c>
       <c r="N7">
-        <v>4943817.03</v>
+        <v>14319234.42</v>
       </c>
       <c r="O7">
-        <v>765026.58</v>
+        <v>1424928.1</v>
       </c>
       <c r="P7">
-        <v>717385.05</v>
+        <v>20447000.789999999</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,28 +987,28 @@
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>40746542.399999999</v>
+        <v>41488142.659999996</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>46567477.030000001</v>
+        <v>43291974.950000003</v>
       </c>
       <c r="L8">
-        <v>113.8</v>
+        <v>105.8</v>
       </c>
       <c r="M8">
-        <v>1940311.54</v>
+        <v>1803832.29</v>
       </c>
       <c r="N8">
-        <v>57819.199999999997</v>
+        <v>-568142.66</v>
       </c>
       <c r="O8">
-        <v>501173.74</v>
+        <v>3401918.13</v>
       </c>
       <c r="P8">
-        <v>417411.89</v>
+        <v>417857.78</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1021,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1031,9 +1035,10 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1058,8 +1063,11 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1079,13 +1087,16 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1105,13 +1116,16 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1131,13 +1145,16 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.9</v>
+      </c>
+      <c r="I4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1157,13 +1174,16 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2.9</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1183,13 +1203,16 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6">
-        <v>17.600000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1209,13 +1232,16 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1235,13 +1261,16 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H8">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1258,16 +1287,19 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H9">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1284,13 +1316,16 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H10">
-        <v>5.3</v>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I10">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: inputs 2026-05-29-1745 + datasets regenerados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEA745CE-4110-408C-9C00-952E9E51130D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920F8D3E-B3CA-4677-8193-BEFAA306DFA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="36">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -75,9 +75,6 @@
     <t>BENITEZ RAUL</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>JOFRE GUILLERMO AGUSTIN</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>PEÑAFLOR GRUPO OBJETIVO</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>SANCHEZ FERNANDO JAVIER</t>
   </si>
   <si>
@@ -99,33 +93,18 @@
     <t>GRIBAUDO ESTEBAN</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>ALVAREZ VANESA  KAFF</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>GAMBINO NADIA</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>ORTEGA MILAGROS DESIREE</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>PEYRONEL ANDREA</t>
   </si>
   <si>
@@ -136,9 +115,6 @@
   </si>
   <si>
     <t>PorcRechazo</t>
-  </si>
-  <si>
-    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -230,12 +206,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
-  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -244,7 +220,6 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -580,8 +555,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
@@ -653,44 +627,44 @@
       <c r="C2">
         <v>105007</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>22</v>
       </c>
       <c r="H2">
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>2868375.87</v>
+        <v>2785000.09</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2993087.87</v>
+        <v>2906087.05</v>
       </c>
       <c r="L2">
-        <v>26.65</v>
+        <v>25.87</v>
       </c>
       <c r="M2">
-        <v>124711.99</v>
+        <v>121086.96</v>
       </c>
       <c r="N2">
-        <v>8363624.1299999999</v>
+        <v>8446999.9100000001</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>14607.99</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -706,44 +680,44 @@
       <c r="C3">
         <v>120039</v>
       </c>
-      <c r="D3" t="s">
-        <v>23</v>
+      <c r="D3" s="1">
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
       </c>
       <c r="H3">
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>40474173.079999998</v>
+        <v>42968523.109999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>42233919.740000002</v>
+        <v>44836719.770000003</v>
       </c>
       <c r="L3">
-        <v>98.75</v>
+        <v>104.84</v>
       </c>
       <c r="M3">
-        <v>1759746.66</v>
+        <v>1868196.66</v>
       </c>
       <c r="N3">
-        <v>2293826.92</v>
+        <v>-200523.11</v>
       </c>
       <c r="O3">
-        <v>945695.68</v>
+        <v>140558.04</v>
       </c>
       <c r="P3">
-        <v>623068.23</v>
+        <v>620920.59</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -751,52 +725,52 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4">
         <v>105008</v>
       </c>
-      <c r="D4" t="s">
-        <v>27</v>
+      <c r="D4" s="1">
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
         <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
       </c>
       <c r="H4">
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>118357765.34999999</v>
+        <v>117175910.90000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>123503755.14</v>
+        <v>122270515.72</v>
       </c>
       <c r="L4">
-        <v>119.14</v>
+        <v>117.95</v>
       </c>
       <c r="M4">
-        <v>5145989.8</v>
+        <v>5094604.82</v>
       </c>
       <c r="N4">
-        <v>-14693765.35</v>
+        <v>-13511910.9</v>
       </c>
       <c r="O4">
-        <v>173189.14</v>
+        <v>5420805.5899999999</v>
       </c>
       <c r="P4">
-        <v>488926.39</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -804,52 +778,52 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C5">
         <v>105003</v>
       </c>
-      <c r="D5" t="s">
-        <v>29</v>
+      <c r="D5" s="1">
+        <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
         <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
       </c>
       <c r="H5">
         <v>8184000</v>
       </c>
       <c r="I5">
-        <v>11927690.050000001</v>
+        <v>11961501.74</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>12446285.27</v>
+        <v>12481567.029999999</v>
       </c>
       <c r="L5">
-        <v>152.08000000000001</v>
+        <v>152.51</v>
       </c>
       <c r="M5">
-        <v>518595.22</v>
+        <v>520065.29</v>
       </c>
       <c r="N5">
-        <v>-3743690.05</v>
+        <v>-3777501.74</v>
       </c>
       <c r="O5">
-        <v>197788.91</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>14623.46</v>
+        <v>20932.21</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -857,52 +831,52 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6">
         <v>105004</v>
       </c>
-      <c r="D6" t="s">
-        <v>31</v>
+      <c r="D6" s="1">
+        <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
         <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>22</v>
       </c>
       <c r="H6">
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>29712880.890000001</v>
+        <v>30475423.809999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>31004745.280000001</v>
+        <v>31800442.239999998</v>
       </c>
       <c r="L6">
-        <v>75.77</v>
+        <v>77.709999999999994</v>
       </c>
       <c r="M6">
-        <v>1291864.3899999999</v>
+        <v>1325018.43</v>
       </c>
       <c r="N6">
-        <v>11207119.109999999</v>
+        <v>10444576.189999999</v>
       </c>
       <c r="O6">
-        <v>961667.35</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>185467.97</v>
+        <v>12321691.17</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -910,52 +884,52 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C7">
         <v>120041</v>
       </c>
-      <c r="D7" t="s">
-        <v>33</v>
+      <c r="D7" s="1">
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
         <v>21</v>
-      </c>
-      <c r="G7" t="s">
-        <v>22</v>
       </c>
       <c r="H7">
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>64792765.579999998</v>
+        <v>72427059.489999995</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>67609842.340000004</v>
+        <v>75576062.079999998</v>
       </c>
       <c r="L7">
-        <v>85.46</v>
+        <v>95.53</v>
       </c>
       <c r="M7">
-        <v>2817076.76</v>
+        <v>3149002.59</v>
       </c>
       <c r="N7">
-        <v>14319234.42</v>
+        <v>6684940.5099999998</v>
       </c>
       <c r="O7">
-        <v>1424928.1</v>
+        <v>186105.37</v>
       </c>
       <c r="P7">
-        <v>20447000.789999999</v>
+        <v>5268747.87</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -963,52 +937,52 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>105006</v>
       </c>
-      <c r="D8" t="s">
-        <v>35</v>
+      <c r="D8" s="1">
+        <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
         <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>22</v>
       </c>
       <c r="H8">
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>41488142.659999996</v>
+        <v>43718563.090000004</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>43291974.950000003</v>
+        <v>45619370.18</v>
       </c>
       <c r="L8">
-        <v>105.8</v>
+        <v>111.48</v>
       </c>
       <c r="M8">
-        <v>1803832.29</v>
+        <v>1900807.09</v>
       </c>
       <c r="N8">
-        <v>-568142.66</v>
+        <v>-2798563.09</v>
       </c>
       <c r="O8">
-        <v>3401918.13</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>417857.78</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1025,7 +999,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1035,12 +1009,11 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1058,103 +1031,91 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D2">
         <v>105003</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H2">
-        <v>0.9</v>
-      </c>
-      <c r="I2">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D3">
         <v>105004</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H3">
         <v>0.4</v>
       </c>
-      <c r="I3">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D4">
         <v>105006</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H4">
         <v>1.9</v>
       </c>
-      <c r="I4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1167,52 +1128,46 @@
       <c r="D5">
         <v>105007</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5">
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H5">
-        <v>2.9</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>105008</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6">
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H6">
-        <v>17.399999999999999</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>19.600000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1225,52 +1180,46 @@
       <c r="D7">
         <v>120039</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H7">
-        <v>0.7</v>
-      </c>
-      <c r="I7">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8">
         <v>120041</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="H8">
-        <v>0.8</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1283,49 +1232,43 @@
       <c r="D9">
         <v>106002</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="H9">
         <v>0.8</v>
       </c>
-      <c r="I9">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D10">
         <v>105021</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10">
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G10" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="H10">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="I10">
-        <v>0.5</v>
+        <v>5.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: cierre de mes + datasets actualizados 2026-06-01
- server_orbit.py: endpoint /api/gerencia/cierre_mes (objetivos desde resultado.xlsx, CCC desde ventas_acumulada.csv con filtro Empresa=Peñaflor)
- portal.html: sidebar 'Cierre de Mes' + pantalla gCierreMes con selector de mes, tarjetas empresa y tabla por vendedor
- Datasets y ventas actualizados al 2026-05-30

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920F8D3E-B3CA-4677-8193-BEFAA306DFA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4B979AB-CA15-4A7A-B923-E29F11B5D488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -75,6 +75,9 @@
     <t>BENITEZ RAUL</t>
   </si>
   <si>
+    <t>7</t>
+  </si>
+  <si>
     <t>JOFRE GUILLERMO AGUSTIN</t>
   </si>
   <si>
@@ -84,6 +87,9 @@
     <t>PEÑAFLOR GRUPO OBJETIVO</t>
   </si>
   <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>SANCHEZ FERNANDO JAVIER</t>
   </si>
   <si>
@@ -93,18 +99,33 @@
     <t>GRIBAUDO ESTEBAN</t>
   </si>
   <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>ALVAREZ VANESA  KAFF</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>GAMBINO NADIA</t>
   </si>
   <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>ORTEGA MILAGROS DESIREE</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>PEYRONEL ANDREA</t>
   </si>
   <si>
@@ -115,6 +136,9 @@
   </si>
   <si>
     <t>PorcRechazo</t>
+  </si>
+  <si>
+    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -206,12 +230,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
+  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="8">
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -220,6 +244,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -555,8 +580,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -627,44 +651,44 @@
       <c r="C2">
         <v>105007</v>
       </c>
-      <c r="D2" s="1">
-        <v>7</v>
+      <c r="D2" t="s">
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H2">
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>2785000.09</v>
+        <v>3097000.62</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2906087.05</v>
+        <v>3097000.62</v>
       </c>
       <c r="L2">
-        <v>25.87</v>
+        <v>27.57</v>
       </c>
       <c r="M2">
-        <v>121086.96</v>
+        <v>129041.69</v>
       </c>
       <c r="N2">
-        <v>8446999.9100000001</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>14607.99</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -680,44 +704,44 @@
       <c r="C3">
         <v>120039</v>
       </c>
-      <c r="D3" s="1">
-        <v>9</v>
+      <c r="D3" t="s">
+        <v>23</v>
       </c>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
         <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
       </c>
       <c r="H3">
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>42968523.109999999</v>
+        <v>43014748.859999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>44836719.770000003</v>
+        <v>43014748.859999999</v>
       </c>
       <c r="L3">
-        <v>104.84</v>
+        <v>100.58</v>
       </c>
       <c r="M3">
-        <v>1868196.66</v>
+        <v>1792281.2</v>
       </c>
       <c r="N3">
-        <v>-200523.11</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>140558.04</v>
+        <v>735836.71</v>
       </c>
       <c r="P3">
-        <v>620920.59</v>
+        <v>399467.92</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -725,52 +749,52 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4">
         <v>105008</v>
       </c>
-      <c r="D4" s="1">
-        <v>8</v>
+      <c r="D4" t="s">
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4">
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>117175910.90000001</v>
+        <v>119391188.09999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>122270515.72</v>
+        <v>119391188.09999999</v>
       </c>
       <c r="L4">
-        <v>117.95</v>
+        <v>115.17</v>
       </c>
       <c r="M4">
-        <v>5094604.82</v>
+        <v>4974632.84</v>
       </c>
       <c r="N4">
-        <v>-13511910.9</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>5420805.5899999999</v>
+        <v>37530041.719999999</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>294215.25</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -778,25 +802,25 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>105003</v>
       </c>
-      <c r="D5" s="1">
-        <v>3</v>
+      <c r="D5" t="s">
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H5">
         <v>8184000</v>
@@ -808,22 +832,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>12481567.029999999</v>
+        <v>11961501.74</v>
       </c>
       <c r="L5">
-        <v>152.51</v>
+        <v>146.16</v>
       </c>
       <c r="M5">
-        <v>520065.29</v>
+        <v>498395.91</v>
       </c>
       <c r="N5">
-        <v>-3777501.74</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>151408.07</v>
       </c>
       <c r="P5">
-        <v>20932.21</v>
+        <v>28092.28</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -831,52 +855,52 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6">
         <v>105004</v>
       </c>
-      <c r="D6" s="1">
-        <v>4</v>
+      <c r="D6" t="s">
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H6">
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>30475423.809999999</v>
+        <v>30531285.41</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>31800442.239999998</v>
+        <v>30531285.41</v>
       </c>
       <c r="L6">
-        <v>77.709999999999994</v>
+        <v>74.61</v>
       </c>
       <c r="M6">
-        <v>1325018.43</v>
+        <v>1272136.8899999999</v>
       </c>
       <c r="N6">
-        <v>10444576.189999999</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>1493000.43</v>
       </c>
       <c r="P6">
-        <v>12321691.17</v>
+        <v>123438.1</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -884,52 +908,52 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7">
         <v>120041</v>
       </c>
-      <c r="D7" s="1">
-        <v>10</v>
+      <c r="D7" t="s">
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H7">
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>72427059.489999995</v>
+        <v>72725692.379999995</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>75576062.079999998</v>
+        <v>72725692.379999995</v>
       </c>
       <c r="L7">
-        <v>95.53</v>
+        <v>91.93</v>
       </c>
       <c r="M7">
-        <v>3149002.59</v>
+        <v>3030237.18</v>
       </c>
       <c r="N7">
-        <v>6684940.5099999998</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>186105.37</v>
+        <v>2398476.87</v>
       </c>
       <c r="P7">
-        <v>5268747.87</v>
+        <v>799213.02</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -937,52 +961,52 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8">
         <v>105006</v>
       </c>
-      <c r="D8" s="1">
-        <v>6</v>
+      <c r="D8" t="s">
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H8">
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>43718563.090000004</v>
+        <v>43619746.170000002</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>45619370.18</v>
+        <v>43619746.170000002</v>
       </c>
       <c r="L8">
-        <v>111.48</v>
+        <v>106.6</v>
       </c>
       <c r="M8">
-        <v>1900807.09</v>
+        <v>1817489.42</v>
       </c>
       <c r="N8">
-        <v>-2798563.09</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>780470.3</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>878686.94</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -999,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1009,11 +1033,12 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1031,91 +1056,103 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>105003</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>105004</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H3">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4">
         <v>105006</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H4">
-        <v>1.9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2.1</v>
+      </c>
+      <c r="I4">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1128,46 +1165,52 @@
       <c r="D5">
         <v>105007</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>3.1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6">
         <v>105008</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H6">
-        <v>19.600000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>19.3</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1180,46 +1223,52 @@
       <c r="D7">
         <v>120039</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H7">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.7</v>
+      </c>
+      <c r="I7">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D8">
         <v>120041</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H8">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1232,43 +1281,49 @@
       <c r="D9">
         <v>106002</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H9">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.9</v>
+      </c>
+      <c r="I9">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>105021</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="1">
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H10">
         <v>5.4</v>
+      </c>
+      <c r="I10">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-02_2211 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4B979AB-CA15-4A7A-B923-E29F11B5D488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0A5CD5D-AB6E-4C43-8E37-BBBB71935C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>PorcRechazo</t>
-  </si>
-  <si>
-    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -230,12 +227,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
-  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -244,7 +241,6 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -580,7 +576,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -667,28 +664,28 @@
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>3097000.62</v>
+        <v>63992.98</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3097000.62</v>
+        <v>767915.71</v>
       </c>
       <c r="L2">
-        <v>27.57</v>
+        <v>6.84</v>
       </c>
       <c r="M2">
-        <v>129041.69</v>
+        <v>31996.49</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>507636.68</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>-10112.450000000001</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>-14607.99</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -720,28 +717,28 @@
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>43014748.859999999</v>
+        <v>998005.26</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>43014748.859999999</v>
+        <v>11976063.130000001</v>
       </c>
       <c r="L3">
-        <v>100.58</v>
+        <v>28</v>
       </c>
       <c r="M3">
-        <v>1792281.2</v>
+        <v>499002.63</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>1898636.12</v>
       </c>
       <c r="O3">
-        <v>735836.71</v>
+        <v>876986.28</v>
       </c>
       <c r="P3">
-        <v>399467.92</v>
+        <v>194881.91</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -773,28 +770,28 @@
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>119391188.09999999</v>
+        <v>5981157.2999999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>119391188.09999999</v>
+        <v>71773887.659999996</v>
       </c>
       <c r="L4">
-        <v>115.17</v>
+        <v>69.239999999999995</v>
       </c>
       <c r="M4">
-        <v>4974632.84</v>
+        <v>2990578.65</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>4440129.21</v>
       </c>
       <c r="O4">
-        <v>37530041.719999999</v>
+        <v>1149986.8700000001</v>
       </c>
       <c r="P4">
-        <v>294215.25</v>
+        <v>1855821.89</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -826,28 +823,28 @@
         <v>8184000</v>
       </c>
       <c r="I5">
-        <v>11961501.74</v>
+        <v>95470.23</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>11961501.74</v>
+        <v>1145642.81</v>
       </c>
       <c r="L5">
-        <v>146.16</v>
+        <v>14</v>
       </c>
       <c r="M5">
-        <v>498395.91</v>
+        <v>47735.12</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>367660.44</v>
       </c>
       <c r="O5">
-        <v>151408.07</v>
+        <v>192659.8</v>
       </c>
       <c r="P5">
-        <v>28092.28</v>
+        <v>2170700.08</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -879,28 +876,28 @@
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>30531285.41</v>
+        <v>354591.74</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>30531285.41</v>
+        <v>4255100.8600000003</v>
       </c>
       <c r="L6">
-        <v>74.61</v>
+        <v>10.4</v>
       </c>
       <c r="M6">
-        <v>1272136.8899999999</v>
+        <v>177295.87</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>1843882.19</v>
       </c>
       <c r="O6">
-        <v>1493000.43</v>
+        <v>2511554.75</v>
       </c>
       <c r="P6">
-        <v>123438.1</v>
+        <v>2199718.59</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -932,28 +929,28 @@
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>72725692.379999995</v>
+        <v>3174653.9</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>72725692.379999995</v>
+        <v>38095846.840000004</v>
       </c>
       <c r="L7">
-        <v>91.93</v>
+        <v>48.15</v>
       </c>
       <c r="M7">
-        <v>3030237.18</v>
+        <v>1587326.95</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>3451697.55</v>
       </c>
       <c r="O7">
-        <v>2398476.87</v>
+        <v>6553989.9900000002</v>
       </c>
       <c r="P7">
-        <v>799213.02</v>
+        <v>6952588.4199999999</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -985,28 +982,28 @@
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>43619746.170000002</v>
+        <v>5330653.67</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>43619746.170000002</v>
+        <v>63967844.020000003</v>
       </c>
       <c r="L8">
-        <v>106.6</v>
+        <v>156.32</v>
       </c>
       <c r="M8">
-        <v>1817489.42</v>
+        <v>2665326.83</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>1617697.56</v>
       </c>
       <c r="O8">
-        <v>780470.3</v>
+        <v>1200502.3400000001</v>
       </c>
       <c r="P8">
-        <v>878686.94</v>
+        <v>1967561.5</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1023,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1033,10 +1030,9 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1061,11 +1057,8 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1085,16 +1078,13 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="I2">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1114,16 +1104,13 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>0.4</v>
-      </c>
-      <c r="I3">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1143,16 +1130,13 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>2.1</v>
-      </c>
-      <c r="I4">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1172,16 +1156,13 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>3.1</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1201,16 +1182,13 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6">
-        <v>19.3</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1230,16 +1208,13 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7">
-        <v>0.7</v>
-      </c>
-      <c r="I7">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1259,16 +1234,13 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8">
-        <v>0.8</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1285,19 +1257,16 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
         <v>42</v>
       </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
       <c r="H9">
-        <v>0.9</v>
-      </c>
-      <c r="I9">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1314,16 +1283,13 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
       <c r="H10">
-        <v>5.4</v>
-      </c>
-      <c r="I10">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(refresh): ventas/datasets al 2026-06-03 (matinal jueves)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0A5CD5D-AB6E-4C43-8E37-BBBB71935C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5423708C-8497-4945-B02B-DEDBD4AE4509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -664,28 +664,28 @@
         <v>11232000</v>
       </c>
       <c r="I2">
-        <v>63992.98</v>
+        <v>90012.45</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>767915.71</v>
+        <v>720099.62</v>
       </c>
       <c r="L2">
-        <v>6.84</v>
+        <v>6.41</v>
       </c>
       <c r="M2">
-        <v>31996.49</v>
+        <v>30004.15</v>
       </c>
       <c r="N2">
-        <v>507636.68</v>
+        <v>530570.84</v>
       </c>
       <c r="O2">
-        <v>-10112.450000000001</v>
+        <v>214398.45</v>
       </c>
       <c r="P2">
-        <v>-14607.99</v>
+        <v>327165.53999999998</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -717,28 +717,28 @@
         <v>42768000</v>
       </c>
       <c r="I3">
-        <v>998005.26</v>
+        <v>2237651.9900000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>11976063.130000001</v>
+        <v>17901215.899999999</v>
       </c>
       <c r="L3">
-        <v>28</v>
+        <v>41.86</v>
       </c>
       <c r="M3">
-        <v>499002.63</v>
+        <v>745884</v>
       </c>
       <c r="N3">
-        <v>1898636.12</v>
+        <v>1930016.57</v>
       </c>
       <c r="O3">
-        <v>876986.28</v>
+        <v>2185505.7999999998</v>
       </c>
       <c r="P3">
-        <v>194881.91</v>
+        <v>1404850.69</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -770,28 +770,28 @@
         <v>103664000</v>
       </c>
       <c r="I4">
-        <v>5981157.2999999998</v>
+        <v>6790238.9000000004</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>71773887.659999996</v>
+        <v>54321911.229999997</v>
       </c>
       <c r="L4">
-        <v>69.239999999999995</v>
+        <v>52.4</v>
       </c>
       <c r="M4">
-        <v>2990578.65</v>
+        <v>2263412.9700000002</v>
       </c>
       <c r="N4">
-        <v>4440129.21</v>
+        <v>4613036.24</v>
       </c>
       <c r="O4">
-        <v>1149986.8700000001</v>
+        <v>1294302.58</v>
       </c>
       <c r="P4">
-        <v>1855821.89</v>
+        <v>1184778.75</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -823,28 +823,28 @@
         <v>8184000</v>
       </c>
       <c r="I5">
-        <v>95470.23</v>
+        <v>391694.24</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1145642.81</v>
+        <v>3133553.91</v>
       </c>
       <c r="L5">
-        <v>14</v>
+        <v>38.29</v>
       </c>
       <c r="M5">
-        <v>47735.12</v>
+        <v>130564.75</v>
       </c>
       <c r="N5">
-        <v>367660.44</v>
+        <v>371062.18</v>
       </c>
       <c r="O5">
-        <v>192659.8</v>
+        <v>36524.79</v>
       </c>
       <c r="P5">
-        <v>2170700.08</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -876,28 +876,28 @@
         <v>40920000</v>
       </c>
       <c r="I6">
-        <v>354591.74</v>
+        <v>740912.36</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4255100.8600000003</v>
+        <v>5927298.8700000001</v>
       </c>
       <c r="L6">
-        <v>10.4</v>
+        <v>14.49</v>
       </c>
       <c r="M6">
-        <v>177295.87</v>
+        <v>246970.79</v>
       </c>
       <c r="N6">
-        <v>1843882.19</v>
+        <v>1913289.89</v>
       </c>
       <c r="O6">
-        <v>2511554.75</v>
+        <v>2509730.8199999998</v>
       </c>
       <c r="P6">
-        <v>2199718.59</v>
+        <v>79729.490000000005</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -929,28 +929,28 @@
         <v>79112000</v>
       </c>
       <c r="I7">
-        <v>3174653.9</v>
+        <v>3630309.76</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>38095846.840000004</v>
+        <v>29042478.07</v>
       </c>
       <c r="L7">
-        <v>48.15</v>
+        <v>36.71</v>
       </c>
       <c r="M7">
-        <v>1587326.95</v>
+        <v>1210103.25</v>
       </c>
       <c r="N7">
-        <v>3451697.55</v>
+        <v>3594366.2</v>
       </c>
       <c r="O7">
-        <v>6553989.9900000002</v>
+        <v>575210.05000000005</v>
       </c>
       <c r="P7">
-        <v>6952588.4199999999</v>
+        <v>792811.15</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -982,28 +982,28 @@
         <v>40920000</v>
       </c>
       <c r="I8">
-        <v>5330653.67</v>
+        <v>5833023.2300000004</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>63967844.020000003</v>
+        <v>46664185.859999999</v>
       </c>
       <c r="L8">
-        <v>156.32</v>
+        <v>114.04</v>
       </c>
       <c r="M8">
-        <v>2665326.83</v>
+        <v>1944341.08</v>
       </c>
       <c r="N8">
-        <v>1617697.56</v>
+        <v>1670808.42</v>
       </c>
       <c r="O8">
-        <v>1200502.3400000001</v>
+        <v>741600.26</v>
       </c>
       <c r="P8">
-        <v>1967561.5</v>
+        <v>501173.74</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1081,7 +1081,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1289,7 +1289,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-04 — datasets + inputs (push pendiente del bat roto)
Datos regenerados por el cierre del usuario (ya reflejan las correcciones:
11T=11 marcas, innovaciones junio, planes con direccion). El bat no pudo
pushearlos por los finales de linea LF; se suben aca.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5423708C-8497-4945-B02B-DEDBD4AE4509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD6662EB-C875-4367-B535-21F09613039D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,31 +661,31 @@
         <v>22</v>
       </c>
       <c r="H2">
-        <v>11232000</v>
+        <v>5500000</v>
       </c>
       <c r="I2">
-        <v>90012.45</v>
+        <v>509680.7</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>720099.62</v>
+        <v>3058084.18</v>
       </c>
       <c r="L2">
-        <v>6.41</v>
+        <v>55.6</v>
       </c>
       <c r="M2">
-        <v>30004.15</v>
+        <v>127420.17</v>
       </c>
       <c r="N2">
-        <v>530570.84</v>
+        <v>249515.97</v>
       </c>
       <c r="O2">
-        <v>214398.45</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>327165.53999999998</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,31 +714,31 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>42768000</v>
+        <v>49500000</v>
       </c>
       <c r="I3">
-        <v>2237651.9900000002</v>
+        <v>9065050.7799999993</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>17901215.899999999</v>
+        <v>54390304.68</v>
       </c>
       <c r="L3">
-        <v>41.86</v>
+        <v>109.88</v>
       </c>
       <c r="M3">
-        <v>745884</v>
+        <v>2266262.69</v>
       </c>
       <c r="N3">
-        <v>1930016.57</v>
+        <v>2021747.46</v>
       </c>
       <c r="O3">
-        <v>2185505.7999999998</v>
+        <v>2494350.0299999998</v>
       </c>
       <c r="P3">
-        <v>1404850.69</v>
+        <v>945695.68</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,31 +767,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>103664000</v>
+        <v>112750000</v>
       </c>
       <c r="I4">
-        <v>6790238.9000000004</v>
+        <v>7030112.8700000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>54321911.229999997</v>
+        <v>42180677.240000002</v>
       </c>
       <c r="L4">
-        <v>52.4</v>
+        <v>37.409999999999997</v>
       </c>
       <c r="M4">
-        <v>2263412.9700000002</v>
+        <v>1757528.22</v>
       </c>
       <c r="N4">
-        <v>4613036.24</v>
+        <v>5285994.3600000003</v>
       </c>
       <c r="O4">
-        <v>1294302.58</v>
+        <v>-1619390.32</v>
       </c>
       <c r="P4">
-        <v>1184778.75</v>
+        <v>173189.14</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,31 +820,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>8184000</v>
+        <v>13750000</v>
       </c>
       <c r="I5">
-        <v>391694.24</v>
+        <v>472463.61</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3133553.91</v>
+        <v>2834781.67</v>
       </c>
       <c r="L5">
-        <v>38.29</v>
+        <v>20.62</v>
       </c>
       <c r="M5">
-        <v>130564.75</v>
+        <v>118115.9</v>
       </c>
       <c r="N5">
-        <v>371062.18</v>
+        <v>663876.81999999995</v>
       </c>
       <c r="O5">
-        <v>36524.79</v>
+        <v>33811.69</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>197788.91</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -873,31 +873,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>40920000</v>
+        <v>33000000</v>
       </c>
       <c r="I6">
-        <v>740912.36</v>
+        <v>981774.51</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5927298.8700000001</v>
+        <v>5890647.0700000003</v>
       </c>
       <c r="L6">
-        <v>14.49</v>
+        <v>17.850000000000001</v>
       </c>
       <c r="M6">
-        <v>246970.79</v>
+        <v>245443.63</v>
       </c>
       <c r="N6">
-        <v>1913289.89</v>
+        <v>1600911.27</v>
       </c>
       <c r="O6">
-        <v>2509730.8199999998</v>
+        <v>651521.93999999994</v>
       </c>
       <c r="P6">
-        <v>79729.490000000005</v>
+        <v>961667.35</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,31 +926,31 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>79112000</v>
+        <v>71500000</v>
       </c>
       <c r="I7">
-        <v>3630309.76</v>
+        <v>3988161.03</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>29042478.07</v>
+        <v>23928966.199999999</v>
       </c>
       <c r="L7">
-        <v>36.71</v>
+        <v>33.47</v>
       </c>
       <c r="M7">
-        <v>1210103.25</v>
+        <v>997040.26</v>
       </c>
       <c r="N7">
-        <v>3594366.2</v>
+        <v>3375591.95</v>
       </c>
       <c r="O7">
-        <v>575210.05000000005</v>
+        <v>8989234.3699999992</v>
       </c>
       <c r="P7">
-        <v>792811.15</v>
+        <v>1424928.1</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,31 +979,31 @@
         <v>22</v>
       </c>
       <c r="H8">
-        <v>40920000</v>
+        <v>44000000</v>
       </c>
       <c r="I8">
-        <v>5833023.2300000004</v>
+        <v>6099563.8300000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>46664185.859999999</v>
+        <v>36597382.990000002</v>
       </c>
       <c r="L8">
-        <v>114.04</v>
+        <v>83.18</v>
       </c>
       <c r="M8">
-        <v>1944341.08</v>
+        <v>1524890.96</v>
       </c>
       <c r="N8">
-        <v>1670808.42</v>
+        <v>1895021.81</v>
       </c>
       <c r="O8">
-        <v>741600.26</v>
+        <v>2942910.32</v>
       </c>
       <c r="P8">
-        <v>501173.74</v>
+        <v>3401918.13</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1081,7 +1081,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1107,7 +1107,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1133,7 +1133,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1289,7 +1289,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-05_1756 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD6662EB-C875-4367-B535-21F09613039D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35FF4162-B26A-4B8A-8A7F-1F36D78549CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>PorcRechazo</t>
+  </si>
+  <si>
+    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -227,12 +230,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
+  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="8">
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -241,6 +244,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -576,8 +580,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -664,25 +667,25 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>509680.7</v>
+        <v>533324.49</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3058084.18</v>
+        <v>2559957.5299999998</v>
       </c>
       <c r="L2">
-        <v>55.6</v>
+        <v>46.54</v>
       </c>
       <c r="M2">
-        <v>127420.17</v>
+        <v>106664.9</v>
       </c>
       <c r="N2">
-        <v>249515.97</v>
+        <v>261403.97</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>312000.53000000003</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -717,28 +720,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>9065050.7799999993</v>
+        <v>17543860.710000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>54390304.68</v>
+        <v>84210531.409999996</v>
       </c>
       <c r="L3">
-        <v>109.88</v>
+        <v>170.12</v>
       </c>
       <c r="M3">
-        <v>2266262.69</v>
+        <v>3508772.14</v>
       </c>
       <c r="N3">
-        <v>2021747.46</v>
+        <v>1681902.07</v>
       </c>
       <c r="O3">
-        <v>2494350.0299999998</v>
+        <v>46225.75</v>
       </c>
       <c r="P3">
-        <v>945695.68</v>
+        <v>140558.04</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -770,28 +773,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>7030112.8700000001</v>
+        <v>7197927.8399999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>42180677.240000002</v>
+        <v>34550053.640000001</v>
       </c>
       <c r="L4">
-        <v>37.409999999999997</v>
+        <v>30.64</v>
       </c>
       <c r="M4">
-        <v>1757528.22</v>
+        <v>1439585.57</v>
       </c>
       <c r="N4">
-        <v>5285994.3600000003</v>
+        <v>5555372.2199999997</v>
       </c>
       <c r="O4">
-        <v>-1619390.32</v>
+        <v>1993306.04</v>
       </c>
       <c r="P4">
-        <v>173189.14</v>
+        <v>5448882.6299999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -823,28 +826,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>472463.61</v>
+        <v>566355.03</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2834781.67</v>
+        <v>2718504.13</v>
       </c>
       <c r="L5">
-        <v>20.62</v>
+        <v>19.77</v>
       </c>
       <c r="M5">
-        <v>118115.9</v>
+        <v>113271.01</v>
       </c>
       <c r="N5">
-        <v>663876.81999999995</v>
+        <v>693876.05</v>
       </c>
       <c r="O5">
-        <v>33811.69</v>
+        <v>95470.23</v>
       </c>
       <c r="P5">
-        <v>197788.91</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -876,28 +879,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>981774.51</v>
+        <v>1125153.29</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5890647.0700000003</v>
+        <v>5400735.7699999996</v>
       </c>
       <c r="L6">
-        <v>17.850000000000001</v>
+        <v>16.37</v>
       </c>
       <c r="M6">
-        <v>245443.63</v>
+        <v>225030.66</v>
       </c>
       <c r="N6">
-        <v>1600911.27</v>
+        <v>1677623.51</v>
       </c>
       <c r="O6">
-        <v>651521.93999999994</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>961667.35</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -929,28 +932,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>3988161.03</v>
+        <v>5471225.2199999997</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>23928966.199999999</v>
+        <v>26261881.07</v>
       </c>
       <c r="L7">
-        <v>33.47</v>
+        <v>36.729999999999997</v>
       </c>
       <c r="M7">
-        <v>997040.26</v>
+        <v>1094245.04</v>
       </c>
       <c r="N7">
-        <v>3375591.95</v>
+        <v>3475198.67</v>
       </c>
       <c r="O7">
-        <v>8989234.3699999992</v>
+        <v>-62422.63</v>
       </c>
       <c r="P7">
-        <v>1424928.1</v>
+        <v>186105.37</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -982,28 +985,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>6099563.8300000001</v>
+        <v>6710619.8300000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36597382.990000002</v>
+        <v>32210975.190000001</v>
       </c>
       <c r="L8">
-        <v>83.18</v>
+        <v>73.209999999999994</v>
       </c>
       <c r="M8">
-        <v>1524890.96</v>
+        <v>1342123.97</v>
       </c>
       <c r="N8">
-        <v>1895021.81</v>
+        <v>1962598.96</v>
       </c>
       <c r="O8">
-        <v>2942910.32</v>
+        <v>-98816.91</v>
       </c>
       <c r="P8">
-        <v>3401918.13</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1020,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1030,9 +1033,10 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1057,8 +1061,11 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1078,13 +1085,16 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I2">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1104,13 +1114,16 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1130,13 +1143,16 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.4</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1156,13 +1172,16 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1182,13 +1201,16 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1208,13 +1230,16 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1234,13 +1259,16 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.4</v>
+      </c>
+      <c r="I8">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1257,16 +1285,19 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1283,13 +1314,16 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H10">
-        <v>0.6</v>
+        <v>0.8</v>
+      </c>
+      <c r="I10">
+        <v>1.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-06_1442 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35FF4162-B26A-4B8A-8A7F-1F36D78549CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{24ABF4E6-A6F5-4DC0-B9B9-C1476D18C135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,7 +580,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -667,25 +668,25 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>533324.49</v>
+        <v>489485.05</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2559957.5299999998</v>
+        <v>1957940.19</v>
       </c>
       <c r="L2">
-        <v>46.54</v>
+        <v>35.6</v>
       </c>
       <c r="M2">
-        <v>106664.9</v>
+        <v>81580.84</v>
       </c>
       <c r="N2">
-        <v>261403.97</v>
+        <v>278361.94</v>
       </c>
       <c r="O2">
-        <v>312000.53000000003</v>
+        <v>33779.980000000003</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -720,28 +721,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>17543860.710000001</v>
+        <v>18895811.32</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>84210531.409999996</v>
+        <v>75583245.280000001</v>
       </c>
       <c r="L3">
-        <v>170.12</v>
+        <v>152.69</v>
       </c>
       <c r="M3">
-        <v>3508772.14</v>
+        <v>3149301.89</v>
       </c>
       <c r="N3">
-        <v>1681902.07</v>
+        <v>1700232.7</v>
       </c>
       <c r="O3">
-        <v>46225.75</v>
+        <v>27787.5</v>
       </c>
       <c r="P3">
-        <v>140558.04</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -779,22 +780,22 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>34550053.640000001</v>
+        <v>28791711.370000001</v>
       </c>
       <c r="L4">
-        <v>30.64</v>
+        <v>25.54</v>
       </c>
       <c r="M4">
-        <v>1439585.57</v>
+        <v>1199654.6399999999</v>
       </c>
       <c r="N4">
-        <v>5555372.2199999997</v>
+        <v>5864004.0099999998</v>
       </c>
       <c r="O4">
-        <v>1993306.04</v>
+        <v>3986949.21</v>
       </c>
       <c r="P4">
-        <v>5448882.6299999999</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -826,25 +827,25 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>566355.03</v>
+        <v>890289.1</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2718504.13</v>
+        <v>3561156.41</v>
       </c>
       <c r="L5">
-        <v>19.77</v>
+        <v>25.9</v>
       </c>
       <c r="M5">
-        <v>113271.01</v>
+        <v>148381.51999999999</v>
       </c>
       <c r="N5">
-        <v>693876.05</v>
+        <v>714428.38</v>
       </c>
       <c r="O5">
-        <v>95470.23</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -885,19 +886,19 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5400735.7699999996</v>
+        <v>4500613.1399999997</v>
       </c>
       <c r="L6">
-        <v>16.37</v>
+        <v>13.64</v>
       </c>
       <c r="M6">
-        <v>225030.66</v>
+        <v>187525.55</v>
       </c>
       <c r="N6">
-        <v>1677623.51</v>
+        <v>1770824.82</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>70516.2</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -932,28 +933,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>5471225.2199999997</v>
+        <v>41681218.509999998</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>26261881.07</v>
+        <v>166724874.05000001</v>
       </c>
       <c r="L7">
-        <v>36.729999999999997</v>
+        <v>233.18</v>
       </c>
       <c r="M7">
-        <v>1094245.04</v>
+        <v>6946869.75</v>
       </c>
       <c r="N7">
-        <v>3475198.67</v>
+        <v>1656598.97</v>
       </c>
       <c r="O7">
-        <v>-62422.63</v>
+        <v>749207.62</v>
       </c>
       <c r="P7">
-        <v>186105.37</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -991,19 +992,19 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>32210975.190000001</v>
+        <v>26842479.32</v>
       </c>
       <c r="L8">
-        <v>73.209999999999994</v>
+        <v>61.01</v>
       </c>
       <c r="M8">
-        <v>1342123.97</v>
+        <v>1118436.6399999999</v>
       </c>
       <c r="N8">
-        <v>1962598.96</v>
+        <v>2071632.23</v>
       </c>
       <c r="O8">
-        <v>-98816.91</v>
+        <v>4067910.56</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1088,7 +1089,7 @@
         <v>41</v>
       </c>
       <c r="H2">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="I2">
         <v>3.1</v>
@@ -1175,7 +1176,7 @@
         <v>41</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1233,7 +1234,7 @@
         <v>41</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1262,10 +1263,10 @@
         <v>41</v>
       </c>
       <c r="H8">
-        <v>1.4</v>
+        <v>0.2</v>
       </c>
       <c r="I8">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1291,7 +1292,7 @@
         <v>43</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1320,10 +1321,10 @@
         <v>43</v>
       </c>
       <c r="H10">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I10">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-08_1827 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24ABF4E6-A6F5-4DC0-B9B9-C1476D18C135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{394C0C2C-EE5F-48B1-851B-D107CA8AEB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>PorcRechazo</t>
-  </si>
-  <si>
-    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -230,12 +227,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
-  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -244,7 +241,6 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -580,8 +576,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -668,28 +663,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>489485.05</v>
+        <v>566470.78</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1957940.19</v>
+        <v>1942185.54</v>
       </c>
       <c r="L2">
-        <v>35.6</v>
+        <v>35.31</v>
       </c>
       <c r="M2">
-        <v>81580.84</v>
+        <v>80924.399999999994</v>
       </c>
       <c r="N2">
-        <v>278361.94</v>
+        <v>290207.59999999998</v>
       </c>
       <c r="O2">
-        <v>33779.980000000003</v>
+        <v>56232.47</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>421519.04</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -721,28 +716,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>18895811.32</v>
+        <v>19472957.550000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>75583245.280000001</v>
+        <v>66764425.880000003</v>
       </c>
       <c r="L3">
-        <v>152.69</v>
+        <v>134.88</v>
       </c>
       <c r="M3">
-        <v>3149301.89</v>
+        <v>2781851.08</v>
       </c>
       <c r="N3">
-        <v>1700232.7</v>
+        <v>1766296.61</v>
       </c>
       <c r="O3">
-        <v>27787.5</v>
+        <v>1062370.01</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>1730949.72</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -774,28 +769,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>7197927.8399999999</v>
+        <v>18205195.670000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>28791711.370000001</v>
+        <v>62417813.740000002</v>
       </c>
       <c r="L4">
-        <v>25.54</v>
+        <v>55.36</v>
       </c>
       <c r="M4">
-        <v>1199654.6399999999</v>
+        <v>2600742.2400000002</v>
       </c>
       <c r="N4">
-        <v>5864004.0099999998</v>
+        <v>5561459.0800000001</v>
       </c>
       <c r="O4">
-        <v>3986949.21</v>
+        <v>1746652.89</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>2186623.9700000002</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -833,22 +828,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3561156.41</v>
+        <v>3052419.78</v>
       </c>
       <c r="L5">
-        <v>25.9</v>
+        <v>22.2</v>
       </c>
       <c r="M5">
-        <v>148381.51999999999</v>
+        <v>127184.16</v>
       </c>
       <c r="N5">
-        <v>714428.38</v>
+        <v>756453.58</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>42406.31</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -880,28 +875,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>1125153.29</v>
+        <v>1247379.32</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4500613.1399999997</v>
+        <v>4276729.0999999996</v>
       </c>
       <c r="L6">
-        <v>13.64</v>
+        <v>12.96</v>
       </c>
       <c r="M6">
-        <v>187525.55</v>
+        <v>178197.05</v>
       </c>
       <c r="N6">
-        <v>1770824.82</v>
+        <v>1867801.22</v>
       </c>
       <c r="O6">
-        <v>70516.2</v>
+        <v>29231.45</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>892709.03</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -933,28 +928,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>41681218.509999998</v>
+        <v>43032855.130000003</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>166724874.05000001</v>
+        <v>147541217.59999999</v>
       </c>
       <c r="L7">
-        <v>233.18</v>
+        <v>206.35</v>
       </c>
       <c r="M7">
-        <v>6946869.75</v>
+        <v>6147550.7300000004</v>
       </c>
       <c r="N7">
-        <v>1656598.97</v>
+        <v>1674537.93</v>
       </c>
       <c r="O7">
-        <v>749207.62</v>
+        <v>973398.85</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>2889532.65</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -986,28 +981,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>6710619.8300000001</v>
+        <v>7795671.6799999997</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>26842479.32</v>
+        <v>26728017.190000001</v>
       </c>
       <c r="L8">
-        <v>61.01</v>
+        <v>60.75</v>
       </c>
       <c r="M8">
-        <v>1118436.6399999999</v>
+        <v>1113667.3799999999</v>
       </c>
       <c r="N8">
-        <v>2071632.23</v>
+        <v>2129666.37</v>
       </c>
       <c r="O8">
-        <v>4067910.56</v>
+        <v>550253.22</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>1037184.12</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1024,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1034,10 +1029,9 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1062,11 +1056,8 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1086,16 +1077,13 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="I2">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1115,16 +1103,13 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>0.3</v>
-      </c>
-      <c r="I3">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1144,16 +1129,13 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H4">
         <v>0.4</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1173,16 +1155,13 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H5">
-        <v>9</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1202,16 +1181,13 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1231,16 +1207,13 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7">
         <v>0.2</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1260,16 +1233,13 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8">
         <v>0.2</v>
       </c>
-      <c r="I8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1286,19 +1256,16 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
         <v>42</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
       </c>
       <c r="H9">
         <v>0.4</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1315,16 +1282,13 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
       <c r="H10">
-        <v>0.5</v>
-      </c>
-      <c r="I10">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-09_1733 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{394C0C2C-EE5F-48B1-851B-D107CA8AEB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35024E6C-5596-446B-882D-61887EC95633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>PorcRechazo</t>
+  </si>
+  <si>
+    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -227,12 +230,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
+  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="8">
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -241,6 +244,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -576,7 +580,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -663,28 +668,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>566470.78</v>
+        <v>748251.27</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1942185.54</v>
+        <v>2244753.81</v>
       </c>
       <c r="L2">
-        <v>35.31</v>
+        <v>40.81</v>
       </c>
       <c r="M2">
-        <v>80924.399999999994</v>
+        <v>93531.41</v>
       </c>
       <c r="N2">
-        <v>290207.59999999998</v>
+        <v>296984.3</v>
       </c>
       <c r="O2">
-        <v>56232.47</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>421519.04</v>
+        <v>-10112.450000000001</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -716,28 +721,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>19472957.550000001</v>
+        <v>20961798.32</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>66764425.880000003</v>
+        <v>62885394.960000001</v>
       </c>
       <c r="L3">
-        <v>134.88</v>
+        <v>127.04</v>
       </c>
       <c r="M3">
-        <v>2781851.08</v>
+        <v>2620224.79</v>
       </c>
       <c r="N3">
-        <v>1766296.61</v>
+        <v>1783637.6</v>
       </c>
       <c r="O3">
-        <v>1062370.01</v>
+        <v>1050812.26</v>
       </c>
       <c r="P3">
-        <v>1730949.72</v>
+        <v>876986.28</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -769,28 +774,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>18205195.670000002</v>
+        <v>19554421.84</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>62417813.740000002</v>
+        <v>58663265.530000001</v>
       </c>
       <c r="L4">
-        <v>55.36</v>
+        <v>52.03</v>
       </c>
       <c r="M4">
-        <v>2600742.2400000002</v>
+        <v>2444302.73</v>
       </c>
       <c r="N4">
-        <v>5561459.0800000001</v>
+        <v>5824723.6299999999</v>
       </c>
       <c r="O4">
-        <v>1746652.89</v>
+        <v>809081.6</v>
       </c>
       <c r="P4">
-        <v>2186623.9700000002</v>
+        <v>1149986.8700000001</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -822,28 +827,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>890289.1</v>
+        <v>940184.06</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3052419.78</v>
+        <v>2820552.19</v>
       </c>
       <c r="L5">
-        <v>22.2</v>
+        <v>20.51</v>
       </c>
       <c r="M5">
-        <v>127184.16</v>
+        <v>117523.01</v>
       </c>
       <c r="N5">
-        <v>756453.58</v>
+        <v>800613.5</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>296224</v>
       </c>
       <c r="P5">
-        <v>42406.31</v>
+        <v>192659.8</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -875,28 +880,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>1247379.32</v>
+        <v>1443220.99</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4276729.0999999996</v>
+        <v>4329662.97</v>
       </c>
       <c r="L6">
-        <v>12.96</v>
+        <v>13.12</v>
       </c>
       <c r="M6">
-        <v>178197.05</v>
+        <v>180402.62</v>
       </c>
       <c r="N6">
-        <v>1867801.22</v>
+        <v>1972298.69</v>
       </c>
       <c r="O6">
-        <v>29231.45</v>
+        <v>386320.62</v>
       </c>
       <c r="P6">
-        <v>892709.03</v>
+        <v>2511554.75</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -928,28 +933,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>43032855.130000003</v>
+        <v>43942640.07</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>147541217.59999999</v>
+        <v>131827920.22</v>
       </c>
       <c r="L7">
-        <v>206.35</v>
+        <v>184.37</v>
       </c>
       <c r="M7">
-        <v>6147550.7300000004</v>
+        <v>5492830.0099999998</v>
       </c>
       <c r="N7">
-        <v>1674537.93</v>
+        <v>1722335</v>
       </c>
       <c r="O7">
-        <v>973398.85</v>
+        <v>455655.86</v>
       </c>
       <c r="P7">
-        <v>2889532.65</v>
+        <v>6553989.9900000002</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -981,28 +986,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>7795671.6799999997</v>
+        <v>8102990.4199999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>26728017.190000001</v>
+        <v>24308971.25</v>
       </c>
       <c r="L8">
-        <v>60.75</v>
+        <v>55.25</v>
       </c>
       <c r="M8">
-        <v>1113667.3799999999</v>
+        <v>1012873.8</v>
       </c>
       <c r="N8">
-        <v>2129666.37</v>
+        <v>2243563.1</v>
       </c>
       <c r="O8">
-        <v>550253.22</v>
+        <v>502369.56</v>
       </c>
       <c r="P8">
-        <v>1037184.12</v>
+        <v>1200502.3400000001</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1019,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1029,9 +1034,10 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1056,8 +1062,11 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1077,13 +1086,16 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2.1</v>
+      </c>
+      <c r="I2">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1103,13 +1115,16 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I3">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1129,13 +1144,16 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.6</v>
+      </c>
+      <c r="I4">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1155,13 +1173,16 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5">
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>5.9</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1181,13 +1202,16 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1207,13 +1231,16 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1233,13 +1260,16 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H8">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1256,16 +1286,19 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H9">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.3</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1282,13 +1315,16 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H10">
-        <v>0.4</v>
+        <v>0.6</v>
+      </c>
+      <c r="I10">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-10_1825 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35024E6C-5596-446B-882D-61887EC95633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A10B9D0-18C1-424E-8C07-C897E10C323A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>PorcRechazo</t>
-  </si>
-  <si>
-    <t>PorcCambio</t>
   </si>
   <si>
     <t>Vendedor</t>
@@ -230,12 +227,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:I10">
-  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
     <sortCondition ref="E2:E10"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
@@ -244,7 +241,6 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="PorcCambio"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -674,22 +670,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2244753.81</v>
+        <v>1995336.72</v>
       </c>
       <c r="L2">
-        <v>40.81</v>
+        <v>36.28</v>
       </c>
       <c r="M2">
-        <v>93531.41</v>
+        <v>83139.03</v>
       </c>
       <c r="N2">
-        <v>296984.3</v>
+        <v>316783.25</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>443312.03</v>
       </c>
       <c r="P2">
-        <v>-10112.450000000001</v>
+        <v>214398.45</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -721,28 +717,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>20961798.32</v>
+        <v>22213061.390000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>62885394.960000001</v>
+        <v>59234830.369999997</v>
       </c>
       <c r="L3">
-        <v>127.04</v>
+        <v>119.67</v>
       </c>
       <c r="M3">
-        <v>2620224.79</v>
+        <v>2468117.9300000002</v>
       </c>
       <c r="N3">
-        <v>1783637.6</v>
+        <v>1819129.24</v>
       </c>
       <c r="O3">
-        <v>1050812.26</v>
+        <v>6833382.5700000003</v>
       </c>
       <c r="P3">
-        <v>876986.28</v>
+        <v>2185505.7999999998</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -774,28 +770,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>19554421.84</v>
+        <v>21250760.370000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>58663265.530000001</v>
+        <v>56668694.32</v>
       </c>
       <c r="L4">
-        <v>52.03</v>
+        <v>50.26</v>
       </c>
       <c r="M4">
-        <v>2444302.73</v>
+        <v>2361195.6</v>
       </c>
       <c r="N4">
-        <v>5824723.6299999999</v>
+        <v>6099949.3099999996</v>
       </c>
       <c r="O4">
-        <v>809081.6</v>
+        <v>239873.97</v>
       </c>
       <c r="P4">
-        <v>1149986.8700000001</v>
+        <v>1294302.58</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -827,28 +823,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>940184.06</v>
+        <v>1220559.8</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2820552.19</v>
+        <v>3254826.12</v>
       </c>
       <c r="L5">
-        <v>20.51</v>
+        <v>23.67</v>
       </c>
       <c r="M5">
-        <v>117523.01</v>
+        <v>135617.76</v>
       </c>
       <c r="N5">
-        <v>800613.5</v>
+        <v>835296.01</v>
       </c>
       <c r="O5">
-        <v>296224</v>
+        <v>80769.37</v>
       </c>
       <c r="P5">
-        <v>192659.8</v>
+        <v>36524.79</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -880,28 +876,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>1443220.99</v>
+        <v>1551861.7</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4329662.97</v>
+        <v>4138297.87</v>
       </c>
       <c r="L6">
-        <v>13.12</v>
+        <v>12.54</v>
       </c>
       <c r="M6">
-        <v>180402.62</v>
+        <v>172429.08</v>
       </c>
       <c r="N6">
-        <v>1972298.69</v>
+        <v>2096542.55</v>
       </c>
       <c r="O6">
-        <v>386320.62</v>
+        <v>240862.15</v>
       </c>
       <c r="P6">
-        <v>2511554.75</v>
+        <v>2509730.8199999998</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -933,28 +929,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>43942640.07</v>
+        <v>44132519.969999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>131827920.22</v>
+        <v>117686719.91</v>
       </c>
       <c r="L7">
-        <v>184.37</v>
+        <v>164.6</v>
       </c>
       <c r="M7">
-        <v>5492830.0099999998</v>
+        <v>4903613.33</v>
       </c>
       <c r="N7">
-        <v>1722335</v>
+        <v>1824498.67</v>
       </c>
       <c r="O7">
-        <v>455655.86</v>
+        <v>357851.28</v>
       </c>
       <c r="P7">
-        <v>6553989.9900000002</v>
+        <v>575210.05000000005</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -986,28 +982,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>8102990.4199999999</v>
+        <v>9534288.8900000006</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>24308971.25</v>
+        <v>25424770.370000001</v>
       </c>
       <c r="L8">
-        <v>55.25</v>
+        <v>57.78</v>
       </c>
       <c r="M8">
-        <v>1012873.8</v>
+        <v>1059365.43</v>
       </c>
       <c r="N8">
-        <v>2243563.1</v>
+        <v>2297714.0699999998</v>
       </c>
       <c r="O8">
-        <v>502369.56</v>
+        <v>266540.59999999998</v>
       </c>
       <c r="P8">
-        <v>1200502.3400000001</v>
+        <v>741600.26</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1024,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1034,10 +1030,9 @@
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -1062,11 +1057,8 @@
       <c r="H1" t="s">
         <v>39</v>
       </c>
-      <c r="I1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>105021</v>
       </c>
@@ -1086,16 +1078,13 @@
         <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>2.1</v>
-      </c>
-      <c r="I2">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>105021</v>
       </c>
@@ -1115,16 +1104,13 @@
         <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="I3">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>105021</v>
       </c>
@@ -1144,16 +1130,13 @@
         <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>0.6</v>
-      </c>
-      <c r="I4">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>106002</v>
       </c>
@@ -1173,16 +1156,13 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H5">
         <v>5.9</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>105021</v>
       </c>
@@ -1202,16 +1182,13 @@
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>106002</v>
       </c>
@@ -1231,16 +1208,13 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7">
         <v>0.1</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>105021</v>
       </c>
@@ -1260,16 +1234,13 @@
         <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8">
         <v>0.2</v>
       </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>106002</v>
       </c>
@@ -1286,19 +1257,16 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
         <v>42</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
       </c>
       <c r="H9">
         <v>0.3</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>105021</v>
       </c>
@@ -1315,16 +1283,13 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="G10" t="s">
-        <v>43</v>
-      </c>
       <c r="H10">
-        <v>0.6</v>
-      </c>
-      <c r="I10">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-11_2115 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A10B9D0-18C1-424E-8C07-C897E10C323A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{76499CC0-00F1-4939-B5CC-598EA20CC559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="47">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -117,6 +117,12 @@
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>LUDUEÑA JULIANA</t>
+  </si>
+  <si>
     <t>10</t>
   </si>
   <si>
@@ -127,6 +133,12 @@
   </si>
   <si>
     <t>PEYRONEL ANDREA</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>VERGARA MARIA JOSE</t>
   </si>
   <si>
     <t>SupervisorId</t>
@@ -203,6 +215,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
   <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q8">
+    <sortCondition ref="D2:D8"/>
+  </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -227,11 +242,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
-    <sortCondition ref="E2:E10"/>
-  </sortState>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H12">
+  <autoFilter ref="A1:H12" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
@@ -640,19 +652,19 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C2">
-        <v>105007</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
+        <v>105003</v>
+      </c>
+      <c r="D2" s="1">
+        <v>3</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
         <v>21</v>
@@ -661,31 +673,31 @@
         <v>22</v>
       </c>
       <c r="H2">
-        <v>5500000</v>
+        <v>13750000</v>
       </c>
       <c r="I2">
-        <v>748251.27</v>
+        <v>1290152</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1995336.72</v>
+        <v>3096364.79</v>
       </c>
       <c r="L2">
-        <v>36.28</v>
+        <v>22.52</v>
       </c>
       <c r="M2">
-        <v>83139.03</v>
+        <v>129015.2</v>
       </c>
       <c r="N2">
-        <v>316783.25</v>
+        <v>889989.14</v>
       </c>
       <c r="O2">
-        <v>443312.03</v>
+        <v>93891.42</v>
       </c>
       <c r="P2">
-        <v>214398.45</v>
+        <v>33811.69</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -693,19 +705,19 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C3">
-        <v>120039</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
+        <v>105004</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
         <v>21</v>
@@ -714,31 +726,31 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>49500000</v>
+        <v>33000000</v>
       </c>
       <c r="I3">
-        <v>22213061.390000001</v>
+        <v>1818665.25</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>59234830.369999997</v>
+        <v>4364796.59</v>
       </c>
       <c r="L3">
-        <v>119.67</v>
+        <v>13.23</v>
       </c>
       <c r="M3">
-        <v>2468117.9300000002</v>
+        <v>181866.52</v>
       </c>
       <c r="N3">
-        <v>1819129.24</v>
+        <v>2227238.2000000002</v>
       </c>
       <c r="O3">
-        <v>6833382.5700000003</v>
+        <v>143378.76999999999</v>
       </c>
       <c r="P3">
-        <v>2185505.7999999998</v>
+        <v>651521.93999999994</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -752,13 +764,13 @@
         <v>26</v>
       </c>
       <c r="C4">
-        <v>105008</v>
-      </c>
-      <c r="D4" t="s">
-        <v>27</v>
+        <v>105006</v>
+      </c>
+      <c r="D4" s="1">
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
         <v>21</v>
@@ -767,31 +779,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>112750000</v>
+        <v>44000000</v>
       </c>
       <c r="I4">
-        <v>21250760.370000001</v>
+        <v>9621738.9900000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>56668694.32</v>
+        <v>23092173.559999999</v>
       </c>
       <c r="L4">
-        <v>50.26</v>
+        <v>52.48</v>
       </c>
       <c r="M4">
-        <v>2361195.6</v>
+        <v>962173.9</v>
       </c>
       <c r="N4">
-        <v>6099949.3099999996</v>
+        <v>2455590.0699999998</v>
       </c>
       <c r="O4">
-        <v>239873.97</v>
+        <v>611056</v>
       </c>
       <c r="P4">
-        <v>1294302.58</v>
+        <v>2942910.32</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -799,19 +811,19 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C5">
-        <v>105003</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
+        <v>105007</v>
+      </c>
+      <c r="D5" s="1">
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
         <v>21</v>
@@ -820,31 +832,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>13750000</v>
+        <v>5500000</v>
       </c>
       <c r="I5">
-        <v>1220559.8</v>
+        <v>997168.06</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3254826.12</v>
+        <v>2393203.34</v>
       </c>
       <c r="L5">
-        <v>23.67</v>
+        <v>43.51</v>
       </c>
       <c r="M5">
-        <v>135617.76</v>
+        <v>99716.81</v>
       </c>
       <c r="N5">
-        <v>835296.01</v>
+        <v>321630.84999999998</v>
       </c>
       <c r="O5">
-        <v>80769.37</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>36524.79</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -858,13 +870,13 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>105004</v>
-      </c>
-      <c r="D6" t="s">
-        <v>31</v>
+        <v>105008</v>
+      </c>
+      <c r="D6" s="1">
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -873,31 +885,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>33000000</v>
+        <v>112750000</v>
       </c>
       <c r="I6">
-        <v>1551861.7</v>
+        <v>22077612.890000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4138297.87</v>
+        <v>52986270.939999998</v>
       </c>
       <c r="L6">
-        <v>12.54</v>
+        <v>46.99</v>
       </c>
       <c r="M6">
-        <v>172429.08</v>
+        <v>2207761.29</v>
       </c>
       <c r="N6">
-        <v>2096542.55</v>
+        <v>6476599.0800000001</v>
       </c>
       <c r="O6">
-        <v>240862.15</v>
+        <v>167814.97</v>
       </c>
       <c r="P6">
-        <v>2509730.8199999998</v>
+        <v>-1619390.32</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -905,19 +917,19 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C7">
-        <v>120041</v>
-      </c>
-      <c r="D7" t="s">
-        <v>33</v>
+        <v>120039</v>
+      </c>
+      <c r="D7" s="1">
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
         <v>21</v>
@@ -926,31 +938,31 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>71500000</v>
+        <v>49500000</v>
       </c>
       <c r="I7">
-        <v>44132519.969999999</v>
+        <v>22728548.690000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>117686719.91</v>
+        <v>54548516.859999999</v>
       </c>
       <c r="L7">
-        <v>164.6</v>
+        <v>110.2</v>
       </c>
       <c r="M7">
-        <v>4903613.33</v>
+        <v>2272854.87</v>
       </c>
       <c r="N7">
-        <v>1824498.67</v>
+        <v>1912246.52</v>
       </c>
       <c r="O7">
-        <v>357851.28</v>
+        <v>8484253.4100000001</v>
       </c>
       <c r="P7">
-        <v>575210.05000000005</v>
+        <v>2494350.0299999998</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -964,10 +976,10 @@
         <v>26</v>
       </c>
       <c r="C8">
-        <v>105006</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
+        <v>120041</v>
+      </c>
+      <c r="D8" s="1">
+        <v>10</v>
       </c>
       <c r="E8" t="s">
         <v>36</v>
@@ -979,31 +991,31 @@
         <v>22</v>
       </c>
       <c r="H8">
-        <v>44000000</v>
+        <v>71500000</v>
       </c>
       <c r="I8">
-        <v>9534288.8900000006</v>
+        <v>44778132.880000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>25424770.370000001</v>
+        <v>107467518.92</v>
       </c>
       <c r="L8">
-        <v>57.78</v>
+        <v>150.30000000000001</v>
       </c>
       <c r="M8">
-        <v>1059365.43</v>
+        <v>4477813.29</v>
       </c>
       <c r="N8">
-        <v>2297714.0699999998</v>
+        <v>1908704.79</v>
       </c>
       <c r="O8">
-        <v>266540.59999999998</v>
+        <v>1483064.19</v>
       </c>
       <c r="P8">
-        <v>741600.26</v>
+        <v>8989234.3699999992</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1020,7 +1032,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1034,7 +1046,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1052,10 +1064,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1069,19 +1081,19 @@
         <v>26</v>
       </c>
       <c r="D2">
-        <v>105003</v>
-      </c>
-      <c r="E2" s="1">
-        <v>3</v>
+        <v>120008</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1095,19 +1107,19 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>105004</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4</v>
+        <v>105006</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1121,45 +1133,45 @@
         <v>26</v>
       </c>
       <c r="D4">
-        <v>105006</v>
-      </c>
-      <c r="E4" s="1">
-        <v>6</v>
+        <v>105004</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H4">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>106002</v>
+        <v>105021</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D5">
-        <v>105007</v>
-      </c>
-      <c r="E5" s="1">
-        <v>7</v>
+        <v>105002</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H5">
-        <v>5.9</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1173,19 +1185,19 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>105008</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8</v>
+        <v>105003</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1201,69 +1213,69 @@
       <c r="D7">
         <v>120039</v>
       </c>
-      <c r="E7" s="1">
-        <v>9</v>
+      <c r="E7" t="s">
+        <v>23</v>
       </c>
       <c r="F7" t="s">
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H7">
-        <v>0.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>105021</v>
+        <v>106002</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D8">
-        <v>120041</v>
-      </c>
-      <c r="E8" s="1">
-        <v>10</v>
+        <v>105007</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H8">
-        <v>0.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>106002</v>
+        <v>105021</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D9">
-        <v>106002</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1002</v>
+        <v>105008</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H9">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1277,19 +1289,71 @@
         <v>26</v>
       </c>
       <c r="D10">
+        <v>120041</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>105021</v>
       </c>
-      <c r="E10" s="1">
-        <v>20032</v>
-      </c>
-      <c r="F10" t="s">
-        <v>41</v>
-      </c>
-      <c r="G10" t="s">
-        <v>42</v>
-      </c>
-      <c r="H10">
-        <v>0.5</v>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11">
+        <v>105021</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>106002</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12">
+        <v>106002</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12">
+        <v>1.1000000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-12_1726 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76499CC0-00F1-4939-B5CC-598EA20CC559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1AA527A-2A0C-40F0-AF7A-08CC73CA3B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="36">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -75,9 +75,6 @@
     <t>BENITEZ RAUL</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>JOFRE GUILLERMO AGUSTIN</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>PEÑAFLOR GRUPO OBJETIVO</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>SANCHEZ FERNANDO JAVIER</t>
   </si>
   <si>
@@ -99,46 +93,19 @@
     <t>GRIBAUDO ESTEBAN</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>ALVAREZ VANESA  KAFF</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>GAMBINO NADIA</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>LUDUEÑA JULIANA</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>ORTEGA MILAGROS DESIREE</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>PEYRONEL ANDREA</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>VERGARA MARIA JOSE</t>
   </si>
   <si>
     <t>SupervisorId</t>
@@ -215,9 +182,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
   <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q8">
-    <sortCondition ref="D2:D8"/>
-  </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -242,8 +206,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H12">
-  <autoFilter ref="A1:H12" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
+    <sortCondition ref="E2:E10"/>
+  </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
@@ -588,8 +555,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -652,52 +618,52 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C2">
-        <v>105003</v>
+        <v>105007</v>
       </c>
       <c r="D2" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
-        <v>22</v>
-      </c>
       <c r="H2">
-        <v>13750000</v>
+        <v>5500000</v>
       </c>
       <c r="I2">
-        <v>1290152</v>
+        <v>997168.06</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3096364.79</v>
+        <v>2175639.4</v>
       </c>
       <c r="L2">
-        <v>22.52</v>
+        <v>39.56</v>
       </c>
       <c r="M2">
-        <v>129015.2</v>
+        <v>90651.64</v>
       </c>
       <c r="N2">
-        <v>889989.14</v>
+        <v>346371.69</v>
       </c>
       <c r="O2">
-        <v>93891.42</v>
+        <v>76985.73</v>
       </c>
       <c r="P2">
-        <v>33811.69</v>
+        <v>33779.980000000003</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -705,52 +671,52 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C3">
-        <v>105004</v>
+        <v>120039</v>
       </c>
       <c r="D3" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
       <c r="H3">
-        <v>33000000</v>
+        <v>49500000</v>
       </c>
       <c r="I3">
-        <v>1818665.25</v>
+        <v>24282038.760000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>4364796.59</v>
+        <v>52978993.649999999</v>
       </c>
       <c r="L3">
-        <v>13.23</v>
+        <v>107.03</v>
       </c>
       <c r="M3">
-        <v>181866.52</v>
+        <v>2207458.0699999998</v>
       </c>
       <c r="N3">
-        <v>2227238.2000000002</v>
+        <v>1939843.17</v>
       </c>
       <c r="O3">
-        <v>143378.76999999999</v>
+        <v>577146.23</v>
       </c>
       <c r="P3">
-        <v>651521.93999999994</v>
+        <v>27787.5</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -758,52 +724,52 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4">
+        <v>105008</v>
+      </c>
+      <c r="D4" s="1">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4">
-        <v>105006</v>
-      </c>
-      <c r="D4" s="1">
-        <v>6</v>
-      </c>
-      <c r="E4" t="s">
-        <v>38</v>
-      </c>
       <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
       <c r="H4">
-        <v>44000000</v>
+        <v>112750000</v>
       </c>
       <c r="I4">
-        <v>9621738.9900000002</v>
+        <v>25044307.879999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>23092173.559999999</v>
+        <v>54642126.289999999</v>
       </c>
       <c r="L4">
-        <v>52.48</v>
+        <v>48.46</v>
       </c>
       <c r="M4">
-        <v>962173.9</v>
+        <v>2276755.2599999998</v>
       </c>
       <c r="N4">
-        <v>2455590.0699999998</v>
+        <v>6746591.7000000002</v>
       </c>
       <c r="O4">
-        <v>611056</v>
+        <v>11007267.83</v>
       </c>
       <c r="P4">
-        <v>2942910.32</v>
+        <v>3986949.21</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -811,46 +777,46 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C5">
-        <v>105007</v>
+        <v>105003</v>
       </c>
       <c r="D5" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>20</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>21</v>
       </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
       <c r="H5">
-        <v>5500000</v>
+        <v>13750000</v>
       </c>
       <c r="I5">
-        <v>997168.06</v>
+        <v>4032981.96</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2393203.34</v>
+        <v>8799233.3599999994</v>
       </c>
       <c r="L5">
-        <v>43.51</v>
+        <v>63.99</v>
       </c>
       <c r="M5">
-        <v>99716.81</v>
+        <v>366634.72</v>
       </c>
       <c r="N5">
-        <v>321630.84999999998</v>
+        <v>747462.93</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -864,52 +830,52 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6">
-        <v>105008</v>
+        <v>105004</v>
       </c>
       <c r="D6" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" t="s">
-        <v>22</v>
-      </c>
       <c r="H6">
-        <v>112750000</v>
+        <v>33000000</v>
       </c>
       <c r="I6">
-        <v>22077612.890000001</v>
+        <v>2328596.88</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>52986270.939999998</v>
+        <v>5080575.0199999996</v>
       </c>
       <c r="L6">
-        <v>46.99</v>
+        <v>15.4</v>
       </c>
       <c r="M6">
-        <v>2207761.29</v>
+        <v>211690.63</v>
       </c>
       <c r="N6">
-        <v>6476599.0800000001</v>
+        <v>2359338.7000000002</v>
       </c>
       <c r="O6">
-        <v>167814.97</v>
+        <v>122226.03</v>
       </c>
       <c r="P6">
-        <v>-1619390.32</v>
+        <v>70516.2</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -917,52 +883,52 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C7">
-        <v>120039</v>
+        <v>120041</v>
       </c>
       <c r="D7" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
         <v>21</v>
       </c>
-      <c r="G7" t="s">
-        <v>22</v>
-      </c>
       <c r="H7">
-        <v>49500000</v>
+        <v>71500000</v>
       </c>
       <c r="I7">
-        <v>22728548.690000001</v>
+        <v>59777039.710000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>54548516.859999999</v>
+        <v>130422632.09999999</v>
       </c>
       <c r="L7">
-        <v>110.2</v>
+        <v>182.41</v>
       </c>
       <c r="M7">
-        <v>2272854.87</v>
+        <v>5434276.3399999999</v>
       </c>
       <c r="N7">
-        <v>1912246.52</v>
+        <v>901766.18</v>
       </c>
       <c r="O7">
-        <v>8484253.4100000001</v>
+        <v>1351636.62</v>
       </c>
       <c r="P7">
-        <v>2494350.0299999998</v>
+        <v>749207.62</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -970,52 +936,52 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>120041</v>
+        <v>105006</v>
       </c>
       <c r="D8" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
         <v>21</v>
       </c>
-      <c r="G8" t="s">
-        <v>22</v>
-      </c>
       <c r="H8">
-        <v>71500000</v>
+        <v>44000000</v>
       </c>
       <c r="I8">
-        <v>44778132.880000003</v>
+        <v>13347070.859999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>107467518.92</v>
+        <v>29120881.870000001</v>
       </c>
       <c r="L8">
-        <v>150.30000000000001</v>
+        <v>66.180000000000007</v>
       </c>
       <c r="M8">
-        <v>4477813.29</v>
+        <v>1213370.08</v>
       </c>
       <c r="N8">
-        <v>1908704.79</v>
+        <v>2357917.63</v>
       </c>
       <c r="O8">
-        <v>1483064.19</v>
+        <v>938418.24</v>
       </c>
       <c r="P8">
-        <v>8989234.3699999992</v>
+        <v>4067910.56</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1032,7 +998,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1046,7 +1012,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1064,10 +1030,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1075,25 +1041,25 @@
         <v>105021</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2">
+        <v>105003</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
         <v>26</v>
       </c>
-      <c r="D2">
-        <v>120008</v>
-      </c>
-      <c r="E2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" t="s">
-        <v>40</v>
-      </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1101,25 +1067,25 @@
         <v>105021</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D3">
-        <v>105006</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
+        <v>105004</v>
+      </c>
+      <c r="E3" s="1">
+        <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1127,51 +1093,51 @@
         <v>105021</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D4">
-        <v>105004</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
+        <v>105006</v>
+      </c>
+      <c r="E4" s="1">
+        <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H4">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>105021</v>
+        <v>106002</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D5">
-        <v>105002</v>
-      </c>
-      <c r="E5" t="s">
+        <v>105007</v>
+      </c>
+      <c r="E5" s="1">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" t="s">
-        <v>44</v>
-      </c>
       <c r="H5">
-        <v>1.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1179,25 +1145,25 @@
         <v>105021</v>
       </c>
       <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6">
+        <v>105008</v>
+      </c>
+      <c r="E6" s="1">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6">
-        <v>105003</v>
-      </c>
-      <c r="E6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H6">
-        <v>1.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1213,14 +1179,14 @@
       <c r="D7">
         <v>120039</v>
       </c>
-      <c r="E7" t="s">
-        <v>23</v>
+      <c r="E7" s="1">
+        <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1228,54 +1194,54 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>106002</v>
+        <v>105021</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D8">
-        <v>105007</v>
-      </c>
-      <c r="E8" t="s">
-        <v>19</v>
+        <v>120041</v>
+      </c>
+      <c r="E8" s="1">
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="H8">
-        <v>4.4000000000000004</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>105021</v>
+        <v>106002</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D9">
-        <v>105008</v>
-      </c>
-      <c r="E9" t="s">
-        <v>27</v>
+        <v>106002</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="H9">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1283,77 +1249,25 @@
         <v>105021</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D10">
-        <v>120041</v>
-      </c>
-      <c r="E10" t="s">
+        <v>105021</v>
+      </c>
+      <c r="E10" s="1">
+        <v>20032</v>
+      </c>
+      <c r="F10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" t="s">
         <v>35</v>
       </c>
-      <c r="F10" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" t="s">
-        <v>44</v>
-      </c>
       <c r="H10">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>105021</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11">
-        <v>105021</v>
-      </c>
-      <c r="E11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" t="s">
-        <v>46</v>
-      </c>
-      <c r="H11">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>106002</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12">
-        <v>106002</v>
-      </c>
-      <c r="E12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-13_1410 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1AA527A-2A0C-40F0-AF7A-08CC73CA3B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CD9DF07-5E31-4494-A6C6-448C75764BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -75,6 +75,9 @@
     <t>BENITEZ RAUL</t>
   </si>
   <si>
+    <t>7</t>
+  </si>
+  <si>
     <t>JOFRE GUILLERMO AGUSTIN</t>
   </si>
   <si>
@@ -84,6 +87,9 @@
     <t>PEÑAFLOR GRUPO OBJETIVO</t>
   </si>
   <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>SANCHEZ FERNANDO JAVIER</t>
   </si>
   <si>
@@ -93,16 +99,31 @@
     <t>GRIBAUDO ESTEBAN</t>
   </si>
   <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>ALVAREZ VANESA  KAFF</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>GAMBINO NADIA</t>
   </si>
   <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>ORTEGA MILAGROS DESIREE</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
   <si>
     <t>PEYRONEL ANDREA</t>
@@ -555,7 +576,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -626,17 +648,17 @@
       <c r="C2">
         <v>105007</v>
       </c>
-      <c r="D2" s="1">
-        <v>7</v>
+      <c r="D2" t="s">
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H2">
         <v>5500000</v>
@@ -648,22 +670,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2175639.4</v>
+        <v>1994336.11</v>
       </c>
       <c r="L2">
-        <v>39.56</v>
+        <v>36.26</v>
       </c>
       <c r="M2">
-        <v>90651.64</v>
+        <v>83097.34</v>
       </c>
       <c r="N2">
-        <v>346371.69</v>
+        <v>375236</v>
       </c>
       <c r="O2">
-        <v>76985.73</v>
+        <v>181780.49</v>
       </c>
       <c r="P2">
-        <v>33779.980000000003</v>
+        <v>56232.47</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -679,44 +701,44 @@
       <c r="C3">
         <v>120039</v>
       </c>
-      <c r="D3" s="1">
-        <v>9</v>
+      <c r="D3" t="s">
+        <v>23</v>
       </c>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
         <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
       </c>
       <c r="H3">
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>24282038.760000002</v>
+        <v>24621648.550000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>52978993.649999999</v>
+        <v>49243297.109999999</v>
       </c>
       <c r="L3">
-        <v>107.03</v>
+        <v>99.48</v>
       </c>
       <c r="M3">
-        <v>2207458.0699999998</v>
+        <v>2051804.05</v>
       </c>
       <c r="N3">
-        <v>1939843.17</v>
+        <v>2073195.95</v>
       </c>
       <c r="O3">
-        <v>577146.23</v>
+        <v>1478135.97</v>
       </c>
       <c r="P3">
-        <v>27787.5</v>
+        <v>1062370.01</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -724,52 +746,52 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4">
         <v>105008</v>
       </c>
-      <c r="D4" s="1">
-        <v>8</v>
+      <c r="D4" t="s">
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4">
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>25044307.879999999</v>
+        <v>30014653.960000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>54642126.289999999</v>
+        <v>60029307.93</v>
       </c>
       <c r="L4">
-        <v>48.46</v>
+        <v>53.24</v>
       </c>
       <c r="M4">
-        <v>2276755.2599999998</v>
+        <v>2501221.16</v>
       </c>
       <c r="N4">
-        <v>6746591.7000000002</v>
+        <v>6894612.1699999999</v>
       </c>
       <c r="O4">
-        <v>11007267.83</v>
+        <v>1349226.17</v>
       </c>
       <c r="P4">
-        <v>3986949.21</v>
+        <v>1746652.89</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -777,25 +799,25 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>105003</v>
       </c>
-      <c r="D5" s="1">
-        <v>3</v>
+      <c r="D5" t="s">
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H5">
         <v>13750000</v>
@@ -807,19 +829,19 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>8799233.3599999994</v>
+        <v>8065963.9100000001</v>
       </c>
       <c r="L5">
-        <v>63.99</v>
+        <v>58.66</v>
       </c>
       <c r="M5">
-        <v>366634.72</v>
+        <v>336081.83</v>
       </c>
       <c r="N5">
-        <v>747462.93</v>
+        <v>809751.5</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>49894.96</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -830,52 +852,52 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6">
         <v>105004</v>
       </c>
-      <c r="D6" s="1">
-        <v>4</v>
+      <c r="D6" t="s">
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H6">
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>2328596.88</v>
+        <v>2339364.5499999998</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5080575.0199999996</v>
+        <v>4678729.0999999996</v>
       </c>
       <c r="L6">
-        <v>15.4</v>
+        <v>14.18</v>
       </c>
       <c r="M6">
-        <v>211690.63</v>
+        <v>194947.05</v>
       </c>
       <c r="N6">
-        <v>2359338.7000000002</v>
+        <v>2555052.9500000002</v>
       </c>
       <c r="O6">
-        <v>122226.03</v>
+        <v>-16753.03</v>
       </c>
       <c r="P6">
-        <v>70516.2</v>
+        <v>29231.45</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -883,52 +905,52 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7">
         <v>120041</v>
       </c>
-      <c r="D7" s="1">
-        <v>10</v>
+      <c r="D7" t="s">
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H7">
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>59777039.710000001</v>
+        <v>61999016.68</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>130422632.09999999</v>
+        <v>123998033.36</v>
       </c>
       <c r="L7">
-        <v>182.41</v>
+        <v>173.42</v>
       </c>
       <c r="M7">
-        <v>5434276.3399999999</v>
+        <v>5166584.72</v>
       </c>
       <c r="N7">
-        <v>901766.18</v>
+        <v>791748.61</v>
       </c>
       <c r="O7">
-        <v>1351636.62</v>
+        <v>909784.94</v>
       </c>
       <c r="P7">
-        <v>749207.62</v>
+        <v>973398.85</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -936,52 +958,52 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8">
         <v>105006</v>
       </c>
-      <c r="D8" s="1">
-        <v>6</v>
+      <c r="D8" t="s">
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H8">
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>13347070.859999999</v>
+        <v>13694839.91</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>29120881.870000001</v>
+        <v>27389679.829999998</v>
       </c>
       <c r="L8">
-        <v>66.180000000000007</v>
+        <v>62.25</v>
       </c>
       <c r="M8">
-        <v>1213370.08</v>
+        <v>1141236.6599999999</v>
       </c>
       <c r="N8">
-        <v>2357917.63</v>
+        <v>2525430.0099999998</v>
       </c>
       <c r="O8">
-        <v>938418.24</v>
+        <v>1133722.54</v>
       </c>
       <c r="P8">
-        <v>4067910.56</v>
+        <v>550253.22</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1012,7 +1034,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1030,10 +1052,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1041,10 +1063,10 @@
         <v>105021</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>105003</v>
@@ -1053,13 +1075,13 @@
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1067,10 +1089,10 @@
         <v>105021</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>105004</v>
@@ -1079,13 +1101,13 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H3">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1093,10 +1115,10 @@
         <v>105021</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4">
         <v>105006</v>
@@ -1105,13 +1127,13 @@
         <v>6</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H4">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1131,10 +1153,10 @@
         <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H5">
         <v>4.4000000000000004</v>
@@ -1145,10 +1167,10 @@
         <v>105021</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6">
         <v>105008</v>
@@ -1157,10 +1179,10 @@
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H6">
         <v>0.4</v>
@@ -1183,10 +1205,10 @@
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1197,10 +1219,10 @@
         <v>105021</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D8">
         <v>120041</v>
@@ -1209,10 +1231,10 @@
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H8">
         <v>0.1</v>
@@ -1235,13 +1257,13 @@
         <v>1002</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H9">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1249,10 +1271,10 @@
         <v>105021</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D10">
         <v>105021</v>
@@ -1261,13 +1283,13 @@
         <v>20032</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G10" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H10">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-17_1920 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CD9DF07-5E31-4494-A6C6-448C75764BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6562B079-A0DC-4700-B8D3-879C5F9D854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -202,7 +202,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="3RAS MARCAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -576,8 +582,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -638,7 +643,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -664,34 +669,34 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>997168.06</v>
+        <v>1105560.9099999999</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1994336.11</v>
+        <v>1768897.46</v>
       </c>
       <c r="L2">
-        <v>36.26</v>
+        <v>32.159999999999997</v>
       </c>
       <c r="M2">
-        <v>83097.34</v>
+        <v>73704.06</v>
       </c>
       <c r="N2">
-        <v>375236</v>
+        <v>488271.01</v>
       </c>
       <c r="O2">
-        <v>181780.49</v>
+        <v>248916.79</v>
       </c>
       <c r="P2">
-        <v>56232.47</v>
+        <v>443312.03</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -717,34 +722,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>24621648.550000001</v>
+        <v>26367353.600000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49243297.109999999</v>
+        <v>42187765.770000003</v>
       </c>
       <c r="L3">
-        <v>99.48</v>
+        <v>85.23</v>
       </c>
       <c r="M3">
-        <v>2051804.05</v>
+        <v>1757823.57</v>
       </c>
       <c r="N3">
-        <v>2073195.95</v>
+        <v>2570294.04</v>
       </c>
       <c r="O3">
-        <v>1478135.97</v>
+        <v>515487.3</v>
       </c>
       <c r="P3">
-        <v>1062370.01</v>
+        <v>6833382.5700000003</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -770,34 +775,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>30014653.960000001</v>
+        <v>47807374.369999997</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>60029307.93</v>
+        <v>76491798.989999995</v>
       </c>
       <c r="L4">
-        <v>53.24</v>
+        <v>67.84</v>
       </c>
       <c r="M4">
-        <v>2501221.16</v>
+        <v>3187158.29</v>
       </c>
       <c r="N4">
-        <v>6894612.1699999999</v>
+        <v>7215847.29</v>
       </c>
       <c r="O4">
-        <v>1349226.17</v>
+        <v>826852.52</v>
       </c>
       <c r="P4">
-        <v>1746652.89</v>
+        <v>239873.97</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -823,34 +828,34 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>4032981.96</v>
+        <v>7278618.2000000002</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>8065963.9100000001</v>
+        <v>11645789.130000001</v>
       </c>
       <c r="L5">
-        <v>58.66</v>
+        <v>84.7</v>
       </c>
       <c r="M5">
-        <v>336081.83</v>
+        <v>485241.21</v>
       </c>
       <c r="N5">
-        <v>809751.5</v>
+        <v>719042.42</v>
       </c>
       <c r="O5">
-        <v>49894.96</v>
+        <v>69592.2</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>80769.37</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -876,34 +881,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>2339364.5499999998</v>
+        <v>5105171.08</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4678729.0999999996</v>
+        <v>8168273.7300000004</v>
       </c>
       <c r="L6">
-        <v>14.18</v>
+        <v>24.75</v>
       </c>
       <c r="M6">
-        <v>194947.05</v>
+        <v>340344.74</v>
       </c>
       <c r="N6">
-        <v>2555052.9500000002</v>
+        <v>3099425.44</v>
       </c>
       <c r="O6">
-        <v>-16753.03</v>
+        <v>266803.53999999998</v>
       </c>
       <c r="P6">
-        <v>29231.45</v>
+        <v>240862.15</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -929,34 +934,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>61999016.68</v>
+        <v>65440131.57</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>123998033.36</v>
+        <v>104704210.5</v>
       </c>
       <c r="L7">
-        <v>173.42</v>
+        <v>146.44</v>
       </c>
       <c r="M7">
-        <v>5166584.72</v>
+        <v>4362675.4400000004</v>
       </c>
       <c r="N7">
-        <v>791748.61</v>
+        <v>673318.71</v>
       </c>
       <c r="O7">
-        <v>909784.94</v>
+        <v>645612.92000000004</v>
       </c>
       <c r="P7">
-        <v>973398.85</v>
+        <v>357851.28</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -982,28 +987,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>13694839.91</v>
+        <v>14832225.76</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>27389679.829999998</v>
+        <v>23731561.219999999</v>
       </c>
       <c r="L8">
-        <v>62.25</v>
+        <v>53.94</v>
       </c>
       <c r="M8">
-        <v>1141236.6599999999</v>
+        <v>988815.05</v>
       </c>
       <c r="N8">
-        <v>2525430.0099999998</v>
+        <v>3240863.8</v>
       </c>
       <c r="O8">
-        <v>1133722.54</v>
+        <v>87450.1</v>
       </c>
       <c r="P8">
-        <v>550253.22</v>
+        <v>266540.59999999998</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1081,7 +1086,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1107,7 +1112,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1133,7 +1138,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1159,7 +1164,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>4.4000000000000004</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1185,7 +1190,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1211,7 +1216,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-06-18_1821 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6562B079-A0DC-4700-B8D3-879C5F9D854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2498C7A-729C-4847-8360-C0E79927320C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -202,13 +202,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="3RAS MARCAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -582,7 +576,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -643,7 +638,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -669,34 +664,34 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>1105560.9099999999</v>
+        <v>1569483.21</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1768897.46</v>
+        <v>2511173.13</v>
       </c>
       <c r="L2">
-        <v>32.159999999999997</v>
+        <v>45.66</v>
       </c>
       <c r="M2">
-        <v>73704.06</v>
+        <v>104632.21</v>
       </c>
       <c r="N2">
-        <v>488271.01</v>
+        <v>436724.09</v>
       </c>
       <c r="O2">
-        <v>248916.79</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>443312.03</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -722,34 +717,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>26367353.600000001</v>
+        <v>27754115.84</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>42187765.770000003</v>
+        <v>44406585.350000001</v>
       </c>
       <c r="L3">
-        <v>85.23</v>
+        <v>89.71</v>
       </c>
       <c r="M3">
-        <v>1757823.57</v>
+        <v>1850274.39</v>
       </c>
       <c r="N3">
-        <v>2570294.04</v>
+        <v>2416209.35</v>
       </c>
       <c r="O3">
-        <v>515487.3</v>
+        <v>1553490.07</v>
       </c>
       <c r="P3">
-        <v>6833382.5700000003</v>
+        <v>8484253.4100000001</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -775,34 +770,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>47807374.369999997</v>
+        <v>50664146.329999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>76491798.989999995</v>
+        <v>81062634.129999995</v>
       </c>
       <c r="L4">
-        <v>67.84</v>
+        <v>71.900000000000006</v>
       </c>
       <c r="M4">
-        <v>3187158.29</v>
+        <v>3377609.76</v>
       </c>
       <c r="N4">
-        <v>7215847.29</v>
+        <v>6898428.1900000004</v>
       </c>
       <c r="O4">
-        <v>826852.52</v>
+        <v>2966694.99</v>
       </c>
       <c r="P4">
-        <v>239873.97</v>
+        <v>167814.97</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -828,34 +823,34 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>7278618.2000000002</v>
+        <v>8238024.1799999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>11645789.130000001</v>
+        <v>13180838.689999999</v>
       </c>
       <c r="L5">
-        <v>84.7</v>
+        <v>95.86</v>
       </c>
       <c r="M5">
-        <v>485241.21</v>
+        <v>549201.61</v>
       </c>
       <c r="N5">
-        <v>719042.42</v>
+        <v>612441.76</v>
       </c>
       <c r="O5">
-        <v>69592.2</v>
+        <v>2742829.96</v>
       </c>
       <c r="P5">
-        <v>80769.37</v>
+        <v>93891.42</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -881,34 +876,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>5105171.08</v>
+        <v>6719893.1699999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>8168273.7300000004</v>
+        <v>10751829.07</v>
       </c>
       <c r="L6">
-        <v>24.75</v>
+        <v>32.58</v>
       </c>
       <c r="M6">
-        <v>340344.74</v>
+        <v>447992.88</v>
       </c>
       <c r="N6">
-        <v>3099425.44</v>
+        <v>2920011.87</v>
       </c>
       <c r="O6">
-        <v>266803.53999999998</v>
+        <v>509931.64</v>
       </c>
       <c r="P6">
-        <v>240862.15</v>
+        <v>143378.76999999999</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -934,34 +929,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>65440131.57</v>
+        <v>66908522.030000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>104704210.5</v>
+        <v>107053635.23999999</v>
       </c>
       <c r="L7">
-        <v>146.44</v>
+        <v>149.72999999999999</v>
       </c>
       <c r="M7">
-        <v>4362675.4400000004</v>
+        <v>4460568.1399999997</v>
       </c>
       <c r="N7">
-        <v>673318.71</v>
+        <v>510164.22</v>
       </c>
       <c r="O7">
-        <v>645612.92000000004</v>
+        <v>14998906.83</v>
       </c>
       <c r="P7">
-        <v>357851.28</v>
+        <v>1483064.19</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -987,28 +982,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>14832225.76</v>
+        <v>15989716.09</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23731561.219999999</v>
+        <v>25583545.739999998</v>
       </c>
       <c r="L8">
-        <v>53.94</v>
+        <v>58.14</v>
       </c>
       <c r="M8">
-        <v>988815.05</v>
+        <v>1065981.07</v>
       </c>
       <c r="N8">
-        <v>3240863.8</v>
+        <v>3112253.77</v>
       </c>
       <c r="O8">
-        <v>87450.1</v>
+        <v>4073100.93</v>
       </c>
       <c r="P8">
-        <v>266540.59999999998</v>
+        <v>611056</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1086,7 +1081,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1112,7 +1107,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1138,7 +1133,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1164,7 +1159,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1190,7 +1185,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1268,7 +1263,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1294,7 +1289,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-19_1755 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2498C7A-729C-4847-8360-C0E79927320C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B4FCE03-FF62-48C2-B6BF-135024128A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -180,9 +180,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -229,9 +228,6 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
   <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H10">
-    <sortCondition ref="E2:E10"/>
-  </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
@@ -670,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2511173.13</v>
+        <v>2354224.81</v>
       </c>
       <c r="L2">
-        <v>45.66</v>
+        <v>42.8</v>
       </c>
       <c r="M2">
-        <v>104632.21</v>
+        <v>98092.7</v>
       </c>
       <c r="N2">
-        <v>436724.09</v>
+        <v>491314.6</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>76985.73</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -717,28 +713,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>27754115.84</v>
+        <v>34931212.009999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>44406585.350000001</v>
+        <v>52396818.009999998</v>
       </c>
       <c r="L3">
-        <v>89.71</v>
+        <v>105.85</v>
       </c>
       <c r="M3">
-        <v>1850274.39</v>
+        <v>2183200.75</v>
       </c>
       <c r="N3">
-        <v>2416209.35</v>
+        <v>1821098.5</v>
       </c>
       <c r="O3">
-        <v>1553490.07</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>8484253.4100000001</v>
+        <v>577146.23</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -770,28 +766,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>50664146.329999998</v>
+        <v>50971730.810000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>81062634.129999995</v>
+        <v>76457596.209999993</v>
       </c>
       <c r="L4">
-        <v>71.900000000000006</v>
+        <v>67.81</v>
       </c>
       <c r="M4">
-        <v>3377609.76</v>
+        <v>3185733.18</v>
       </c>
       <c r="N4">
-        <v>6898428.1900000004</v>
+        <v>7722283.6500000004</v>
       </c>
       <c r="O4">
-        <v>2966694.99</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>167814.97</v>
+        <v>11007267.83</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -823,28 +819,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8238024.1799999997</v>
+        <v>7949496.5300000003</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>13180838.689999999</v>
+        <v>11924244.800000001</v>
       </c>
       <c r="L5">
-        <v>95.86</v>
+        <v>86.72</v>
       </c>
       <c r="M5">
-        <v>549201.61</v>
+        <v>496843.53</v>
       </c>
       <c r="N5">
-        <v>612441.76</v>
+        <v>725062.93</v>
       </c>
       <c r="O5">
-        <v>2742829.96</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>93891.42</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -876,28 +872,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>6719893.1699999999</v>
+        <v>6860294.9699999997</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10751829.07</v>
+        <v>10290442.460000001</v>
       </c>
       <c r="L6">
-        <v>32.58</v>
+        <v>31.18</v>
       </c>
       <c r="M6">
-        <v>447992.88</v>
+        <v>428768.44</v>
       </c>
       <c r="N6">
-        <v>2920011.87</v>
+        <v>3267463.13</v>
       </c>
       <c r="O6">
-        <v>509931.64</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>143378.76999999999</v>
+        <v>122226.03</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -929,28 +925,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>66908522.030000001</v>
+        <v>67728055.019999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>107053635.23999999</v>
+        <v>101592082.52</v>
       </c>
       <c r="L7">
-        <v>149.72999999999999</v>
+        <v>142.09</v>
       </c>
       <c r="M7">
-        <v>4460568.1399999997</v>
+        <v>4233003.4400000004</v>
       </c>
       <c r="N7">
-        <v>510164.22</v>
+        <v>471493.12</v>
       </c>
       <c r="O7">
-        <v>14998906.83</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>1483064.19</v>
+        <v>1351636.62</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -982,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>15989716.09</v>
+        <v>17102345.98</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>25583545.739999998</v>
+        <v>25653518.969999999</v>
       </c>
       <c r="L8">
-        <v>58.14</v>
+        <v>58.3</v>
       </c>
       <c r="M8">
-        <v>1065981.07</v>
+        <v>1068896.6200000001</v>
       </c>
       <c r="N8">
-        <v>3112253.77</v>
+        <v>3362206.75</v>
       </c>
       <c r="O8">
-        <v>4073100.93</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>611056</v>
+        <v>938418.24</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1069,19 +1065,19 @@
         <v>26</v>
       </c>
       <c r="D2">
-        <v>105003</v>
-      </c>
-      <c r="E2" s="1">
-        <v>3</v>
+        <v>105006</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
         <v>40</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1097,8 +1093,8 @@
       <c r="D3">
         <v>105004</v>
       </c>
-      <c r="E3" s="1">
-        <v>4</v>
+      <c r="E3" t="s">
+        <v>31</v>
       </c>
       <c r="F3" t="s">
         <v>32</v>
@@ -1107,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1121,19 +1117,19 @@
         <v>26</v>
       </c>
       <c r="D4">
-        <v>105006</v>
-      </c>
-      <c r="E4" s="1">
-        <v>6</v>
+        <v>105003</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1147,71 +1143,71 @@
         <v>18</v>
       </c>
       <c r="D5">
-        <v>105007</v>
-      </c>
-      <c r="E5" s="1">
-        <v>7</v>
+        <v>120039</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
         <v>40</v>
       </c>
       <c r="H5">
-        <v>2.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>105021</v>
+        <v>106002</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D6">
-        <v>105008</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8</v>
+        <v>105007</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>106002</v>
+        <v>105021</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D7">
-        <v>120039</v>
-      </c>
-      <c r="E7" s="1">
-        <v>9</v>
+        <v>105008</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G7" t="s">
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1227,8 +1223,8 @@
       <c r="D8">
         <v>120041</v>
       </c>
-      <c r="E8" s="1">
-        <v>10</v>
+      <c r="E8" t="s">
+        <v>33</v>
       </c>
       <c r="F8" t="s">
         <v>34</v>
@@ -1242,19 +1238,19 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>106002</v>
+        <v>105021</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D9">
-        <v>106002</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1002</v>
+        <v>105021</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
       </c>
       <c r="F9" t="s">
         <v>41</v>
@@ -1263,24 +1259,24 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>105021</v>
+        <v>106002</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D10">
-        <v>105021</v>
-      </c>
-      <c r="E10" s="1">
-        <v>20032</v>
+        <v>106002</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
       </c>
       <c r="F10" t="s">
         <v>41</v>
@@ -1289,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-22_2146 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B4FCE03-FF62-48C2-B6BF-135024128A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D55AB030-0662-4CB0-AFF8-3FAC01282ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -660,28 +660,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>1569483.21</v>
+        <v>1956769.31</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2354224.81</v>
+        <v>2762497.85</v>
       </c>
       <c r="L2">
-        <v>42.8</v>
+        <v>50.23</v>
       </c>
       <c r="M2">
-        <v>98092.7</v>
+        <v>115104.08</v>
       </c>
       <c r="N2">
-        <v>491314.6</v>
+        <v>506175.81</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>108392.86</v>
       </c>
       <c r="P2">
-        <v>76985.73</v>
+        <v>181780.49</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>34931212.009999998</v>
+        <v>35168131.439999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>52396818.009999998</v>
+        <v>49649126.740000002</v>
       </c>
       <c r="L3">
-        <v>105.85</v>
+        <v>100.3</v>
       </c>
       <c r="M3">
-        <v>2183200.75</v>
+        <v>2068713.61</v>
       </c>
       <c r="N3">
-        <v>1821098.5</v>
+        <v>2047409.79</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>1312976.44</v>
       </c>
       <c r="P3">
-        <v>577146.23</v>
+        <v>1478135.97</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>50971730.810000002</v>
+        <v>85663656.390000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>76457596.209999993</v>
+        <v>120936926.67</v>
       </c>
       <c r="L4">
-        <v>67.81</v>
+        <v>107.26</v>
       </c>
       <c r="M4">
-        <v>3185733.18</v>
+        <v>5039038.6100000003</v>
       </c>
       <c r="N4">
-        <v>7722283.6500000004</v>
+        <v>3869477.66</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>4789775.1500000004</v>
       </c>
       <c r="P4">
-        <v>11007267.83</v>
+        <v>1349226.17</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>11924244.800000001</v>
+        <v>11222818.640000001</v>
       </c>
       <c r="L5">
-        <v>86.72</v>
+        <v>81.62</v>
       </c>
       <c r="M5">
-        <v>496843.53</v>
+        <v>467617.44</v>
       </c>
       <c r="N5">
-        <v>725062.93</v>
+        <v>828643.35</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>110832.37</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>49894.96</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>6860294.9699999997</v>
+        <v>6920920.1100000003</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10290442.460000001</v>
+        <v>9770710.75</v>
       </c>
       <c r="L6">
-        <v>31.18</v>
+        <v>29.61</v>
       </c>
       <c r="M6">
-        <v>428768.44</v>
+        <v>407112.95</v>
       </c>
       <c r="N6">
-        <v>3267463.13</v>
+        <v>3725582.84</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>106672.2</v>
       </c>
       <c r="P6">
-        <v>122226.03</v>
+        <v>-16753.03</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>67728055.019999996</v>
+        <v>68096092.040000007</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>101592082.52</v>
+        <v>96135659.349999994</v>
       </c>
       <c r="L7">
-        <v>142.09</v>
+        <v>134.46</v>
       </c>
       <c r="M7">
-        <v>4233003.4400000004</v>
+        <v>4005652.47</v>
       </c>
       <c r="N7">
-        <v>471493.12</v>
+        <v>486272.57</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>2037778.17</v>
       </c>
       <c r="P7">
-        <v>1351636.62</v>
+        <v>909784.94</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>17102345.98</v>
+        <v>27499975.620000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>25653518.969999999</v>
+        <v>38823494.990000002</v>
       </c>
       <c r="L8">
-        <v>58.3</v>
+        <v>88.24</v>
       </c>
       <c r="M8">
-        <v>1068896.6200000001</v>
+        <v>1617645.62</v>
       </c>
       <c r="N8">
-        <v>3362206.75</v>
+        <v>2357146.34</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>771647.87</v>
       </c>
       <c r="P8">
-        <v>938418.24</v>
+        <v>1133722.54</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>2.8</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-06-23_1750 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D55AB030-0662-4CB0-AFF8-3FAC01282ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E88F3319-66BE-4EC8-992C-07E241BCAF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>1956769.31</v>
+        <v>4816008.28</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2762497.85</v>
+        <v>6421344.3700000001</v>
       </c>
       <c r="L2">
-        <v>50.23</v>
+        <v>116.75</v>
       </c>
       <c r="M2">
-        <v>115104.08</v>
+        <v>267556.02</v>
       </c>
       <c r="N2">
-        <v>506175.81</v>
+        <v>113998.62</v>
       </c>
       <c r="O2">
-        <v>108392.86</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>181780.49</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>35168131.439999998</v>
+        <v>39680979.659999996</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49649126.740000002</v>
+        <v>52907972.880000003</v>
       </c>
       <c r="L3">
-        <v>100.3</v>
+        <v>106.88</v>
       </c>
       <c r="M3">
-        <v>2068713.61</v>
+        <v>2204498.87</v>
       </c>
       <c r="N3">
-        <v>2047409.79</v>
+        <v>1636503.39</v>
       </c>
       <c r="O3">
-        <v>1312976.44</v>
+        <v>458635.6</v>
       </c>
       <c r="P3">
-        <v>1478135.97</v>
+        <v>1261967.8700000001</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>85663656.390000001</v>
+        <v>87753530.129999995</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>120936926.67</v>
+        <v>117004706.83</v>
       </c>
       <c r="L4">
-        <v>107.26</v>
+        <v>103.77</v>
       </c>
       <c r="M4">
-        <v>5039038.6100000003</v>
+        <v>4875196.12</v>
       </c>
       <c r="N4">
-        <v>3869477.66</v>
+        <v>4166078.31</v>
       </c>
       <c r="O4">
-        <v>4789775.1500000004</v>
+        <v>11977439.109999999</v>
       </c>
       <c r="P4">
-        <v>1349226.17</v>
+        <v>1696338.53</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>7949496.5300000003</v>
+        <v>8005356.8899999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>11222818.640000001</v>
+        <v>10673809.189999999</v>
       </c>
       <c r="L5">
-        <v>81.62</v>
+        <v>77.63</v>
       </c>
       <c r="M5">
-        <v>467617.44</v>
+        <v>444742.05</v>
       </c>
       <c r="N5">
-        <v>828643.35</v>
+        <v>957440.52</v>
       </c>
       <c r="O5">
-        <v>110832.37</v>
+        <v>3134803.88</v>
       </c>
       <c r="P5">
-        <v>49894.96</v>
+        <v>280375.73</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>6920920.1100000003</v>
+        <v>6987356.6799999997</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>9770710.75</v>
+        <v>9316475.5700000003</v>
       </c>
       <c r="L6">
-        <v>29.61</v>
+        <v>28.23</v>
       </c>
       <c r="M6">
-        <v>407112.95</v>
+        <v>388186.48</v>
       </c>
       <c r="N6">
-        <v>3725582.84</v>
+        <v>4335440.55</v>
       </c>
       <c r="O6">
-        <v>106672.2</v>
+        <v>2659134.33</v>
       </c>
       <c r="P6">
-        <v>-16753.03</v>
+        <v>321235.42</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>68096092.040000007</v>
+        <v>69287776.560000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>96135659.349999994</v>
+        <v>92383702.079999998</v>
       </c>
       <c r="L7">
-        <v>134.46</v>
+        <v>129.21</v>
       </c>
       <c r="M7">
-        <v>4005652.47</v>
+        <v>3849320.92</v>
       </c>
       <c r="N7">
-        <v>486272.57</v>
+        <v>368703.91</v>
       </c>
       <c r="O7">
-        <v>2037778.17</v>
+        <v>1403336.71</v>
       </c>
       <c r="P7">
-        <v>909784.94</v>
+        <v>189879.89</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>27499975.620000001</v>
+        <v>28804435.370000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>38823494.990000002</v>
+        <v>38405913.82</v>
       </c>
       <c r="L8">
-        <v>88.24</v>
+        <v>87.29</v>
       </c>
       <c r="M8">
-        <v>1617645.62</v>
+        <v>1600246.41</v>
       </c>
       <c r="N8">
-        <v>2357146.34</v>
+        <v>2532594.11</v>
       </c>
       <c r="O8">
-        <v>771647.87</v>
+        <v>365737.98</v>
       </c>
       <c r="P8">
-        <v>1133722.54</v>
+        <v>604894.67000000004</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>2.2000000000000002</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-24_1811 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E88F3319-66BE-4EC8-992C-07E241BCAF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13BB7B4-2CCB-4DC8-9A48-066170C656ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>4816008.28</v>
+        <v>4634242.46</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6421344.3700000001</v>
+        <v>5853779.9500000002</v>
       </c>
       <c r="L2">
-        <v>116.75</v>
+        <v>106.43</v>
       </c>
       <c r="M2">
-        <v>267556.02</v>
+        <v>243907.5</v>
       </c>
       <c r="N2">
-        <v>113998.62</v>
+        <v>173151.51</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>463922.29</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>248916.79</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>39680979.659999996</v>
+        <v>40365298.689999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>52907972.880000003</v>
+        <v>50987745.710000001</v>
       </c>
       <c r="L3">
-        <v>106.88</v>
+        <v>103.01</v>
       </c>
       <c r="M3">
-        <v>2204498.87</v>
+        <v>2124489.4</v>
       </c>
       <c r="N3">
-        <v>1636503.39</v>
+        <v>1826940.26</v>
       </c>
       <c r="O3">
-        <v>458635.6</v>
+        <v>1386762.24</v>
       </c>
       <c r="P3">
-        <v>1261967.8700000001</v>
+        <v>515487.3</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>87753530.129999995</v>
+        <v>89451553.670000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>117004706.83</v>
+        <v>112991436.20999999</v>
       </c>
       <c r="L4">
-        <v>103.77</v>
+        <v>100.21</v>
       </c>
       <c r="M4">
-        <v>4875196.12</v>
+        <v>4707976.51</v>
       </c>
       <c r="N4">
-        <v>4166078.31</v>
+        <v>4659689.2699999996</v>
       </c>
       <c r="O4">
-        <v>11977439.109999999</v>
+        <v>2590776.62</v>
       </c>
       <c r="P4">
-        <v>1696338.53</v>
+        <v>826852.52</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8005356.8899999997</v>
+        <v>8193379.2699999996</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10673809.189999999</v>
+        <v>10349531.710000001</v>
       </c>
       <c r="L5">
-        <v>77.63</v>
+        <v>75.27</v>
       </c>
       <c r="M5">
-        <v>444742.05</v>
+        <v>431230.49</v>
       </c>
       <c r="N5">
-        <v>957440.52</v>
+        <v>1111324.1499999999</v>
       </c>
       <c r="O5">
-        <v>3134803.88</v>
+        <v>959405.98</v>
       </c>
       <c r="P5">
-        <v>280375.73</v>
+        <v>69592.2</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>6987356.6799999997</v>
+        <v>7250226.0999999996</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>9316475.5700000003</v>
+        <v>9158180.3300000001</v>
       </c>
       <c r="L6">
-        <v>28.23</v>
+        <v>27.75</v>
       </c>
       <c r="M6">
-        <v>388186.48</v>
+        <v>381590.85</v>
       </c>
       <c r="N6">
-        <v>4335440.55</v>
+        <v>5149954.78</v>
       </c>
       <c r="O6">
-        <v>2659134.33</v>
+        <v>1570106.04</v>
       </c>
       <c r="P6">
-        <v>321235.42</v>
+        <v>266803.53999999998</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>69287776.560000002</v>
+        <v>69496839.090000004</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>92383702.079999998</v>
+        <v>87785480.959999993</v>
       </c>
       <c r="L7">
-        <v>129.21</v>
+        <v>122.78</v>
       </c>
       <c r="M7">
-        <v>3849320.92</v>
+        <v>3657728.37</v>
       </c>
       <c r="N7">
-        <v>368703.91</v>
+        <v>400632.18</v>
       </c>
       <c r="O7">
-        <v>1403336.71</v>
+        <v>1468390.46</v>
       </c>
       <c r="P7">
-        <v>189879.89</v>
+        <v>645612.92000000004</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>28804435.370000001</v>
+        <v>29054848.739999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>38405913.82</v>
+        <v>36700861.57</v>
       </c>
       <c r="L8">
-        <v>87.29</v>
+        <v>83.41</v>
       </c>
       <c r="M8">
-        <v>1600246.41</v>
+        <v>1529202.57</v>
       </c>
       <c r="N8">
-        <v>2532594.11</v>
+        <v>2989030.25</v>
       </c>
       <c r="O8">
-        <v>365737.98</v>
+        <v>1157490.33</v>
       </c>
       <c r="P8">
-        <v>604894.67000000004</v>
+        <v>87450.1</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0.9</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-25_2018 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13BB7B4-2CCB-4DC8-9A48-066170C656ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCBEBF91-9F0F-4B56-B1B9-102A30D79A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,7 +201,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="3RAS MARCAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -634,7 +640,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -660,34 +666,34 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>4634242.46</v>
+        <v>4704769.63</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5853779.9500000002</v>
+        <v>5645723.5499999998</v>
       </c>
       <c r="L2">
-        <v>106.43</v>
+        <v>102.65</v>
       </c>
       <c r="M2">
-        <v>243907.5</v>
+        <v>235238.48</v>
       </c>
       <c r="N2">
-        <v>173151.51</v>
+        <v>198807.59</v>
       </c>
       <c r="O2">
-        <v>463922.29</v>
+        <v>190558.71</v>
       </c>
       <c r="P2">
-        <v>248916.79</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -713,34 +719,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>40365298.689999998</v>
+        <v>40897045.609999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>50987745.710000001</v>
+        <v>49076454.729999997</v>
       </c>
       <c r="L3">
-        <v>103.01</v>
+        <v>99.14</v>
       </c>
       <c r="M3">
-        <v>2124489.4</v>
+        <v>2044852.28</v>
       </c>
       <c r="N3">
-        <v>1826940.26</v>
+        <v>2150738.6</v>
       </c>
       <c r="O3">
-        <v>1386762.24</v>
+        <v>7177096.1600000001</v>
       </c>
       <c r="P3">
-        <v>515487.3</v>
+        <v>1553490.07</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -766,34 +772,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>89451553.670000002</v>
+        <v>91190998.180000007</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>112991436.20999999</v>
+        <v>109429197.81</v>
       </c>
       <c r="L4">
-        <v>100.21</v>
+        <v>97.05</v>
       </c>
       <c r="M4">
-        <v>4707976.51</v>
+        <v>4559549.91</v>
       </c>
       <c r="N4">
-        <v>4659689.2699999996</v>
+        <v>5389750.46</v>
       </c>
       <c r="O4">
-        <v>2590776.62</v>
+        <v>307584.48</v>
       </c>
       <c r="P4">
-        <v>826852.52</v>
+        <v>2966694.99</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -819,34 +825,34 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8193379.2699999996</v>
+        <v>8299809.6799999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10349531.710000001</v>
+        <v>9959771.6199999992</v>
       </c>
       <c r="L5">
-        <v>75.27</v>
+        <v>72.430000000000007</v>
       </c>
       <c r="M5">
-        <v>431230.49</v>
+        <v>414990.48</v>
       </c>
       <c r="N5">
-        <v>1111324.1499999999</v>
+        <v>1362547.58</v>
       </c>
       <c r="O5">
-        <v>959405.98</v>
+        <v>-288527.65000000002</v>
       </c>
       <c r="P5">
-        <v>69592.2</v>
+        <v>2742829.96</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -872,34 +878,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>7250226.0999999996</v>
+        <v>7581511.1600000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>9158180.3300000001</v>
+        <v>9097813.3900000006</v>
       </c>
       <c r="L6">
-        <v>27.75</v>
+        <v>27.57</v>
       </c>
       <c r="M6">
-        <v>381590.85</v>
+        <v>379075.56</v>
       </c>
       <c r="N6">
-        <v>5149954.78</v>
+        <v>6354622.21</v>
       </c>
       <c r="O6">
-        <v>1570106.04</v>
+        <v>185017.85</v>
       </c>
       <c r="P6">
-        <v>266803.53999999998</v>
+        <v>509931.64</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -925,34 +931,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>69496839.090000004</v>
+        <v>72850468.349999994</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>87785480.959999993</v>
+        <v>87420562.019999996</v>
       </c>
       <c r="L7">
-        <v>122.78</v>
+        <v>122.27</v>
       </c>
       <c r="M7">
-        <v>3657728.37</v>
+        <v>3642523.42</v>
       </c>
       <c r="N7">
-        <v>400632.18</v>
+        <v>-337617.09</v>
       </c>
       <c r="O7">
-        <v>1468390.46</v>
+        <v>819532.99</v>
       </c>
       <c r="P7">
-        <v>645612.92000000004</v>
+        <v>14998906.83</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -978,28 +984,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>29054848.739999998</v>
+        <v>30897610.5</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36700861.57</v>
+        <v>37077132.600000001</v>
       </c>
       <c r="L8">
-        <v>83.41</v>
+        <v>84.27</v>
       </c>
       <c r="M8">
-        <v>1529202.57</v>
+        <v>1544880.52</v>
       </c>
       <c r="N8">
-        <v>2989030.25</v>
+        <v>3275597.38</v>
       </c>
       <c r="O8">
-        <v>1157490.33</v>
+        <v>1112629.8899999999</v>
       </c>
       <c r="P8">
-        <v>87450.1</v>
+        <v>4073100.93</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1109,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1135,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1187,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.9000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1239,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-06-26_1718 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCBEBF91-9F0F-4B56-B1B9-102A30D79A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5649B3B8-2DC0-4274-A1C7-51F1C672A900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,13 +201,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="3RAS MARCAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -640,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -672,19 +666,19 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5645723.5499999998</v>
+        <v>5376879.5700000003</v>
       </c>
       <c r="L2">
-        <v>102.65</v>
+        <v>97.76</v>
       </c>
       <c r="M2">
-        <v>235238.48</v>
+        <v>224036.65</v>
       </c>
       <c r="N2">
-        <v>198807.59</v>
+        <v>265076.78999999998</v>
       </c>
       <c r="O2">
-        <v>190558.71</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -693,7 +687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -719,34 +713,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>40897045.609999999</v>
+        <v>40724749.109999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49076454.729999997</v>
+        <v>46542570.409999996</v>
       </c>
       <c r="L3">
-        <v>99.14</v>
+        <v>94.03</v>
       </c>
       <c r="M3">
-        <v>2044852.28</v>
+        <v>1939273.77</v>
       </c>
       <c r="N3">
-        <v>2150738.6</v>
+        <v>2925083.63</v>
       </c>
       <c r="O3">
-        <v>7177096.1600000001</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>1553490.07</v>
+        <v>313702.81</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -772,34 +766,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>91190998.180000007</v>
+        <v>94553391.959999993</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>109429197.81</v>
+        <v>108061019.39</v>
       </c>
       <c r="L4">
-        <v>97.05</v>
+        <v>95.84</v>
       </c>
       <c r="M4">
-        <v>4559549.91</v>
+        <v>4502542.47</v>
       </c>
       <c r="N4">
-        <v>5389750.46</v>
+        <v>6065536.0099999998</v>
       </c>
       <c r="O4">
-        <v>307584.48</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>2966694.99</v>
+        <v>6261847.5599999996</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -831,28 +825,28 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>9959771.6199999992</v>
+        <v>9485496.7799999993</v>
       </c>
       <c r="L5">
-        <v>72.430000000000007</v>
+        <v>68.989999999999995</v>
       </c>
       <c r="M5">
-        <v>414990.48</v>
+        <v>395229.03</v>
       </c>
       <c r="N5">
-        <v>1362547.58</v>
+        <v>1816730.11</v>
       </c>
       <c r="O5">
-        <v>-288527.65000000002</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>2742829.96</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -878,34 +872,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>7581511.1600000001</v>
+        <v>55757054.780000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>9097813.3900000006</v>
+        <v>63722348.329999998</v>
       </c>
       <c r="L6">
-        <v>27.57</v>
+        <v>193.1</v>
       </c>
       <c r="M6">
-        <v>379075.56</v>
+        <v>2655097.85</v>
       </c>
       <c r="N6">
-        <v>6354622.21</v>
+        <v>-7585684.9299999997</v>
       </c>
       <c r="O6">
-        <v>185017.85</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>509931.64</v>
+        <v>10767.67</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -931,34 +925,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>72850468.349999994</v>
+        <v>73326321.069999993</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>87420562.019999996</v>
+        <v>83801509.799999997</v>
       </c>
       <c r="L7">
-        <v>122.27</v>
+        <v>117.2</v>
       </c>
       <c r="M7">
-        <v>3642523.42</v>
+        <v>3491729.57</v>
       </c>
       <c r="N7">
-        <v>-337617.09</v>
+        <v>-608773.68999999994</v>
       </c>
       <c r="O7">
-        <v>819532.99</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>14998906.83</v>
+        <v>2221976.96</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -984,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>30897610.5</v>
+        <v>32201260.039999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>37077132.600000001</v>
+        <v>36801440.049999997</v>
       </c>
       <c r="L8">
-        <v>84.27</v>
+        <v>83.64</v>
       </c>
       <c r="M8">
-        <v>1544880.52</v>
+        <v>1533393.34</v>
       </c>
       <c r="N8">
-        <v>3275597.38</v>
+        <v>3932913.32</v>
       </c>
       <c r="O8">
-        <v>1112629.8899999999</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>4073100.93</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1083,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1109,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1135,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1161,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1239,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1291,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.4</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-06-28_2355 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5649B3B8-2DC0-4274-A1C7-51F1C672A900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEE84E4C-7B60-47E8-984C-076E59B7DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,7 +201,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="3RAS MARCAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -634,7 +640,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -660,25 +666,25 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>4704769.63</v>
+        <v>4720428.57</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5376879.5700000003</v>
+        <v>5149558.45</v>
       </c>
       <c r="L2">
-        <v>97.76</v>
+        <v>93.63</v>
       </c>
       <c r="M2">
-        <v>224036.65</v>
+        <v>214564.94</v>
       </c>
       <c r="N2">
-        <v>265076.78999999998</v>
+        <v>389785.71</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>196727.4</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -687,7 +693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -713,34 +719,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>40724749.109999999</v>
+        <v>41329730.490000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>46542570.409999996</v>
+        <v>45086978.719999999</v>
       </c>
       <c r="L3">
-        <v>94.03</v>
+        <v>91.08</v>
       </c>
       <c r="M3">
-        <v>1939273.77</v>
+        <v>1878624.11</v>
       </c>
       <c r="N3">
-        <v>2925083.63</v>
+        <v>4085134.75</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>236919.44</v>
       </c>
       <c r="P3">
-        <v>313702.81</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -766,34 +772,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>94553391.959999993</v>
+        <v>94022968.480000004</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>108061019.39</v>
+        <v>102570511.06999999</v>
       </c>
       <c r="L4">
-        <v>95.84</v>
+        <v>90.97</v>
       </c>
       <c r="M4">
-        <v>4502542.47</v>
+        <v>4273771.29</v>
       </c>
       <c r="N4">
-        <v>6065536.0099999998</v>
+        <v>9363515.7599999998</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>34691925.590000004</v>
       </c>
       <c r="P4">
-        <v>6261847.5599999996</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -819,22 +825,22 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8299809.6799999997</v>
+        <v>8321698.1799999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>9485496.7799999993</v>
+        <v>9078216.1899999995</v>
       </c>
       <c r="L5">
-        <v>68.989999999999995</v>
+        <v>66.02</v>
       </c>
       <c r="M5">
-        <v>395229.03</v>
+        <v>378259.01</v>
       </c>
       <c r="N5">
-        <v>1816730.11</v>
+        <v>2714150.91</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -846,7 +852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -872,34 +878,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>55757054.780000001</v>
+        <v>58684199</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>63722348.329999998</v>
+        <v>64019126.189999998</v>
       </c>
       <c r="L6">
-        <v>193.1</v>
+        <v>194</v>
       </c>
       <c r="M6">
-        <v>2655097.85</v>
+        <v>2667463.59</v>
       </c>
       <c r="N6">
-        <v>-7585684.9299999997</v>
+        <v>-12842099.5</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>60625.14</v>
       </c>
       <c r="P6">
-        <v>10767.67</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -925,34 +931,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>73326321.069999993</v>
+        <v>76560419.930000007</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>83801509.799999997</v>
+        <v>83520458.099999994</v>
       </c>
       <c r="L7">
-        <v>117.2</v>
+        <v>116.81</v>
       </c>
       <c r="M7">
-        <v>3491729.57</v>
+        <v>3480019.09</v>
       </c>
       <c r="N7">
-        <v>-608773.68999999994</v>
+        <v>-2530209.96</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>368037.02</v>
       </c>
       <c r="P7">
-        <v>2221976.96</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -978,25 +984,25 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>32201260.039999999</v>
+        <v>58562816.280000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36801440.049999997</v>
+        <v>63886708.659999996</v>
       </c>
       <c r="L8">
-        <v>83.64</v>
+        <v>145.19999999999999</v>
       </c>
       <c r="M8">
-        <v>1533393.34</v>
+        <v>2661946.19</v>
       </c>
       <c r="N8">
-        <v>3932913.32</v>
+        <v>-7281408.1399999997</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>10360021.949999999</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1077,7 +1083,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1109,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1135,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1161,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1187,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1213,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1239,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1265,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-06-29_1903 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BEE84E4C-7B60-47E8-984C-076E59B7DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51B8F765-79CD-4C72-BF4A-399ECC361680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,13 +201,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="3RAS MARCAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -640,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -666,34 +660,34 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>4720428.57</v>
+        <v>4855376.1500000004</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5149558.45</v>
+        <v>5066479.46</v>
       </c>
       <c r="L2">
-        <v>93.63</v>
+        <v>92.12</v>
       </c>
       <c r="M2">
-        <v>214564.94</v>
+        <v>211103.31</v>
       </c>
       <c r="N2">
-        <v>389785.71</v>
+        <v>644623.85</v>
       </c>
       <c r="O2">
-        <v>196727.4</v>
+        <v>2859238.97</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>108392.86</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -719,34 +713,34 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>41329730.490000002</v>
+        <v>41460307.119999997</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>45086978.719999999</v>
+        <v>43262929.170000002</v>
       </c>
       <c r="L3">
-        <v>91.08</v>
+        <v>87.4</v>
       </c>
       <c r="M3">
-        <v>1878624.11</v>
+        <v>1802622.05</v>
       </c>
       <c r="N3">
-        <v>4085134.75</v>
+        <v>8039692.8799999999</v>
       </c>
       <c r="O3">
-        <v>236919.44</v>
+        <v>4473126.68</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>1312976.44</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -772,34 +766,34 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>94022968.480000004</v>
+        <v>97158174.790000007</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>102570511.06999999</v>
+        <v>101382443.26000001</v>
       </c>
       <c r="L4">
-        <v>90.97</v>
+        <v>89.92</v>
       </c>
       <c r="M4">
-        <v>4273771.29</v>
+        <v>4224268.47</v>
       </c>
       <c r="N4">
-        <v>9363515.7599999998</v>
+        <v>15591825.210000001</v>
       </c>
       <c r="O4">
-        <v>34691925.590000004</v>
+        <v>2089873.73</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>4789775.1500000004</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -825,34 +819,34 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8321698.1799999997</v>
+        <v>8901170.9700000007</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>9078216.1899999995</v>
+        <v>9288178.4000000004</v>
       </c>
       <c r="L5">
-        <v>66.02</v>
+        <v>67.55</v>
       </c>
       <c r="M5">
-        <v>378259.01</v>
+        <v>387007.43</v>
       </c>
       <c r="N5">
-        <v>2714150.91</v>
+        <v>4848829.03</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>55860.36</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>110832.37</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -878,34 +872,34 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>58684199</v>
+        <v>59653938.920000002</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>64019126.189999998</v>
+        <v>62247588.439999998</v>
       </c>
       <c r="L6">
-        <v>194</v>
+        <v>188.63</v>
       </c>
       <c r="M6">
-        <v>2667463.59</v>
+        <v>2593649.52</v>
       </c>
       <c r="N6">
-        <v>-12842099.5</v>
+        <v>-26653938.920000002</v>
       </c>
       <c r="O6">
-        <v>60625.14</v>
+        <v>66436.56</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>106672.2</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -931,34 +925,34 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>76560419.930000007</v>
+        <v>86270679.760000005</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>83520458.099999994</v>
+        <v>90021578.870000005</v>
       </c>
       <c r="L7">
-        <v>116.81</v>
+        <v>125.9</v>
       </c>
       <c r="M7">
-        <v>3480019.09</v>
+        <v>3750899.12</v>
       </c>
       <c r="N7">
-        <v>-2530209.96</v>
+        <v>-14770679.76</v>
       </c>
       <c r="O7">
-        <v>368037.02</v>
+        <v>1044689.21</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>2037778.17</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -984,28 +978,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>58562816.280000001</v>
+        <v>59306202.450000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>63886708.659999996</v>
+        <v>61884732.990000002</v>
       </c>
       <c r="L8">
-        <v>145.19999999999999</v>
+        <v>140.65</v>
       </c>
       <c r="M8">
-        <v>2661946.19</v>
+        <v>2578530.54</v>
       </c>
       <c r="N8">
-        <v>-7281408.1399999997</v>
+        <v>-15306202.449999999</v>
       </c>
       <c r="O8">
-        <v>10360021.949999999</v>
+        <v>1342067.43</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>771647.87</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1083,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1135,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1187,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.0999999999999996</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-06-30_1746 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51B8F765-79CD-4C72-BF4A-399ECC361680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{36C26F2D-4F6D-49FB-B254-453637C56BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -666,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5066479.46</v>
+        <v>4855376.1500000004</v>
       </c>
       <c r="L2">
-        <v>92.12</v>
+        <v>88.28</v>
       </c>
       <c r="M2">
-        <v>211103.31</v>
+        <v>202307.34</v>
       </c>
       <c r="N2">
-        <v>644623.85</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>2859238.97</v>
+        <v>-181765.82</v>
       </c>
       <c r="P2">
-        <v>108392.86</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>41460307.119999997</v>
+        <v>41996782.25</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>43262929.170000002</v>
+        <v>41996782.25</v>
       </c>
       <c r="L3">
-        <v>87.4</v>
+        <v>84.84</v>
       </c>
       <c r="M3">
-        <v>1802622.05</v>
+        <v>1749865.93</v>
       </c>
       <c r="N3">
-        <v>8039692.8799999999</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>4473126.68</v>
+        <v>702630.97</v>
       </c>
       <c r="P3">
-        <v>1312976.44</v>
+        <v>458635.6</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>97158174.790000007</v>
+        <v>97527180.609999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>101382443.26000001</v>
+        <v>97527180.609999999</v>
       </c>
       <c r="L4">
-        <v>89.92</v>
+        <v>86.5</v>
       </c>
       <c r="M4">
-        <v>4224268.47</v>
+        <v>4063632.53</v>
       </c>
       <c r="N4">
-        <v>15591825.210000001</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>2089873.73</v>
+        <v>1680125.82</v>
       </c>
       <c r="P4">
-        <v>4789775.1500000004</v>
+        <v>11977439.109999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +818,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>8901170.9700000007</v>
+        <v>9416944.7400000002</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>9288178.4000000004</v>
+        <v>9416944.7400000002</v>
       </c>
       <c r="L5">
-        <v>67.55</v>
+        <v>68.489999999999995</v>
       </c>
       <c r="M5">
-        <v>387007.43</v>
+        <v>392372.7</v>
       </c>
       <c r="N5">
-        <v>4848829.03</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>55860.36</v>
+        <v>188022.38</v>
       </c>
       <c r="P5">
-        <v>110832.37</v>
+        <v>3134803.88</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>59653938.920000002</v>
+        <v>59991092.859999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>62247588.439999998</v>
+        <v>59991092.859999999</v>
       </c>
       <c r="L6">
-        <v>188.63</v>
+        <v>181.79</v>
       </c>
       <c r="M6">
-        <v>2593649.52</v>
+        <v>2499628.87</v>
       </c>
       <c r="N6">
-        <v>-26653938.920000002</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>66436.56</v>
+        <v>262869.42</v>
       </c>
       <c r="P6">
-        <v>106672.2</v>
+        <v>2659134.33</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>86270679.760000005</v>
+        <v>86388567.519999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>90021578.870000005</v>
+        <v>86388567.519999996</v>
       </c>
       <c r="L7">
-        <v>125.9</v>
+        <v>120.82</v>
       </c>
       <c r="M7">
-        <v>3750899.12</v>
+        <v>3599523.65</v>
       </c>
       <c r="N7">
-        <v>-14770679.76</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>1044689.21</v>
+        <v>356057.85</v>
       </c>
       <c r="P7">
-        <v>2037778.17</v>
+        <v>1403336.71</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>59306202.450000003</v>
+        <v>69384867.189999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>61884732.990000002</v>
+        <v>69384867.189999998</v>
       </c>
       <c r="L8">
-        <v>140.65</v>
+        <v>157.69</v>
       </c>
       <c r="M8">
-        <v>2578530.54</v>
+        <v>2891036.13</v>
       </c>
       <c r="N8">
-        <v>-15306202.449999999</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>1342067.43</v>
+        <v>1749258.65</v>
       </c>
       <c r="P8">
-        <v>771647.87</v>
+        <v>365737.98</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-03_2300 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3FDA5E3-EE19-49B8-A719-93BD930338DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABD64E2C-D4DA-4D84-B7D2-8EBBE0E2F20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -660,28 +659,28 @@
         <v>5500000</v>
       </c>
       <c r="I2">
-        <v>415894.77</v>
+        <v>865213.22</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5406631.9699999997</v>
+        <v>7498514.5599999996</v>
       </c>
       <c r="L2">
-        <v>98.3</v>
+        <v>136.34</v>
       </c>
       <c r="M2">
-        <v>207947.38</v>
+        <v>288404.40999999997</v>
       </c>
       <c r="N2">
-        <v>211837.72</v>
+        <v>201512.47</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>15658.95</v>
       </c>
       <c r="P2">
-        <v>190558.71</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>49500000</v>
       </c>
       <c r="I3">
-        <v>1382902.71</v>
+        <v>8481334.3399999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>17977735.219999999</v>
+        <v>73504897.609999999</v>
       </c>
       <c r="L3">
-        <v>36.32</v>
+        <v>148.49</v>
       </c>
       <c r="M3">
-        <v>691451.35</v>
+        <v>2827111.45</v>
       </c>
       <c r="N3">
-        <v>2004879.05</v>
+        <v>1783420.25</v>
       </c>
       <c r="O3">
-        <v>-342803.04</v>
+        <v>399557.34</v>
       </c>
       <c r="P3">
-        <v>7177096.1600000001</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>112750000</v>
       </c>
       <c r="I4">
-        <v>3216375.98</v>
+        <v>5705395.5800000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>41812887.700000003</v>
+        <v>49446761.700000003</v>
       </c>
       <c r="L4">
-        <v>37.08</v>
+        <v>43.86</v>
       </c>
       <c r="M4">
-        <v>1608187.99</v>
+        <v>1901798.53</v>
       </c>
       <c r="N4">
-        <v>4563901</v>
+        <v>4654113.24</v>
       </c>
       <c r="O4">
-        <v>2831970.3</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>307584.48</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +818,28 @@
         <v>13750000</v>
       </c>
       <c r="I5">
-        <v>181077.86</v>
+        <v>208785.95</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2354012.14</v>
+        <v>1809478.23</v>
       </c>
       <c r="L5">
-        <v>17.12</v>
+        <v>13.16</v>
       </c>
       <c r="M5">
-        <v>90538.93</v>
+        <v>69595.320000000007</v>
       </c>
       <c r="N5">
-        <v>565371.76</v>
+        <v>588748.43999999994</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>21888.49</v>
       </c>
       <c r="P5">
-        <v>-288527.65000000002</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>33000000</v>
       </c>
       <c r="I6">
-        <v>590451.98</v>
+        <v>768602.43</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>7675875.7800000003</v>
+        <v>6661221.0700000003</v>
       </c>
       <c r="L6">
-        <v>23.26</v>
+        <v>20.190000000000001</v>
       </c>
       <c r="M6">
-        <v>295225.99</v>
+        <v>256200.81</v>
       </c>
       <c r="N6">
-        <v>1350397.83</v>
+        <v>1401365.11</v>
       </c>
       <c r="O6">
-        <v>48035649.380000003</v>
+        <v>3067038.47</v>
       </c>
       <c r="P6">
-        <v>185017.85</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>71500000</v>
       </c>
       <c r="I7">
-        <v>18428591.41</v>
+        <v>18816115.780000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>239571688.33000001</v>
+        <v>163073003.40000001</v>
       </c>
       <c r="L7">
-        <v>335.07</v>
+        <v>228.07</v>
       </c>
       <c r="M7">
-        <v>9214295.7100000009</v>
+        <v>6272038.5899999999</v>
       </c>
       <c r="N7">
-        <v>2211308.69</v>
+        <v>2290603.66</v>
       </c>
       <c r="O7">
-        <v>475852.73</v>
+        <v>3234098.85</v>
       </c>
       <c r="P7">
-        <v>819532.99</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>44000000</v>
       </c>
       <c r="I8">
-        <v>827630.01</v>
+        <v>5649828.7800000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>10759190.09</v>
+        <v>48965182.759999998</v>
       </c>
       <c r="L8">
-        <v>24.45</v>
+        <v>111.28</v>
       </c>
       <c r="M8">
-        <v>413815</v>
+        <v>1883276.26</v>
       </c>
       <c r="N8">
-        <v>1798848.75</v>
+        <v>1667398.75</v>
       </c>
       <c r="O8">
-        <v>1303649.54</v>
+        <v>26361556.239999998</v>
       </c>
       <c r="P8">
-        <v>1112629.8899999999</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1207,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-05_2237 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABD64E2C-D4DA-4D84-B7D2-8EBBE0E2F20F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{993866C5-8199-441C-A20F-59555BE2C280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,7 +201,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="3RAS MARCAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -572,7 +578,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -633,7 +640,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -656,37 +663,37 @@
         <v>22</v>
       </c>
       <c r="H2">
-        <v>5500000</v>
+        <v>9860000</v>
       </c>
       <c r="I2">
-        <v>865213.22</v>
+        <v>891927.95</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>7498514.5599999996</v>
+        <v>5797531.6699999999</v>
       </c>
       <c r="L2">
-        <v>136.34</v>
+        <v>58.8</v>
       </c>
       <c r="M2">
-        <v>288404.40999999997</v>
+        <v>222981.99</v>
       </c>
       <c r="N2">
-        <v>201512.47</v>
+        <v>407639.64</v>
       </c>
       <c r="O2">
-        <v>15658.95</v>
+        <v>134947.57999999999</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>196727.4</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -709,7 +716,7 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>49500000</v>
+        <v>48140000</v>
       </c>
       <c r="I3">
         <v>8481334.3399999999</v>
@@ -718,28 +725,28 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>73504897.609999999</v>
+        <v>55128673.210000001</v>
       </c>
       <c r="L3">
-        <v>148.49</v>
+        <v>114.52</v>
       </c>
       <c r="M3">
-        <v>2827111.45</v>
+        <v>2120333.58</v>
       </c>
       <c r="N3">
-        <v>1783420.25</v>
+        <v>1802666.62</v>
       </c>
       <c r="O3">
-        <v>399557.34</v>
+        <v>315717.89</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>236919.44</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -762,37 +769,37 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>112750000</v>
+        <v>130000000</v>
       </c>
       <c r="I4">
-        <v>5705395.5800000001</v>
+        <v>9264876.1099999994</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>49446761.700000003</v>
+        <v>60221694.700000003</v>
       </c>
       <c r="L4">
-        <v>43.86</v>
+        <v>46.32</v>
       </c>
       <c r="M4">
-        <v>1901798.53</v>
+        <v>2316219.0299999998</v>
       </c>
       <c r="N4">
-        <v>4654113.24</v>
+        <v>5487960.1799999997</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>3155939.81</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>34691925.590000004</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -815,28 +822,28 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>13750000</v>
+        <v>13000000</v>
       </c>
       <c r="I5">
-        <v>208785.95</v>
+        <v>245750.97</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1809478.23</v>
+        <v>1597381.32</v>
       </c>
       <c r="L5">
-        <v>13.16</v>
+        <v>12.29</v>
       </c>
       <c r="M5">
-        <v>69595.320000000007</v>
+        <v>61437.74</v>
       </c>
       <c r="N5">
-        <v>588748.43999999994</v>
+        <v>579738.59</v>
       </c>
       <c r="O5">
-        <v>21888.49</v>
+        <v>579472.79</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -845,7 +852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -868,7 +875,7 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>33000000</v>
+        <v>45500000</v>
       </c>
       <c r="I6">
         <v>768602.43</v>
@@ -877,28 +884,28 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>6661221.0700000003</v>
+        <v>4995915.8</v>
       </c>
       <c r="L6">
-        <v>20.190000000000001</v>
+        <v>10.98</v>
       </c>
       <c r="M6">
-        <v>256200.81</v>
+        <v>192150.61</v>
       </c>
       <c r="N6">
-        <v>1401365.11</v>
+        <v>2033245.34</v>
       </c>
       <c r="O6">
-        <v>3067038.47</v>
+        <v>1088444.5900000001</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>60625.14</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -921,37 +928,37 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>71500000</v>
+        <v>91000000</v>
       </c>
       <c r="I7">
-        <v>18816115.780000001</v>
+        <v>19037059.140000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>163073003.40000001</v>
+        <v>123740884.43000001</v>
       </c>
       <c r="L7">
-        <v>228.07</v>
+        <v>135.97999999999999</v>
       </c>
       <c r="M7">
-        <v>6272038.5899999999</v>
+        <v>4759264.79</v>
       </c>
       <c r="N7">
-        <v>2290603.66</v>
+        <v>3271042.77</v>
       </c>
       <c r="O7">
-        <v>3234098.85</v>
+        <v>9710259.8300000001</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>368037.02</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -974,7 +981,7 @@
         <v>22</v>
       </c>
       <c r="H8">
-        <v>44000000</v>
+        <v>45500000</v>
       </c>
       <c r="I8">
         <v>5649828.7800000003</v>
@@ -983,22 +990,22 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>48965182.759999998</v>
+        <v>36723887.07</v>
       </c>
       <c r="L8">
-        <v>111.28</v>
+        <v>80.709999999999994</v>
       </c>
       <c r="M8">
-        <v>1883276.26</v>
+        <v>1412457.2</v>
       </c>
       <c r="N8">
-        <v>1667398.75</v>
+        <v>1811371.42</v>
       </c>
       <c r="O8">
-        <v>26361556.239999998</v>
+        <v>10548816.68</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>10360021.949999999</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1206,7 +1213,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: actualizar inputs penaflor
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{993866C5-8199-441C-A20F-59555BE2C280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EE0DE98-AE2F-4C75-9506-62E05FEF4062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,13 +201,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="3RAS MARCAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -640,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -672,28 +666,28 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5797531.6699999999</v>
+        <v>4638025.34</v>
       </c>
       <c r="L2">
-        <v>58.8</v>
+        <v>47.04</v>
       </c>
       <c r="M2">
-        <v>222981.99</v>
+        <v>178385.59</v>
       </c>
       <c r="N2">
-        <v>407639.64</v>
+        <v>427051.05</v>
       </c>
       <c r="O2">
-        <v>134947.57999999999</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>196727.4</v>
+        <v>-181765.82</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -719,34 +713,34 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>8481334.3399999999</v>
+        <v>8829627.5700000003</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>55128673.210000001</v>
+        <v>45914063.340000004</v>
       </c>
       <c r="L3">
-        <v>114.52</v>
+        <v>95.38</v>
       </c>
       <c r="M3">
-        <v>2120333.58</v>
+        <v>1765925.51</v>
       </c>
       <c r="N3">
-        <v>1802666.62</v>
+        <v>1871922.5</v>
       </c>
       <c r="O3">
-        <v>315717.89</v>
+        <v>395241.47</v>
       </c>
       <c r="P3">
-        <v>236919.44</v>
+        <v>702630.97</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -772,34 +766,34 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>9264876.1099999994</v>
+        <v>10306795.449999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>60221694.700000003</v>
+        <v>53595336.32</v>
       </c>
       <c r="L4">
-        <v>46.32</v>
+        <v>41.23</v>
       </c>
       <c r="M4">
-        <v>2316219.0299999998</v>
+        <v>2061359.09</v>
       </c>
       <c r="N4">
-        <v>5487960.1799999997</v>
+        <v>5699676.4100000001</v>
       </c>
       <c r="O4">
-        <v>3155939.81</v>
+        <v>702757.91</v>
       </c>
       <c r="P4">
-        <v>34691925.590000004</v>
+        <v>1680125.82</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -825,34 +819,34 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>245750.97</v>
+        <v>220305.6</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1597381.32</v>
+        <v>1145589.1100000001</v>
       </c>
       <c r="L5">
-        <v>12.29</v>
+        <v>8.81</v>
       </c>
       <c r="M5">
-        <v>61437.74</v>
+        <v>44061.120000000003</v>
       </c>
       <c r="N5">
-        <v>579738.59</v>
+        <v>608556.88</v>
       </c>
       <c r="O5">
-        <v>579472.79</v>
+        <v>117844.11</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>188022.38</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -878,34 +872,34 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>768602.43</v>
+        <v>795516.05</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4995915.8</v>
+        <v>4136683.46</v>
       </c>
       <c r="L6">
-        <v>10.98</v>
+        <v>9.09</v>
       </c>
       <c r="M6">
-        <v>192150.61</v>
+        <v>159103.21</v>
       </c>
       <c r="N6">
-        <v>2033245.34</v>
+        <v>2128784.9500000002</v>
       </c>
       <c r="O6">
-        <v>1088444.5900000001</v>
+        <v>304316.25</v>
       </c>
       <c r="P6">
-        <v>60625.14</v>
+        <v>262869.42</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -931,34 +925,34 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>19037059.140000001</v>
+        <v>19317665.469999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>123740884.43000001</v>
+        <v>100451860.44</v>
       </c>
       <c r="L7">
-        <v>135.97999999999999</v>
+        <v>110.39</v>
       </c>
       <c r="M7">
-        <v>4759264.79</v>
+        <v>3863533.09</v>
       </c>
       <c r="N7">
-        <v>3271042.77</v>
+        <v>3413444.5</v>
       </c>
       <c r="O7">
-        <v>9710259.8300000001</v>
+        <v>318727.33</v>
       </c>
       <c r="P7">
-        <v>368037.02</v>
+        <v>356057.85</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -984,28 +978,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>5649828.7800000003</v>
+        <v>6364473.2999999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36723887.07</v>
+        <v>33095261.140000001</v>
       </c>
       <c r="L8">
-        <v>80.709999999999994</v>
+        <v>72.739999999999995</v>
       </c>
       <c r="M8">
-        <v>1412457.2</v>
+        <v>1272894.6599999999</v>
       </c>
       <c r="N8">
-        <v>1811371.42</v>
+        <v>1863596.51</v>
       </c>
       <c r="O8">
-        <v>10548816.68</v>
+        <v>318111.77</v>
       </c>
       <c r="P8">
-        <v>10360021.949999999</v>
+        <v>1749258.65</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1083,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1109,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1135,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1213,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1265,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: actualizar inputs penaflor para cierre dia
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EE0DE98-AE2F-4C75-9506-62E05FEF4062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3EE8C93-6313-478F-9BFF-9CC5C99E0156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -666,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4638025.34</v>
+        <v>3865021.11</v>
       </c>
       <c r="L2">
-        <v>47.04</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="M2">
-        <v>178385.59</v>
+        <v>148654.66</v>
       </c>
       <c r="N2">
-        <v>427051.05</v>
+        <v>448403.6</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>415894.77</v>
       </c>
       <c r="P2">
-        <v>-181765.82</v>
+        <v>70527.16</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>8829627.5700000003</v>
+        <v>15615052.939999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>45914063.340000004</v>
+        <v>67665229.420000002</v>
       </c>
       <c r="L3">
-        <v>95.38</v>
+        <v>140.56</v>
       </c>
       <c r="M3">
-        <v>1765925.51</v>
+        <v>2602508.8199999998</v>
       </c>
       <c r="N3">
-        <v>1871922.5</v>
+        <v>1626247.35</v>
       </c>
       <c r="O3">
-        <v>395241.47</v>
+        <v>987661.24</v>
       </c>
       <c r="P3">
-        <v>702630.97</v>
+        <v>723663.06</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>10306795.449999999</v>
+        <v>11507053.800000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>53595336.32</v>
+        <v>49863899.799999997</v>
       </c>
       <c r="L4">
-        <v>41.23</v>
+        <v>38.36</v>
       </c>
       <c r="M4">
-        <v>2061359.09</v>
+        <v>1917842.3</v>
       </c>
       <c r="N4">
-        <v>5699676.4100000001</v>
+        <v>5924647.3099999996</v>
       </c>
       <c r="O4">
-        <v>702757.91</v>
+        <v>1040768.47</v>
       </c>
       <c r="P4">
-        <v>1680125.82</v>
+        <v>1757342.23</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>220305.6</v>
+        <v>544043.37</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1145589.1100000001</v>
+        <v>2357521.2799999998</v>
       </c>
       <c r="L5">
-        <v>8.81</v>
+        <v>18.13</v>
       </c>
       <c r="M5">
-        <v>44061.120000000003</v>
+        <v>90673.9</v>
       </c>
       <c r="N5">
-        <v>608556.88</v>
+        <v>622797.82999999996</v>
       </c>
       <c r="O5">
-        <v>117844.11</v>
+        <v>18186.580000000002</v>
       </c>
       <c r="P5">
-        <v>188022.38</v>
+        <v>106430.41</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>795516.05</v>
+        <v>1026908.81</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4136683.46</v>
+        <v>4449938.1900000004</v>
       </c>
       <c r="L6">
-        <v>9.09</v>
+        <v>9.7799999999999994</v>
       </c>
       <c r="M6">
-        <v>159103.21</v>
+        <v>171151.47</v>
       </c>
       <c r="N6">
-        <v>2128784.9500000002</v>
+        <v>2223654.56</v>
       </c>
       <c r="O6">
-        <v>304316.25</v>
+        <v>264768.62</v>
       </c>
       <c r="P6">
-        <v>262869.42</v>
+        <v>331285.06</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>19317665.469999999</v>
+        <v>19398237.550000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>100451860.44</v>
+        <v>84059029.390000001</v>
       </c>
       <c r="L7">
-        <v>110.39</v>
+        <v>92.37</v>
       </c>
       <c r="M7">
-        <v>3863533.09</v>
+        <v>3233039.59</v>
       </c>
       <c r="N7">
-        <v>3413444.5</v>
+        <v>3580088.12</v>
       </c>
       <c r="O7">
-        <v>318727.33</v>
+        <v>17390273.739999998</v>
       </c>
       <c r="P7">
-        <v>356057.85</v>
+        <v>3353629.25</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>6364473.2999999998</v>
+        <v>7240028.8099999996</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>33095261.140000001</v>
+        <v>31373458.170000002</v>
       </c>
       <c r="L8">
-        <v>72.739999999999995</v>
+        <v>68.95</v>
       </c>
       <c r="M8">
-        <v>1272894.6599999999</v>
+        <v>1206671.47</v>
       </c>
       <c r="N8">
-        <v>1863596.51</v>
+        <v>1912998.56</v>
       </c>
       <c r="O8">
-        <v>318111.77</v>
+        <v>291324.99</v>
       </c>
       <c r="P8">
-        <v>1749258.65</v>
+        <v>343916.48</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: actualizar inputs penaflor post-cierre 2026-07-07
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3EE8C93-6313-478F-9BFF-9CC5C99E0156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{444C1F05-03D4-4E09-AEFB-788B1F64AE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>891927.95</v>
+        <v>1768327.83</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3865021.11</v>
+        <v>6568074.7800000003</v>
       </c>
       <c r="L2">
-        <v>39.200000000000003</v>
+        <v>66.61</v>
       </c>
       <c r="M2">
-        <v>148654.66</v>
+        <v>252618.26</v>
       </c>
       <c r="N2">
-        <v>448403.6</v>
+        <v>425877.48</v>
       </c>
       <c r="O2">
-        <v>415894.77</v>
+        <v>449318.45</v>
       </c>
       <c r="P2">
-        <v>70527.16</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>15615052.939999999</v>
+        <v>17237230.52</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>67665229.420000002</v>
+        <v>64023999.079999998</v>
       </c>
       <c r="L3">
-        <v>140.56</v>
+        <v>133</v>
       </c>
       <c r="M3">
-        <v>2602508.8199999998</v>
+        <v>2462461.5</v>
       </c>
       <c r="N3">
-        <v>1626247.35</v>
+        <v>1626461.55</v>
       </c>
       <c r="O3">
-        <v>987661.24</v>
+        <v>488800.04</v>
       </c>
       <c r="P3">
-        <v>723663.06</v>
+        <v>-342803.04</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>11507053.800000001</v>
+        <v>11048319.32</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>49863899.799999997</v>
+        <v>41036614.619999997</v>
       </c>
       <c r="L4">
-        <v>38.36</v>
+        <v>31.57</v>
       </c>
       <c r="M4">
-        <v>1917842.3</v>
+        <v>1578331.33</v>
       </c>
       <c r="N4">
-        <v>5924647.3099999996</v>
+        <v>6260614.7699999996</v>
       </c>
       <c r="O4">
-        <v>1040768.47</v>
+        <v>2285204.46</v>
       </c>
       <c r="P4">
-        <v>1757342.23</v>
+        <v>2831970.3</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>544043.37</v>
+        <v>669564.28</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2357521.2799999998</v>
+        <v>2486953.0299999998</v>
       </c>
       <c r="L5">
-        <v>18.13</v>
+        <v>19.13</v>
       </c>
       <c r="M5">
-        <v>90673.9</v>
+        <v>95652.04</v>
       </c>
       <c r="N5">
-        <v>622797.82999999996</v>
+        <v>648970.30000000005</v>
       </c>
       <c r="O5">
-        <v>18186.580000000002</v>
+        <v>27708.09</v>
       </c>
       <c r="P5">
-        <v>106430.41</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4449938.1900000004</v>
+        <v>3814232.74</v>
       </c>
       <c r="L6">
-        <v>9.7799999999999994</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="M6">
-        <v>171151.47</v>
+        <v>146701.26</v>
       </c>
       <c r="N6">
-        <v>2223654.56</v>
+        <v>2340689.0099999998</v>
       </c>
       <c r="O6">
-        <v>264768.62</v>
+        <v>178150.45</v>
       </c>
       <c r="P6">
-        <v>331285.06</v>
+        <v>48035649.380000003</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>19398237.550000001</v>
+        <v>20206402.109999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>84059029.390000001</v>
+        <v>75052350.709999993</v>
       </c>
       <c r="L7">
-        <v>92.37</v>
+        <v>82.48</v>
       </c>
       <c r="M7">
-        <v>3233039.59</v>
+        <v>2886628.87</v>
       </c>
       <c r="N7">
-        <v>3580088.12</v>
+        <v>3725978.84</v>
       </c>
       <c r="O7">
-        <v>17390273.739999998</v>
+        <v>424987.6</v>
       </c>
       <c r="P7">
-        <v>3353629.25</v>
+        <v>475852.73</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>7240028.8099999996</v>
+        <v>7490500.8300000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>31373458.170000002</v>
+        <v>27821860.219999999</v>
       </c>
       <c r="L8">
-        <v>68.95</v>
+        <v>61.15</v>
       </c>
       <c r="M8">
-        <v>1206671.47</v>
+        <v>1070071.55</v>
       </c>
       <c r="N8">
-        <v>1912998.56</v>
+        <v>2000499.96</v>
       </c>
       <c r="O8">
-        <v>291324.99</v>
+        <v>4776120.17</v>
       </c>
       <c r="P8">
-        <v>343916.48</v>
+        <v>1303649.54</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1.1000000000000001</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.7</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-10_1758 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{444C1F05-03D4-4E09-AEFB-788B1F64AE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70BED65A-D58B-425B-ABC8-795B301047C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>1768327.83</v>
+        <v>1722758.42</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6568074.7800000003</v>
+        <v>5598964.8499999996</v>
       </c>
       <c r="L2">
-        <v>66.61</v>
+        <v>56.78</v>
       </c>
       <c r="M2">
-        <v>252618.26</v>
+        <v>215344.8</v>
       </c>
       <c r="N2">
-        <v>425877.48</v>
+        <v>452068.98</v>
       </c>
       <c r="O2">
-        <v>449318.45</v>
+        <v>26714.73</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>15658.95</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>17237230.52</v>
+        <v>18072233.800000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>64023999.079999998</v>
+        <v>58734759.859999999</v>
       </c>
       <c r="L3">
-        <v>133</v>
+        <v>122.01</v>
       </c>
       <c r="M3">
-        <v>2462461.5</v>
+        <v>2259029.23</v>
       </c>
       <c r="N3">
-        <v>1626461.55</v>
+        <v>1670431.46</v>
       </c>
       <c r="O3">
-        <v>488800.04</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>-342803.04</v>
+        <v>399557.34</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>11048319.32</v>
+        <v>11311141.34</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>41036614.619999997</v>
+        <v>36761209.369999997</v>
       </c>
       <c r="L4">
-        <v>31.57</v>
+        <v>28.28</v>
       </c>
       <c r="M4">
-        <v>1578331.33</v>
+        <v>1413892.67</v>
       </c>
       <c r="N4">
-        <v>6260614.7699999996</v>
+        <v>6593825.4800000004</v>
       </c>
       <c r="O4">
-        <v>2285204.46</v>
+        <v>3559480.53</v>
       </c>
       <c r="P4">
-        <v>2831970.3</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>669564.28</v>
+        <v>880093.02</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2486953.0299999998</v>
+        <v>2860302.33</v>
       </c>
       <c r="L5">
-        <v>19.13</v>
+        <v>22</v>
       </c>
       <c r="M5">
-        <v>95652.04</v>
+        <v>110011.63</v>
       </c>
       <c r="N5">
-        <v>648970.30000000005</v>
+        <v>673328.17</v>
       </c>
       <c r="O5">
-        <v>27708.09</v>
+        <v>11519.65</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>21888.49</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>1026908.81</v>
+        <v>1090642.3600000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3814232.74</v>
+        <v>3544587.67</v>
       </c>
       <c r="L6">
-        <v>8.3800000000000008</v>
+        <v>7.79</v>
       </c>
       <c r="M6">
-        <v>146701.26</v>
+        <v>136330.29</v>
       </c>
       <c r="N6">
-        <v>2340689.0099999998</v>
+        <v>2467186.54</v>
       </c>
       <c r="O6">
-        <v>178150.45</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>48035649.380000003</v>
+        <v>3067038.47</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>20206402.109999999</v>
+        <v>20882953</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>75052350.709999993</v>
+        <v>67869597.25</v>
       </c>
       <c r="L7">
-        <v>82.48</v>
+        <v>74.58</v>
       </c>
       <c r="M7">
-        <v>2886628.87</v>
+        <v>2610369.12</v>
       </c>
       <c r="N7">
-        <v>3725978.84</v>
+        <v>3895391.5</v>
       </c>
       <c r="O7">
-        <v>424987.6</v>
+        <v>220943.37</v>
       </c>
       <c r="P7">
-        <v>475852.73</v>
+        <v>3234098.85</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>7490500.8300000001</v>
+        <v>8356459.8200000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>27821860.219999999</v>
+        <v>27158494.41</v>
       </c>
       <c r="L8">
-        <v>61.15</v>
+        <v>59.69</v>
       </c>
       <c r="M8">
-        <v>1070071.55</v>
+        <v>1044557.48</v>
       </c>
       <c r="N8">
-        <v>2000499.96</v>
+        <v>2063530.01</v>
       </c>
       <c r="O8">
-        <v>4776120.17</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>1303649.54</v>
+        <v>26361556.239999998</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>17.3</v>
+        <v>16.899999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-12_1256 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70BED65A-D58B-425B-ABC8-795B301047C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{50444F4D-B835-4604-AC51-80765564331E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>1722758.42</v>
+        <v>1737658.55</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5598964.8499999996</v>
+        <v>5019902.4800000004</v>
       </c>
       <c r="L2">
-        <v>56.78</v>
+        <v>50.91</v>
       </c>
       <c r="M2">
-        <v>215344.8</v>
+        <v>193073.17</v>
       </c>
       <c r="N2">
-        <v>452068.98</v>
+        <v>477784.79</v>
       </c>
       <c r="O2">
-        <v>26714.73</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>15658.95</v>
+        <v>134947.57999999999</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>18072233.800000001</v>
+        <v>18298432.149999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>58734759.859999999</v>
+        <v>52862137.329999998</v>
       </c>
       <c r="L3">
-        <v>122.01</v>
+        <v>109.81</v>
       </c>
       <c r="M3">
-        <v>2259029.23</v>
+        <v>2033159.13</v>
       </c>
       <c r="N3">
-        <v>1670431.46</v>
+        <v>1755386.34</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>348293.23</v>
       </c>
       <c r="P3">
-        <v>399557.34</v>
+        <v>315717.89</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>11311141.34</v>
+        <v>11323821.130000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>36761209.369999997</v>
+        <v>32713261.050000001</v>
       </c>
       <c r="L4">
-        <v>28.28</v>
+        <v>25.16</v>
       </c>
       <c r="M4">
-        <v>1413892.67</v>
+        <v>1258202.3500000001</v>
       </c>
       <c r="N4">
-        <v>6593825.4800000004</v>
+        <v>6980951.7000000002</v>
       </c>
       <c r="O4">
-        <v>3559480.53</v>
+        <v>1245734.48</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>3155939.81</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2860302.33</v>
+        <v>2542490.96</v>
       </c>
       <c r="L5">
-        <v>22</v>
+        <v>19.559999999999999</v>
       </c>
       <c r="M5">
-        <v>110011.63</v>
+        <v>97788.11</v>
       </c>
       <c r="N5">
-        <v>673328.17</v>
+        <v>712935.7</v>
       </c>
       <c r="O5">
-        <v>11519.65</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>21888.49</v>
+        <v>579472.79</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3544587.67</v>
+        <v>3150744.59</v>
       </c>
       <c r="L6">
-        <v>7.79</v>
+        <v>6.92</v>
       </c>
       <c r="M6">
-        <v>136330.29</v>
+        <v>121182.48</v>
       </c>
       <c r="N6">
-        <v>2467186.54</v>
+        <v>2612315.16</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>26913.62</v>
       </c>
       <c r="P6">
-        <v>3067038.47</v>
+        <v>1088444.5900000001</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>20882953</v>
+        <v>20862670.219999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>67869597.25</v>
+        <v>60269936.189999998</v>
       </c>
       <c r="L7">
-        <v>74.58</v>
+        <v>66.23</v>
       </c>
       <c r="M7">
-        <v>2610369.12</v>
+        <v>2318074.4700000002</v>
       </c>
       <c r="N7">
-        <v>3895391.5</v>
+        <v>4125725.28</v>
       </c>
       <c r="O7">
-        <v>220943.37</v>
+        <v>372790.18</v>
       </c>
       <c r="P7">
-        <v>3234098.85</v>
+        <v>9710259.8300000001</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>8356459.8200000003</v>
+        <v>8277551.3300000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>27158494.41</v>
+        <v>23912926.059999999</v>
       </c>
       <c r="L8">
-        <v>59.69</v>
+        <v>52.56</v>
       </c>
       <c r="M8">
-        <v>1044557.48</v>
+        <v>919727.93</v>
       </c>
       <c r="N8">
-        <v>2063530.01</v>
+        <v>2189555.7999999998</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>828460.1</v>
       </c>
       <c r="P8">
-        <v>26361556.239999998</v>
+        <v>10548816.68</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>16.899999999999999</v>
+        <v>17.399999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-13_1827 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{50444F4D-B835-4604-AC51-80765564331E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD1849A8-125E-4F81-A535-FF45F50C3B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>1737658.55</v>
+        <v>1708916.06</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5019902.4800000004</v>
+        <v>4443181.7699999996</v>
       </c>
       <c r="L2">
-        <v>50.91</v>
+        <v>45.06</v>
       </c>
       <c r="M2">
-        <v>193073.17</v>
+        <v>170891.61</v>
       </c>
       <c r="N2">
-        <v>477784.79</v>
+        <v>509442.75</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>117618.27</v>
       </c>
       <c r="P2">
-        <v>134947.57999999999</v>
+        <v>1455032.16</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>18298432.149999999</v>
+        <v>20555495.190000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>52862137.329999998</v>
+        <v>53444287.5</v>
       </c>
       <c r="L3">
-        <v>109.81</v>
+        <v>111.02</v>
       </c>
       <c r="M3">
-        <v>2033159.13</v>
+        <v>2055549.52</v>
       </c>
       <c r="N3">
-        <v>1755386.34</v>
+        <v>1724031.55</v>
       </c>
       <c r="O3">
-        <v>348293.23</v>
+        <v>6868071.1100000003</v>
       </c>
       <c r="P3">
-        <v>315717.89</v>
+        <v>7202218.3300000001</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>11323821.130000001</v>
+        <v>18527845.969999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>32713261.050000001</v>
+        <v>48172399.530000001</v>
       </c>
       <c r="L4">
-        <v>25.16</v>
+        <v>37.06</v>
       </c>
       <c r="M4">
-        <v>1258202.3500000001</v>
+        <v>1852784.6</v>
       </c>
       <c r="N4">
-        <v>6980951.7000000002</v>
+        <v>6967009.6299999999</v>
       </c>
       <c r="O4">
-        <v>1245734.48</v>
+        <v>1200258.3500000001</v>
       </c>
       <c r="P4">
-        <v>3155939.81</v>
+        <v>1841855.42</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2542490.96</v>
+        <v>2288241.86</v>
       </c>
       <c r="L5">
-        <v>19.559999999999999</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="M5">
-        <v>97788.11</v>
+        <v>88009.3</v>
       </c>
       <c r="N5">
-        <v>712935.7</v>
+        <v>757494.19</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>323737.77</v>
       </c>
       <c r="P5">
-        <v>579472.79</v>
+        <v>560820.93000000005</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>1090642.3600000001</v>
+        <v>1172001.48</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3150744.59</v>
+        <v>3047203.84</v>
       </c>
       <c r="L6">
-        <v>6.92</v>
+        <v>6.7</v>
       </c>
       <c r="M6">
-        <v>121182.48</v>
+        <v>117200.15</v>
       </c>
       <c r="N6">
-        <v>2612315.16</v>
+        <v>2770499.91</v>
       </c>
       <c r="O6">
-        <v>26913.62</v>
+        <v>231392.76</v>
       </c>
       <c r="P6">
-        <v>1088444.5900000001</v>
+        <v>218449.26</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>20862670.219999999</v>
+        <v>21190015.670000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>60269936.189999998</v>
+        <v>55094040.740000002</v>
       </c>
       <c r="L7">
-        <v>66.23</v>
+        <v>60.54</v>
       </c>
       <c r="M7">
-        <v>2318074.4700000002</v>
+        <v>2119001.5699999998</v>
       </c>
       <c r="N7">
-        <v>4125725.28</v>
+        <v>4363124.0199999996</v>
       </c>
       <c r="O7">
-        <v>372790.18</v>
+        <v>80572.08</v>
       </c>
       <c r="P7">
-        <v>9710259.8300000001</v>
+        <v>707831.01</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>8277551.3300000001</v>
+        <v>8398011.1199999992</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23912926.059999999</v>
+        <v>21834828.920000002</v>
       </c>
       <c r="L8">
-        <v>52.56</v>
+        <v>47.99</v>
       </c>
       <c r="M8">
-        <v>919727.93</v>
+        <v>839801.11</v>
       </c>
       <c r="N8">
-        <v>2189555.7999999998</v>
+        <v>2318874.2999999998</v>
       </c>
       <c r="O8">
-        <v>828460.1</v>
+        <v>807818.53</v>
       </c>
       <c r="P8">
-        <v>10548816.68</v>
+        <v>491427.49</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>17.399999999999999</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2000000000000002</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-15_1503 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3521A281-3983-4D4C-9733-FD0280825ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA1440F2-CC5B-43B7-AFE3-8BCF463A9AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4314530.17</v>
+        <v>3954985.99</v>
       </c>
       <c r="L2">
-        <v>43.76</v>
+        <v>40.11</v>
       </c>
       <c r="M2">
-        <v>165943.47</v>
+        <v>152114.85</v>
       </c>
       <c r="N2">
-        <v>535641.46</v>
+        <v>573901.56000000006</v>
       </c>
       <c r="O2">
-        <v>713212.19</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>415894.77</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>22721946.800000001</v>
+        <v>22850529.48</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>53706419.719999999</v>
+        <v>49509480.549999997</v>
       </c>
       <c r="L3">
-        <v>111.56</v>
+        <v>102.84</v>
       </c>
       <c r="M3">
-        <v>2065631.53</v>
+        <v>1904210.79</v>
       </c>
       <c r="N3">
-        <v>1694536.88</v>
+        <v>1806390.75</v>
       </c>
       <c r="O3">
-        <v>8236614.79</v>
+        <v>132922.32999999999</v>
       </c>
       <c r="P3">
-        <v>395241.47</v>
+        <v>987661.24</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>19718206.789999999</v>
+        <v>20921134.390000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>46606670.600000001</v>
+        <v>45329124.509999998</v>
       </c>
       <c r="L4">
-        <v>35.85</v>
+        <v>34.869999999999997</v>
       </c>
       <c r="M4">
-        <v>1792564.25</v>
+        <v>1743427.87</v>
       </c>
       <c r="N4">
-        <v>7352119.5499999998</v>
+        <v>7791347.54</v>
       </c>
       <c r="O4">
-        <v>-458734.48</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>702757.91</v>
+        <v>1040768.47</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>948256.86</v>
+        <v>970911.52</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2241334.39</v>
+        <v>2103641.64</v>
       </c>
       <c r="L5">
-        <v>17.239999999999998</v>
+        <v>16.18</v>
       </c>
       <c r="M5">
-        <v>86205.17</v>
+        <v>80909.289999999994</v>
       </c>
       <c r="N5">
-        <v>803449.54</v>
+        <v>859220.61</v>
       </c>
       <c r="O5">
-        <v>125520.9</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>117844.11</v>
+        <v>18186.580000000002</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>1197661.95</v>
+        <v>1427337.2</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>2830837.33</v>
+        <v>3092563.94</v>
       </c>
       <c r="L6">
-        <v>6.22</v>
+        <v>6.8</v>
       </c>
       <c r="M6">
-        <v>108878.36</v>
+        <v>118944.77</v>
       </c>
       <c r="N6">
-        <v>2953489.2</v>
+        <v>3148047.34</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>304316.25</v>
+        <v>264768.62</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>24470313.039999999</v>
+        <v>24681002.280000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>57838921.719999999</v>
+        <v>53475504.939999998</v>
       </c>
       <c r="L7">
-        <v>63.56</v>
+        <v>58.76</v>
       </c>
       <c r="M7">
-        <v>2224573.91</v>
+        <v>2056750.19</v>
       </c>
       <c r="N7">
-        <v>4435312.46</v>
+        <v>4737071.2699999996</v>
       </c>
       <c r="O7">
-        <v>804063.74</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>318727.33</v>
+        <v>17390273.739999998</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>8628124.4100000001</v>
+        <v>9331932.3900000006</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20393748.609999999</v>
+        <v>20219186.84</v>
       </c>
       <c r="L8">
-        <v>44.82</v>
+        <v>44.44</v>
       </c>
       <c r="M8">
-        <v>784374.95</v>
+        <v>777661.03</v>
       </c>
       <c r="N8">
-        <v>2458125.04</v>
+        <v>2583433.4</v>
       </c>
       <c r="O8">
-        <v>250472.02</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>318111.77</v>
+        <v>291324.99</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-16_1928 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA1440F2-CC5B-43B7-AFE3-8BCF463A9AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD230D04-5707-4DF0-BD18-6871B77C47AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>1825378.15</v>
+        <v>2880718.44</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3954985.99</v>
+        <v>5761436.8799999999</v>
       </c>
       <c r="L2">
-        <v>40.11</v>
+        <v>58.43</v>
       </c>
       <c r="M2">
-        <v>152114.85</v>
+        <v>221593.73</v>
       </c>
       <c r="N2">
-        <v>573901.56000000006</v>
+        <v>536867.81000000006</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>415894.77</v>
+        <v>449318.45</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>22850529.48</v>
+        <v>24769694.100000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49509480.549999997</v>
+        <v>49539388.210000001</v>
       </c>
       <c r="L3">
-        <v>102.84</v>
+        <v>102.91</v>
       </c>
       <c r="M3">
-        <v>1904210.79</v>
+        <v>1905361.08</v>
       </c>
       <c r="N3">
-        <v>1806390.75</v>
+        <v>1797715.84</v>
       </c>
       <c r="O3">
-        <v>132922.32999999999</v>
+        <v>565082.69999999995</v>
       </c>
       <c r="P3">
-        <v>987661.24</v>
+        <v>488800.04</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>20921134.390000001</v>
+        <v>24544254.359999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>45329124.509999998</v>
+        <v>49088508.719999999</v>
       </c>
       <c r="L4">
-        <v>34.869999999999997</v>
+        <v>37.76</v>
       </c>
       <c r="M4">
-        <v>1743427.87</v>
+        <v>1888019.57</v>
       </c>
       <c r="N4">
-        <v>7791347.54</v>
+        <v>8111980.4299999997</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>262822.02</v>
       </c>
       <c r="P4">
-        <v>1040768.47</v>
+        <v>2285204.46</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>970911.52</v>
+        <v>991959.14</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2103641.64</v>
+        <v>1983918.28</v>
       </c>
       <c r="L5">
-        <v>16.18</v>
+        <v>15.26</v>
       </c>
       <c r="M5">
-        <v>80909.289999999994</v>
+        <v>76304.55</v>
       </c>
       <c r="N5">
-        <v>859220.61</v>
+        <v>923695.45</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>210528.75</v>
       </c>
       <c r="P5">
-        <v>18186.580000000002</v>
+        <v>27708.09</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>1427337.2</v>
+        <v>2440817.54</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3092563.94</v>
+        <v>4881635.09</v>
       </c>
       <c r="L6">
-        <v>6.8</v>
+        <v>10.73</v>
       </c>
       <c r="M6">
-        <v>118944.77</v>
+        <v>187755.2</v>
       </c>
       <c r="N6">
-        <v>3148047.34</v>
+        <v>3312244.8</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>63733.55</v>
       </c>
       <c r="P6">
-        <v>264768.62</v>
+        <v>178150.45</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>24681002.280000001</v>
+        <v>28499952.41</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>53475504.939999998</v>
+        <v>56999904.82</v>
       </c>
       <c r="L7">
-        <v>58.76</v>
+        <v>62.64</v>
       </c>
       <c r="M7">
-        <v>2056750.19</v>
+        <v>2192304.0299999998</v>
       </c>
       <c r="N7">
-        <v>4737071.2699999996</v>
+        <v>4807695.97</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>680651.7</v>
       </c>
       <c r="P7">
-        <v>17390273.739999998</v>
+        <v>424987.6</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>9331932.3900000006</v>
+        <v>10570865.84</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20219186.84</v>
+        <v>21141731.670000002</v>
       </c>
       <c r="L8">
-        <v>44.44</v>
+        <v>46.47</v>
       </c>
       <c r="M8">
-        <v>777661.03</v>
+        <v>813143.53</v>
       </c>
       <c r="N8">
-        <v>2583433.4</v>
+        <v>2686856.47</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>865958.99</v>
       </c>
       <c r="P8">
-        <v>291324.99</v>
+        <v>4776120.17</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.3</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>1.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>9.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-17_1722 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD230D04-5707-4DF0-BD18-6871B77C47AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6E035D3-BB1A-4EDB-9B65-F2E9D4E42672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5761436.8799999999</v>
+        <v>5349905.67</v>
       </c>
       <c r="L2">
-        <v>58.43</v>
+        <v>54.26</v>
       </c>
       <c r="M2">
-        <v>221593.73</v>
+        <v>205765.6</v>
       </c>
       <c r="N2">
-        <v>536867.81000000006</v>
+        <v>581606.80000000005</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>14900.13</v>
       </c>
       <c r="P2">
-        <v>449318.45</v>
+        <v>26714.73</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>24769694.100000001</v>
+        <v>31894141.25</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49539388.210000001</v>
+        <v>59231976.600000001</v>
       </c>
       <c r="L3">
-        <v>102.91</v>
+        <v>123.04</v>
       </c>
       <c r="M3">
-        <v>1905361.08</v>
+        <v>2278152.9500000002</v>
       </c>
       <c r="N3">
-        <v>1797715.84</v>
+        <v>1353821.56</v>
       </c>
       <c r="O3">
-        <v>565082.69999999995</v>
+        <v>226198.35</v>
       </c>
       <c r="P3">
-        <v>488800.04</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>24544254.359999999</v>
+        <v>24736830.460000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>49088508.719999999</v>
+        <v>45939828</v>
       </c>
       <c r="L4">
-        <v>37.76</v>
+        <v>35.340000000000003</v>
       </c>
       <c r="M4">
-        <v>1888019.57</v>
+        <v>1766916.46</v>
       </c>
       <c r="N4">
-        <v>8111980.4299999997</v>
+        <v>8771930.7899999991</v>
       </c>
       <c r="O4">
-        <v>262822.02</v>
+        <v>12679.79</v>
       </c>
       <c r="P4">
-        <v>2285204.46</v>
+        <v>3559480.53</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>991959.14</v>
+        <v>1290758.5900000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1983918.28</v>
+        <v>2397123.09</v>
       </c>
       <c r="L5">
-        <v>15.26</v>
+        <v>18.440000000000001</v>
       </c>
       <c r="M5">
-        <v>76304.55</v>
+        <v>92197.04</v>
       </c>
       <c r="N5">
-        <v>923695.45</v>
+        <v>975770.12</v>
       </c>
       <c r="O5">
-        <v>210528.75</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>27708.09</v>
+        <v>11519.65</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>2440817.54</v>
+        <v>2870846.68</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4881635.09</v>
+        <v>5331572.41</v>
       </c>
       <c r="L6">
-        <v>10.73</v>
+        <v>11.72</v>
       </c>
       <c r="M6">
-        <v>187755.2</v>
+        <v>205060.48000000001</v>
       </c>
       <c r="N6">
-        <v>3312244.8</v>
+        <v>3552429.44</v>
       </c>
       <c r="O6">
-        <v>63733.55</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>178150.45</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>28499952.41</v>
+        <v>30187830.23</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>56999904.82</v>
+        <v>56063113.289999999</v>
       </c>
       <c r="L7">
-        <v>62.64</v>
+        <v>61.61</v>
       </c>
       <c r="M7">
-        <v>2192304.0299999998</v>
+        <v>2156273.59</v>
       </c>
       <c r="N7">
-        <v>4807695.97</v>
+        <v>5067680.8099999996</v>
       </c>
       <c r="O7">
-        <v>680651.7</v>
+        <v>-20282.78</v>
       </c>
       <c r="P7">
-        <v>424987.6</v>
+        <v>220943.37</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>10570865.84</v>
+        <v>11829587.970000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>21141731.670000002</v>
+        <v>21969234.800000001</v>
       </c>
       <c r="L8">
-        <v>46.47</v>
+        <v>48.28</v>
       </c>
       <c r="M8">
-        <v>813143.53</v>
+        <v>844970.57</v>
       </c>
       <c r="N8">
-        <v>2686856.47</v>
+        <v>2805867.67</v>
       </c>
       <c r="O8">
-        <v>865958.99</v>
+        <v>-78908.490000000005</v>
       </c>
       <c r="P8">
-        <v>4776120.17</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.1000000000000001</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-19_2018 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6E035D3-BB1A-4EDB-9B65-F2E9D4E42672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9236E198-8284-4F2C-843C-96E6EC67AD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>2880718.44</v>
+        <v>2895618.57</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5349905.67</v>
+        <v>5019072.1900000004</v>
       </c>
       <c r="L2">
-        <v>54.26</v>
+        <v>50.9</v>
       </c>
       <c r="M2">
-        <v>205765.6</v>
+        <v>193041.24</v>
       </c>
       <c r="N2">
-        <v>581606.80000000005</v>
+        <v>633125.57999999996</v>
       </c>
       <c r="O2">
-        <v>14900.13</v>
+        <v>-28742.49</v>
       </c>
       <c r="P2">
-        <v>26714.73</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>31894141.25</v>
+        <v>32189506.699999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>59231976.600000001</v>
+        <v>55795144.939999998</v>
       </c>
       <c r="L3">
-        <v>123.04</v>
+        <v>115.9</v>
       </c>
       <c r="M3">
-        <v>2278152.9500000002</v>
+        <v>2145967.11</v>
       </c>
       <c r="N3">
-        <v>1353821.56</v>
+        <v>1450044.85</v>
       </c>
       <c r="O3">
-        <v>226198.35</v>
+        <v>642206.39</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>348293.23</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -771,22 +771,22 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>45939828</v>
+        <v>42877172.799999997</v>
       </c>
       <c r="L4">
-        <v>35.340000000000003</v>
+        <v>32.979999999999997</v>
       </c>
       <c r="M4">
-        <v>1766916.46</v>
+        <v>1649122.03</v>
       </c>
       <c r="N4">
-        <v>8771930.7899999991</v>
+        <v>9569379.0500000007</v>
       </c>
       <c r="O4">
-        <v>12679.79</v>
+        <v>7204024.8399999999</v>
       </c>
       <c r="P4">
-        <v>3559480.53</v>
+        <v>1245734.48</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2397123.09</v>
+        <v>2237314.88</v>
       </c>
       <c r="L5">
-        <v>18.440000000000001</v>
+        <v>17.21</v>
       </c>
       <c r="M5">
-        <v>92197.04</v>
+        <v>86050.57</v>
       </c>
       <c r="N5">
-        <v>975770.12</v>
+        <v>1064476.49</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>11519.65</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5331572.41</v>
+        <v>4976134.25</v>
       </c>
       <c r="L6">
-        <v>11.72</v>
+        <v>10.94</v>
       </c>
       <c r="M6">
-        <v>205060.48000000001</v>
+        <v>191389.78</v>
       </c>
       <c r="N6">
-        <v>3552429.44</v>
+        <v>3875377.57</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>81359.12</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>26913.62</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -930,22 +930,22 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>56063113.289999999</v>
+        <v>52325572.399999999</v>
       </c>
       <c r="L7">
-        <v>61.61</v>
+        <v>57.5</v>
       </c>
       <c r="M7">
-        <v>2156273.59</v>
+        <v>2012522.02</v>
       </c>
       <c r="N7">
-        <v>5067680.8099999996</v>
+        <v>5528379.0700000003</v>
       </c>
       <c r="O7">
-        <v>-20282.78</v>
+        <v>327345.45</v>
       </c>
       <c r="P7">
-        <v>220943.37</v>
+        <v>372790.18</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,22 +983,22 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>21969234.800000001</v>
+        <v>20504619.149999999</v>
       </c>
       <c r="L8">
-        <v>48.28</v>
+        <v>45.07</v>
       </c>
       <c r="M8">
-        <v>844970.57</v>
+        <v>788639.2</v>
       </c>
       <c r="N8">
-        <v>2805867.67</v>
+        <v>3060946.55</v>
       </c>
       <c r="O8">
-        <v>-78908.490000000005</v>
+        <v>120459.8</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>828460.1</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.4</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-20_1746 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9236E198-8284-4F2C-843C-96E6EC67AD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{510828BE-BB56-4DB3-A392-0FE7E21F5BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5019072.1900000004</v>
+        <v>4705380.18</v>
       </c>
       <c r="L2">
-        <v>50.9</v>
+        <v>47.72</v>
       </c>
       <c r="M2">
-        <v>193041.24</v>
+        <v>180976.16</v>
       </c>
       <c r="N2">
-        <v>633125.57999999996</v>
+        <v>696438.14</v>
       </c>
       <c r="O2">
-        <v>-28742.49</v>
+        <v>116462.09</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>117618.27</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -718,22 +718,22 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>55795144.939999998</v>
+        <v>52307948.380000003</v>
       </c>
       <c r="L3">
-        <v>115.9</v>
+        <v>108.66</v>
       </c>
       <c r="M3">
-        <v>2145967.11</v>
+        <v>2011844.17</v>
       </c>
       <c r="N3">
-        <v>1450044.85</v>
+        <v>1595049.33</v>
       </c>
       <c r="O3">
-        <v>642206.39</v>
+        <v>1987065.72</v>
       </c>
       <c r="P3">
-        <v>348293.23</v>
+        <v>6868071.1100000003</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>24736830.460000001</v>
+        <v>33097778.16</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>42877172.799999997</v>
+        <v>53783889.509999998</v>
       </c>
       <c r="L4">
-        <v>32.979999999999997</v>
+        <v>41.37</v>
       </c>
       <c r="M4">
-        <v>1649122.03</v>
+        <v>2068611.13</v>
       </c>
       <c r="N4">
-        <v>9569379.0500000007</v>
+        <v>9690222.1799999997</v>
       </c>
       <c r="O4">
-        <v>7204024.8399999999</v>
+        <v>1190360.82</v>
       </c>
       <c r="P4">
-        <v>1245734.48</v>
+        <v>1200258.3500000001</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2237314.88</v>
+        <v>2097482.7000000002</v>
       </c>
       <c r="L5">
-        <v>17.21</v>
+        <v>16.13</v>
       </c>
       <c r="M5">
-        <v>86050.57</v>
+        <v>80672.41</v>
       </c>
       <c r="N5">
-        <v>1064476.49</v>
+        <v>1170924.1399999999</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>68163.83</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>323737.77</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>2870846.68</v>
+        <v>2941011.13</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4976134.25</v>
+        <v>4779143.09</v>
       </c>
       <c r="L6">
-        <v>10.94</v>
+        <v>10.5</v>
       </c>
       <c r="M6">
-        <v>191389.78</v>
+        <v>183813.2</v>
       </c>
       <c r="N6">
-        <v>3875377.57</v>
+        <v>4255898.8899999997</v>
       </c>
       <c r="O6">
-        <v>81359.12</v>
+        <v>25660.47</v>
       </c>
       <c r="P6">
-        <v>26913.62</v>
+        <v>231392.76</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>30187830.23</v>
+        <v>31020778.82</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>52325572.399999999</v>
+        <v>50408765.579999998</v>
       </c>
       <c r="L7">
-        <v>57.5</v>
+        <v>55.39</v>
       </c>
       <c r="M7">
-        <v>2012522.02</v>
+        <v>1938798.68</v>
       </c>
       <c r="N7">
-        <v>5528379.0700000003</v>
+        <v>5997922.1200000001</v>
       </c>
       <c r="O7">
-        <v>327345.45</v>
+        <v>3516082.85</v>
       </c>
       <c r="P7">
-        <v>372790.18</v>
+        <v>80572.08</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>11829587.970000001</v>
+        <v>13366762.15</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20504619.149999999</v>
+        <v>21720988.489999998</v>
       </c>
       <c r="L8">
-        <v>45.07</v>
+        <v>47.74</v>
       </c>
       <c r="M8">
-        <v>788639.2</v>
+        <v>835422.63</v>
       </c>
       <c r="N8">
-        <v>3060946.55</v>
+        <v>3213323.79</v>
       </c>
       <c r="O8">
-        <v>120459.8</v>
+        <v>230113.29</v>
       </c>
       <c r="P8">
-        <v>828460.1</v>
+        <v>807818.53</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.2999999999999998</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-22_1908 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69BA187F-70B7-4DEB-80AD-9F107B1F692A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8442EBA-6CDD-498F-9338-A74D66361010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>2500944.2400000002</v>
+        <v>2757359.96</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3824973.54</v>
+        <v>3982853.27</v>
       </c>
       <c r="L2">
-        <v>38.79</v>
+        <v>40.39</v>
       </c>
       <c r="M2">
-        <v>147114.37</v>
+        <v>153186.66</v>
       </c>
       <c r="N2">
-        <v>817672.86</v>
+        <v>887830.01</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>1055340.29</v>
       </c>
       <c r="P2">
-        <v>713212.19</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>33184223.309999999</v>
+        <v>36042730.649999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>50752341.530000001</v>
+        <v>52061722.060000002</v>
       </c>
       <c r="L3">
-        <v>105.43</v>
+        <v>108.15</v>
       </c>
       <c r="M3">
-        <v>1952013.14</v>
+        <v>2002373.93</v>
       </c>
       <c r="N3">
-        <v>1661752.97</v>
+        <v>1512158.67</v>
       </c>
       <c r="O3">
-        <v>1754369.5</v>
+        <v>2090207.11</v>
       </c>
       <c r="P3">
-        <v>8236614.79</v>
+        <v>132922.32999999999</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>37024999.93</v>
+        <v>39266268.920000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>56626470.479999997</v>
+        <v>56717944</v>
       </c>
       <c r="L4">
-        <v>43.56</v>
+        <v>43.63</v>
       </c>
       <c r="M4">
-        <v>2177941.17</v>
+        <v>2181459.38</v>
       </c>
       <c r="N4">
-        <v>10330555.560000001</v>
+        <v>11341716.380000001</v>
       </c>
       <c r="O4">
-        <v>1202927.6000000001</v>
+        <v>3623119.97</v>
       </c>
       <c r="P4">
-        <v>-458734.48</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>1481200.04</v>
+        <v>1660961.49</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2265364.77</v>
+        <v>2399166.59</v>
       </c>
       <c r="L5">
-        <v>17.43</v>
+        <v>18.46</v>
       </c>
       <c r="M5">
-        <v>87129.41</v>
+        <v>92275.64</v>
       </c>
       <c r="N5">
-        <v>1279866.6599999999</v>
+        <v>1417379.81</v>
       </c>
       <c r="O5">
-        <v>22654.67</v>
+        <v>21047.61</v>
       </c>
       <c r="P5">
-        <v>125520.9</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,25 +871,25 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>3416043.24</v>
+        <v>3672926.07</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5224536.7300000004</v>
+        <v>5305337.6500000004</v>
       </c>
       <c r="L6">
-        <v>11.48</v>
+        <v>11.66</v>
       </c>
       <c r="M6">
-        <v>200943.72</v>
+        <v>204051.45</v>
       </c>
       <c r="N6">
-        <v>4675995.2</v>
+        <v>5228384.24</v>
       </c>
       <c r="O6">
-        <v>229675.25</v>
+        <v>1013480.34</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>49311566.719999999</v>
+        <v>50012785.409999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>75417690.280000001</v>
+        <v>72240690.030000001</v>
       </c>
       <c r="L7">
-        <v>82.88</v>
+        <v>79.39</v>
       </c>
       <c r="M7">
-        <v>2900680.4</v>
+        <v>2778488.08</v>
       </c>
       <c r="N7">
-        <v>4632048.1399999997</v>
+        <v>5123401.82</v>
       </c>
       <c r="O7">
-        <v>210689.24</v>
+        <v>3609912.4</v>
       </c>
       <c r="P7">
-        <v>804063.74</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>14653913.970000001</v>
+        <v>16080401.720000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>22411868.420000002</v>
+        <v>23227246.920000002</v>
       </c>
       <c r="L8">
-        <v>49.26</v>
+        <v>51.05</v>
       </c>
       <c r="M8">
-        <v>861994.94</v>
+        <v>893355.65</v>
       </c>
       <c r="N8">
-        <v>3427342.89</v>
+        <v>3677449.79</v>
       </c>
       <c r="O8">
-        <v>703807.97</v>
+        <v>1238933.45</v>
       </c>
       <c r="P8">
-        <v>250472.02</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>16.899999999999999</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-24_1713 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8442EBA-6CDD-498F-9338-A74D66361010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82DB6C26-E9F9-471C-8B6B-BCD87395CD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>2757359.96</v>
+        <v>3322704.5</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3982853.27</v>
+        <v>4319515.8600000003</v>
       </c>
       <c r="L2">
-        <v>40.39</v>
+        <v>43.81</v>
       </c>
       <c r="M2">
-        <v>153186.66</v>
+        <v>166135.23000000001</v>
       </c>
       <c r="N2">
-        <v>887830.01</v>
+        <v>1089549.25</v>
       </c>
       <c r="O2">
-        <v>1055340.29</v>
+        <v>14900.13</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>14900.13</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>36042730.649999999</v>
+        <v>39014159.560000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>52061722.060000002</v>
+        <v>50718407.43</v>
       </c>
       <c r="L3">
-        <v>108.15</v>
+        <v>105.36</v>
       </c>
       <c r="M3">
-        <v>2002373.93</v>
+        <v>1950707.98</v>
       </c>
       <c r="N3">
-        <v>1512158.67</v>
+        <v>1520973.41</v>
       </c>
       <c r="O3">
-        <v>2090207.11</v>
+        <v>321498.46000000002</v>
       </c>
       <c r="P3">
-        <v>132922.32999999999</v>
+        <v>226198.35</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>39266268.920000002</v>
+        <v>48487962.509999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>56717944</v>
+        <v>63034351.259999998</v>
       </c>
       <c r="L4">
-        <v>43.63</v>
+        <v>48.49</v>
       </c>
       <c r="M4">
-        <v>2181459.38</v>
+        <v>2424398.13</v>
       </c>
       <c r="N4">
-        <v>11341716.380000001</v>
+        <v>13585339.58</v>
       </c>
       <c r="O4">
-        <v>3623119.97</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>12679.79</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,25 +818,25 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>1660961.49</v>
+        <v>1978469.96</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2399166.59</v>
+        <v>2572010.94</v>
       </c>
       <c r="L5">
-        <v>18.46</v>
+        <v>19.78</v>
       </c>
       <c r="M5">
-        <v>92275.64</v>
+        <v>98923.5</v>
       </c>
       <c r="N5">
-        <v>1417379.81</v>
+        <v>1836921.67</v>
       </c>
       <c r="O5">
-        <v>21047.61</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -871,25 +871,25 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>3672926.07</v>
+        <v>13061989.27</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5305337.6500000004</v>
+        <v>16980586.059999999</v>
       </c>
       <c r="L6">
-        <v>11.66</v>
+        <v>37.32</v>
       </c>
       <c r="M6">
-        <v>204051.45</v>
+        <v>653099.46</v>
       </c>
       <c r="N6">
-        <v>5228384.24</v>
+        <v>5406335.1200000001</v>
       </c>
       <c r="O6">
-        <v>1013480.34</v>
+        <v>0</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>50012785.409999996</v>
+        <v>53988705.560000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>72240690.030000001</v>
+        <v>70185317.230000004</v>
       </c>
       <c r="L7">
-        <v>79.39</v>
+        <v>77.13</v>
       </c>
       <c r="M7">
-        <v>2778488.08</v>
+        <v>2699435.28</v>
       </c>
       <c r="N7">
-        <v>5123401.82</v>
+        <v>6168549.0700000003</v>
       </c>
       <c r="O7">
-        <v>3609912.4</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>-20282.78</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>16080401.720000001</v>
+        <v>24158805.079999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23227246.920000002</v>
+        <v>31406446.600000001</v>
       </c>
       <c r="L8">
-        <v>51.05</v>
+        <v>69.03</v>
       </c>
       <c r="M8">
-        <v>893355.65</v>
+        <v>1207940.25</v>
       </c>
       <c r="N8">
-        <v>3677449.79</v>
+        <v>3556865.82</v>
       </c>
       <c r="O8">
-        <v>1238933.45</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>-78908.490000000005</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.4</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>15.4</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>5.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.6</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-25_1422 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82DB6C26-E9F9-471C-8B6B-BCD87395CD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A34C1CD-AE3E-4EC4-95A6-C219B8BC2B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4319515.8600000003</v>
+        <v>4113824.62</v>
       </c>
       <c r="L2">
-        <v>43.81</v>
+        <v>41.72</v>
       </c>
       <c r="M2">
-        <v>166135.23000000001</v>
+        <v>158224.01999999999</v>
       </c>
       <c r="N2">
-        <v>1089549.25</v>
+        <v>1307459.1000000001</v>
       </c>
       <c r="O2">
-        <v>14900.13</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>14900.13</v>
+        <v>-28742.49</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>39014159.560000002</v>
+        <v>38606606.560000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>50718407.43</v>
+        <v>47798655.75</v>
       </c>
       <c r="L3">
-        <v>105.36</v>
+        <v>99.29</v>
       </c>
       <c r="M3">
-        <v>1950707.98</v>
+        <v>1838409.84</v>
       </c>
       <c r="N3">
-        <v>1520973.41</v>
+        <v>1906678.69</v>
       </c>
       <c r="O3">
-        <v>321498.46000000002</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>226198.35</v>
+        <v>642206.39</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>48487962.509999998</v>
+        <v>48657855.420000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>63034351.259999998</v>
+        <v>60243059.090000004</v>
       </c>
       <c r="L4">
-        <v>48.49</v>
+        <v>46.34</v>
       </c>
       <c r="M4">
-        <v>2424398.13</v>
+        <v>2317040.73</v>
       </c>
       <c r="N4">
-        <v>13585339.58</v>
+        <v>16268428.92</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>8360947.6900000004</v>
       </c>
       <c r="P4">
-        <v>12679.79</v>
+        <v>7204024.8399999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,22 +818,22 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>1978469.96</v>
+        <v>2017367.12</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2572010.94</v>
+        <v>2497692.62</v>
       </c>
       <c r="L5">
-        <v>19.78</v>
+        <v>19.21</v>
       </c>
       <c r="M5">
-        <v>98923.5</v>
+        <v>96065.1</v>
       </c>
       <c r="N5">
-        <v>1836921.67</v>
+        <v>2196526.58</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>16980586.059999999</v>
+        <v>16171986.720000001</v>
       </c>
       <c r="L6">
-        <v>37.32</v>
+        <v>35.54</v>
       </c>
       <c r="M6">
-        <v>653099.46</v>
+        <v>621999.49</v>
       </c>
       <c r="N6">
-        <v>5406335.1200000001</v>
+        <v>6487602.1500000004</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>70164.45</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>81359.12</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>53988705.560000002</v>
+        <v>79180405.859999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>70185317.230000004</v>
+        <v>98032883.450000003</v>
       </c>
       <c r="L7">
-        <v>77.13</v>
+        <v>107.73</v>
       </c>
       <c r="M7">
-        <v>2699435.28</v>
+        <v>3770495.52</v>
       </c>
       <c r="N7">
-        <v>6168549.0700000003</v>
+        <v>2363918.83</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>832948.58</v>
       </c>
       <c r="P7">
-        <v>-20282.78</v>
+        <v>327345.45</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>24158805.079999998</v>
+        <v>29525833.710000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>31406446.600000001</v>
+        <v>36555794.119999997</v>
       </c>
       <c r="L8">
-        <v>69.03</v>
+        <v>80.34</v>
       </c>
       <c r="M8">
-        <v>1207940.25</v>
+        <v>1405992.08</v>
       </c>
       <c r="N8">
-        <v>3556865.82</v>
+        <v>3194833.26</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>1537174.18</v>
       </c>
       <c r="P8">
-        <v>-78908.490000000005</v>
+        <v>120459.8</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>4.4000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2999999999999998</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-27_2125 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A34C1CD-AE3E-4EC4-95A6-C219B8BC2B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F973C58-17EF-45BC-8EE3-BFD703C1D7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3322704.5</v>
+        <v>3761879.89</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4113824.62</v>
+        <v>4445858.05</v>
       </c>
       <c r="L2">
-        <v>41.72</v>
+        <v>45.09</v>
       </c>
       <c r="M2">
-        <v>158224.01999999999</v>
+        <v>170994.54</v>
       </c>
       <c r="N2">
-        <v>1307459.1000000001</v>
+        <v>1524530.03</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>-394674.33</v>
       </c>
       <c r="P2">
-        <v>-28742.49</v>
+        <v>116462.09</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>38606606.560000002</v>
+        <v>39105383.25</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>47798655.75</v>
+        <v>46215452.93</v>
       </c>
       <c r="L3">
-        <v>99.29</v>
+        <v>96</v>
       </c>
       <c r="M3">
-        <v>1838409.84</v>
+        <v>1777517.42</v>
       </c>
       <c r="N3">
-        <v>1906678.69</v>
+        <v>2258654.19</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>1010554.6</v>
       </c>
       <c r="P3">
-        <v>642206.39</v>
+        <v>1987065.72</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>48657855.420000002</v>
+        <v>58370903.590000004</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>60243059.090000004</v>
+        <v>68983795.150000006</v>
       </c>
       <c r="L4">
-        <v>46.34</v>
+        <v>53.06</v>
       </c>
       <c r="M4">
-        <v>2317040.73</v>
+        <v>2653222.89</v>
       </c>
       <c r="N4">
-        <v>16268428.92</v>
+        <v>17907274.100000001</v>
       </c>
       <c r="O4">
-        <v>8360947.6900000004</v>
+        <v>3927221.77</v>
       </c>
       <c r="P4">
-        <v>7204024.8399999999</v>
+        <v>1190360.82</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2017367.12</v>
+        <v>2023862.66</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2497692.62</v>
+        <v>2391837.69</v>
       </c>
       <c r="L5">
-        <v>19.21</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="M5">
-        <v>96065.1</v>
+        <v>91993.76</v>
       </c>
       <c r="N5">
-        <v>2196526.58</v>
+        <v>2744034.33</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>190441.46</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>68163.83</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>13061989.27</v>
+        <v>13934315.300000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>16171986.720000001</v>
+        <v>16467827.17</v>
       </c>
       <c r="L6">
-        <v>35.54</v>
+        <v>36.19</v>
       </c>
       <c r="M6">
-        <v>621999.49</v>
+        <v>633377.97</v>
       </c>
       <c r="N6">
-        <v>6487602.1500000004</v>
+        <v>7891421.1799999997</v>
       </c>
       <c r="O6">
-        <v>70164.45</v>
+        <v>475032.11</v>
       </c>
       <c r="P6">
-        <v>81359.12</v>
+        <v>25660.47</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>79180405.859999999</v>
+        <v>80012146.489999995</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>98032883.450000003</v>
+        <v>94559809.489999995</v>
       </c>
       <c r="L7">
-        <v>107.73</v>
+        <v>103.91</v>
       </c>
       <c r="M7">
-        <v>3770495.52</v>
+        <v>3636915.75</v>
       </c>
       <c r="N7">
-        <v>2363918.83</v>
+        <v>2746963.38</v>
       </c>
       <c r="O7">
-        <v>832948.58</v>
+        <v>18165977.399999999</v>
       </c>
       <c r="P7">
-        <v>327345.45</v>
+        <v>3516082.85</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>29525833.710000001</v>
+        <v>30429511.600000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36555794.119999997</v>
+        <v>35962150.07</v>
       </c>
       <c r="L8">
-        <v>80.34</v>
+        <v>79.040000000000006</v>
       </c>
       <c r="M8">
-        <v>1405992.08</v>
+        <v>1383159.62</v>
       </c>
       <c r="N8">
-        <v>3194833.26</v>
+        <v>3767622.1</v>
       </c>
       <c r="O8">
-        <v>1537174.18</v>
+        <v>2380322</v>
       </c>
       <c r="P8">
-        <v>120459.8</v>
+        <v>230113.29</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>12.7</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>5.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.5</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-28_1957 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F973C58-17EF-45BC-8EE3-BFD703C1D7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F9E7975-F98E-4C5C-A78B-9D9179275FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3761879.89</v>
+        <v>3746979.75</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4445858.05</v>
+        <v>4235716.24</v>
       </c>
       <c r="L2">
-        <v>45.09</v>
+        <v>42.96</v>
       </c>
       <c r="M2">
-        <v>170994.54</v>
+        <v>162912.16</v>
       </c>
       <c r="N2">
-        <v>1524530.03</v>
+        <v>2037673.42</v>
       </c>
       <c r="O2">
-        <v>-394674.33</v>
+        <v>256415.72</v>
       </c>
       <c r="P2">
-        <v>116462.09</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>39105383.25</v>
+        <v>40705987.82</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>46215452.93</v>
+        <v>46015464.490000002</v>
       </c>
       <c r="L3">
-        <v>96</v>
+        <v>95.59</v>
       </c>
       <c r="M3">
-        <v>1777517.42</v>
+        <v>1769825.56</v>
       </c>
       <c r="N3">
-        <v>2258654.19</v>
+        <v>2478004.06</v>
       </c>
       <c r="O3">
-        <v>1010554.6</v>
+        <v>2592173.73</v>
       </c>
       <c r="P3">
-        <v>1987065.72</v>
+        <v>1754369.5</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>58370903.590000004</v>
+        <v>60163514.689999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>68983795.150000006</v>
+        <v>68010929.650000006</v>
       </c>
       <c r="L4">
-        <v>53.06</v>
+        <v>52.32</v>
       </c>
       <c r="M4">
-        <v>2653222.89</v>
+        <v>2615804.9900000002</v>
       </c>
       <c r="N4">
-        <v>17907274.100000001</v>
+        <v>23278828.440000001</v>
       </c>
       <c r="O4">
-        <v>3927221.77</v>
+        <v>2241268.9900000002</v>
       </c>
       <c r="P4">
-        <v>1190360.82</v>
+        <v>1202927.6000000001</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2023862.66</v>
+        <v>2059051.52</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2391837.69</v>
+        <v>2327623.4500000002</v>
       </c>
       <c r="L5">
-        <v>18.399999999999999</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="M5">
-        <v>91993.76</v>
+        <v>89523.98</v>
       </c>
       <c r="N5">
-        <v>2744034.33</v>
+        <v>3646982.83</v>
       </c>
       <c r="O5">
-        <v>190441.46</v>
+        <v>179761.44</v>
       </c>
       <c r="P5">
-        <v>68163.83</v>
+        <v>22654.67</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>13934315.300000001</v>
+        <v>36130442.409999996</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>16467827.17</v>
+        <v>40843108.810000002</v>
       </c>
       <c r="L6">
-        <v>36.19</v>
+        <v>89.77</v>
       </c>
       <c r="M6">
-        <v>633377.97</v>
+        <v>1570888.8</v>
       </c>
       <c r="N6">
-        <v>7891421.1799999997</v>
+        <v>3123185.86</v>
       </c>
       <c r="O6">
-        <v>475032.11</v>
+        <v>256882.82</v>
       </c>
       <c r="P6">
-        <v>25660.47</v>
+        <v>229675.25</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>80012146.489999995</v>
+        <v>87389811.189999998</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>94559809.489999995</v>
+        <v>98788482.219999999</v>
       </c>
       <c r="L7">
-        <v>103.91</v>
+        <v>108.56</v>
       </c>
       <c r="M7">
-        <v>3636915.75</v>
+        <v>3799557.01</v>
       </c>
       <c r="N7">
-        <v>2746963.38</v>
+        <v>1203396.27</v>
       </c>
       <c r="O7">
-        <v>18165977.399999999</v>
+        <v>717048.65</v>
       </c>
       <c r="P7">
-        <v>3516082.85</v>
+        <v>210689.24</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>30429511.600000001</v>
+        <v>36654288.189999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>35962150.07</v>
+        <v>41435282.299999997</v>
       </c>
       <c r="L8">
-        <v>79.040000000000006</v>
+        <v>91.07</v>
       </c>
       <c r="M8">
-        <v>1383159.62</v>
+        <v>1593664.7</v>
       </c>
       <c r="N8">
-        <v>3767622.1</v>
+        <v>2948570.6</v>
       </c>
       <c r="O8">
-        <v>2380322</v>
+        <v>452518.64</v>
       </c>
       <c r="P8">
-        <v>230113.29</v>
+        <v>703807.97</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-29_1833 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F9E7975-F98E-4C5C-A78B-9D9179275FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7B5ECCB-8D03-43C0-AC72-B9B18A4B9998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4235716.24</v>
+        <v>4059228.06</v>
       </c>
       <c r="L2">
-        <v>42.96</v>
+        <v>41.17</v>
       </c>
       <c r="M2">
-        <v>162912.16</v>
+        <v>156124.16</v>
       </c>
       <c r="N2">
-        <v>2037673.42</v>
+        <v>3056510.12</v>
       </c>
       <c r="O2">
-        <v>256415.72</v>
+        <v>565344.55000000005</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>1055340.29</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>40705987.82</v>
+        <v>41018278.039999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>46015464.490000002</v>
+        <v>44436467.880000003</v>
       </c>
       <c r="L3">
-        <v>95.59</v>
+        <v>92.31</v>
       </c>
       <c r="M3">
-        <v>1769825.56</v>
+        <v>1709094.92</v>
       </c>
       <c r="N3">
-        <v>2478004.06</v>
+        <v>3560860.98</v>
       </c>
       <c r="O3">
-        <v>2592173.73</v>
+        <v>1138797.95</v>
       </c>
       <c r="P3">
-        <v>1754369.5</v>
+        <v>1445962.09</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>60163514.689999998</v>
+        <v>61502039.520000003</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>68010929.650000006</v>
+        <v>66627209.469999999</v>
       </c>
       <c r="L4">
-        <v>52.32</v>
+        <v>51.25</v>
       </c>
       <c r="M4">
-        <v>2615804.9900000002</v>
+        <v>2562584.98</v>
       </c>
       <c r="N4">
-        <v>23278828.440000001</v>
+        <v>34248980.240000002</v>
       </c>
       <c r="O4">
-        <v>2241268.9900000002</v>
+        <v>2374567.2999999998</v>
       </c>
       <c r="P4">
-        <v>1202927.6000000001</v>
+        <v>3623119.97</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2059051.52</v>
+        <v>2387856.64</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2327623.4500000002</v>
+        <v>2586844.69</v>
       </c>
       <c r="L5">
-        <v>17.899999999999999</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="M5">
-        <v>89523.98</v>
+        <v>99494.03</v>
       </c>
       <c r="N5">
-        <v>3646982.83</v>
+        <v>5306071.68</v>
       </c>
       <c r="O5">
-        <v>179761.44</v>
+        <v>85473.35</v>
       </c>
       <c r="P5">
-        <v>22654.67</v>
+        <v>21047.61</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>36130442.409999996</v>
+        <v>36675955.259999998</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>40843108.810000002</v>
+        <v>39732284.859999999</v>
       </c>
       <c r="L6">
-        <v>89.77</v>
+        <v>87.32</v>
       </c>
       <c r="M6">
-        <v>1570888.8</v>
+        <v>1528164.8</v>
       </c>
       <c r="N6">
-        <v>3123185.86</v>
+        <v>4412022.37</v>
       </c>
       <c r="O6">
-        <v>256882.82</v>
+        <v>846819.87</v>
       </c>
       <c r="P6">
-        <v>229675.25</v>
+        <v>1013480.34</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>87389811.189999998</v>
+        <v>87458963.450000003</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>98788482.219999999</v>
+        <v>94747210.400000006</v>
       </c>
       <c r="L7">
-        <v>108.56</v>
+        <v>104.12</v>
       </c>
       <c r="M7">
-        <v>3799557.01</v>
+        <v>3644123.48</v>
       </c>
       <c r="N7">
-        <v>1203396.27</v>
+        <v>1770518.28</v>
       </c>
       <c r="O7">
-        <v>717048.65</v>
+        <v>2099915.04</v>
       </c>
       <c r="P7">
-        <v>210689.24</v>
+        <v>3609912.4</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>36654288.189999998</v>
+        <v>47355257.649999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>41435282.299999997</v>
+        <v>51301529.119999997</v>
       </c>
       <c r="L8">
-        <v>91.07</v>
+        <v>112.75</v>
       </c>
       <c r="M8">
-        <v>1593664.7</v>
+        <v>1973135.74</v>
       </c>
       <c r="N8">
-        <v>2948570.6</v>
+        <v>-927628.83</v>
       </c>
       <c r="O8">
-        <v>452518.64</v>
+        <v>1023984.12</v>
       </c>
       <c r="P8">
-        <v>703807.97</v>
+        <v>1238933.45</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-30_1744 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7B5ECCB-8D03-43C0-AC72-B9B18A4B9998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6802FB9-5F22-405B-844D-6593A7526D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3746979.75</v>
+        <v>3284129.5</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4059228.06</v>
+        <v>3415494.68</v>
       </c>
       <c r="L2">
-        <v>41.17</v>
+        <v>34.64</v>
       </c>
       <c r="M2">
-        <v>156124.16</v>
+        <v>131365.18</v>
       </c>
       <c r="N2">
-        <v>3056510.12</v>
+        <v>6575870.5</v>
       </c>
       <c r="O2">
-        <v>565344.55000000005</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>1055340.29</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>41018278.039999999</v>
+        <v>34889805.850000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>44436467.880000003</v>
+        <v>36285398.090000004</v>
       </c>
       <c r="L3">
-        <v>92.31</v>
+        <v>75.37</v>
       </c>
       <c r="M3">
-        <v>1709094.92</v>
+        <v>1395592.23</v>
       </c>
       <c r="N3">
-        <v>3560860.98</v>
+        <v>13250194.15</v>
       </c>
       <c r="O3">
-        <v>1138797.95</v>
+        <v>1868793.06</v>
       </c>
       <c r="P3">
-        <v>1445962.09</v>
+        <v>5885955.6200000001</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>61502039.520000003</v>
+        <v>75508746.939999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>66627209.469999999</v>
+        <v>78529096.819999993</v>
       </c>
       <c r="L4">
-        <v>51.25</v>
+        <v>60.41</v>
       </c>
       <c r="M4">
-        <v>2562584.98</v>
+        <v>3020349.88</v>
       </c>
       <c r="N4">
-        <v>34248980.240000002</v>
+        <v>54491253.060000002</v>
       </c>
       <c r="O4">
-        <v>2374567.2999999998</v>
+        <v>5792792.4000000004</v>
       </c>
       <c r="P4">
-        <v>3623119.97</v>
+        <v>159153.79999999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2387856.64</v>
+        <v>2085266.03</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2586844.69</v>
+        <v>2168676.67</v>
       </c>
       <c r="L5">
-        <v>19.899999999999999</v>
+        <v>16.68</v>
       </c>
       <c r="M5">
-        <v>99494.03</v>
+        <v>83410.64</v>
       </c>
       <c r="N5">
-        <v>5306071.68</v>
+        <v>10914733.970000001</v>
       </c>
       <c r="O5">
-        <v>85473.35</v>
+        <v>191764.56</v>
       </c>
       <c r="P5">
-        <v>21047.61</v>
+        <v>246941.69</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>36675955.259999998</v>
+        <v>30486242.52</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>39732284.859999999</v>
+        <v>31705692.23</v>
       </c>
       <c r="L6">
-        <v>87.32</v>
+        <v>69.680000000000007</v>
       </c>
       <c r="M6">
-        <v>1528164.8</v>
+        <v>1219449.7</v>
       </c>
       <c r="N6">
-        <v>4412022.37</v>
+        <v>15013757.48</v>
       </c>
       <c r="O6">
-        <v>846819.87</v>
+        <v>7054913.7699999996</v>
       </c>
       <c r="P6">
-        <v>1013480.34</v>
+        <v>355395.98</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>87458963.450000003</v>
+        <v>75196706.680000007</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>94747210.400000006</v>
+        <v>78204574.939999998</v>
       </c>
       <c r="L7">
-        <v>104.12</v>
+        <v>85.94</v>
       </c>
       <c r="M7">
-        <v>3644123.48</v>
+        <v>3007868.27</v>
       </c>
       <c r="N7">
-        <v>1770518.28</v>
+        <v>15803293.32</v>
       </c>
       <c r="O7">
-        <v>2099915.04</v>
+        <v>1539905.51</v>
       </c>
       <c r="P7">
-        <v>3609912.4</v>
+        <v>1460203.12</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>47355257.649999999</v>
+        <v>38979685.799999997</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>51301529.119999997</v>
+        <v>40538873.229999997</v>
       </c>
       <c r="L8">
-        <v>112.75</v>
+        <v>89.1</v>
       </c>
       <c r="M8">
-        <v>1973135.74</v>
+        <v>1559187.43</v>
       </c>
       <c r="N8">
-        <v>-927628.83</v>
+        <v>6520314.2000000002</v>
       </c>
       <c r="O8">
-        <v>1023984.12</v>
+        <v>5731585.2699999996</v>
       </c>
       <c r="P8">
-        <v>1238933.45</v>
+        <v>1026512.44</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>11.3</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>4.0999999999999996</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-07-30_1831 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6802FB9-5F22-405B-844D-6593A7526D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F413C2D-C2C8-48D4-8620-C6D2A0BEC95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,22 +659,22 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3284129.5</v>
+        <v>3984667.31</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3415494.68</v>
+        <v>4144054</v>
       </c>
       <c r="L2">
-        <v>34.64</v>
+        <v>42.03</v>
       </c>
       <c r="M2">
-        <v>131365.18</v>
+        <v>159386.69</v>
       </c>
       <c r="N2">
-        <v>6575870.5</v>
+        <v>5875332.6900000004</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>34889805.850000001</v>
+        <v>49029548.439999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>36285398.090000004</v>
+        <v>50990730.380000003</v>
       </c>
       <c r="L3">
-        <v>75.37</v>
+        <v>105.92</v>
       </c>
       <c r="M3">
-        <v>1395592.23</v>
+        <v>1961181.94</v>
       </c>
       <c r="N3">
-        <v>13250194.15</v>
+        <v>-889548.44</v>
       </c>
       <c r="O3">
-        <v>1868793.06</v>
+        <v>2261239.6</v>
       </c>
       <c r="P3">
-        <v>5885955.6200000001</v>
+        <v>7122006.3099999996</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>75508746.939999998</v>
+        <v>91440648.930000007</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>78529096.819999993</v>
+        <v>95098274.890000001</v>
       </c>
       <c r="L4">
-        <v>60.41</v>
+        <v>73.150000000000006</v>
       </c>
       <c r="M4">
-        <v>3020349.88</v>
+        <v>3657625.96</v>
       </c>
       <c r="N4">
-        <v>54491253.060000002</v>
+        <v>38559351.07</v>
       </c>
       <c r="O4">
-        <v>5792792.4000000004</v>
+        <v>7017019.2000000002</v>
       </c>
       <c r="P4">
-        <v>159153.79999999999</v>
+        <v>192576.1</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2085266.03</v>
+        <v>2523171.9</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2168676.67</v>
+        <v>2624098.77</v>
       </c>
       <c r="L5">
-        <v>16.68</v>
+        <v>20.190000000000001</v>
       </c>
       <c r="M5">
-        <v>83410.64</v>
+        <v>100926.88</v>
       </c>
       <c r="N5">
-        <v>10914733.970000001</v>
+        <v>10476828.1</v>
       </c>
       <c r="O5">
-        <v>191764.56</v>
+        <v>232035.12</v>
       </c>
       <c r="P5">
-        <v>246941.69</v>
+        <v>298799.45</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>30486242.52</v>
+        <v>36894151.130000003</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>31705692.23</v>
+        <v>38369917.18</v>
       </c>
       <c r="L6">
-        <v>69.680000000000007</v>
+        <v>84.33</v>
       </c>
       <c r="M6">
-        <v>1219449.7</v>
+        <v>1475766.05</v>
       </c>
       <c r="N6">
-        <v>15013757.48</v>
+        <v>8605848.8699999992</v>
       </c>
       <c r="O6">
-        <v>7054913.7699999996</v>
+        <v>8542243.3300000001</v>
       </c>
       <c r="P6">
-        <v>355395.98</v>
+        <v>430029.14</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>75196706.680000007</v>
+        <v>91050594.319999993</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>78204574.939999998</v>
+        <v>94692618.090000004</v>
       </c>
       <c r="L7">
-        <v>85.94</v>
+        <v>104.06</v>
       </c>
       <c r="M7">
-        <v>3007868.27</v>
+        <v>3642023.77</v>
       </c>
       <c r="N7">
-        <v>15803293.32</v>
+        <v>-50594.32</v>
       </c>
       <c r="O7">
-        <v>1539905.51</v>
+        <v>1876005.11</v>
       </c>
       <c r="P7">
-        <v>1460203.12</v>
+        <v>1770110.6</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>38979685.799999997</v>
+        <v>47549897.07</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>40538873.229999997</v>
+        <v>49451892.960000001</v>
       </c>
       <c r="L8">
-        <v>89.1</v>
+        <v>108.69</v>
       </c>
       <c r="M8">
-        <v>1559187.43</v>
+        <v>1901995.88</v>
       </c>
       <c r="N8">
-        <v>6520314.2000000002</v>
+        <v>-2049897.07</v>
       </c>
       <c r="O8">
-        <v>5731585.2699999996</v>
+        <v>6935218.1799999997</v>
       </c>
       <c r="P8">
-        <v>1026512.44</v>
+        <v>1258722.1299999999</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-07-31_1751 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F413C2D-C2C8-48D4-8620-C6D2A0BEC95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B083E9F-DEA2-4106-816F-4657E255DA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,9 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -659,25 +661,25 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3984667.31</v>
+        <v>3969767.17</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4144054</v>
+        <v>3969767.17</v>
       </c>
       <c r="L2">
-        <v>42.03</v>
+        <v>40.26</v>
       </c>
       <c r="M2">
-        <v>159386.69</v>
+        <v>152683.35</v>
       </c>
       <c r="N2">
-        <v>5875332.6900000004</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>14900.13</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -712,28 +714,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>49029548.439999998</v>
+        <v>49393373</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>50990730.380000003</v>
+        <v>49393373</v>
       </c>
       <c r="L3">
-        <v>105.92</v>
+        <v>102.6</v>
       </c>
       <c r="M3">
-        <v>1961181.94</v>
+        <v>1899745.12</v>
       </c>
       <c r="N3">
-        <v>-889548.44</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>2261239.6</v>
+        <v>74417</v>
       </c>
       <c r="P3">
-        <v>7122006.3099999996</v>
+        <v>321498.46000000002</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>91440648.930000007</v>
+        <v>105794987.53</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>95098274.890000001</v>
+        <v>105794987.53</v>
       </c>
       <c r="L4">
-        <v>73.150000000000006</v>
+        <v>81.38</v>
       </c>
       <c r="M4">
-        <v>3657625.96</v>
+        <v>4069037.98</v>
       </c>
       <c r="N4">
-        <v>38559351.07</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>7017019.2000000002</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>192576.1</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +820,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>2523171.9</v>
+        <v>2703081.01</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2624098.77</v>
+        <v>2703081.01</v>
       </c>
       <c r="L5">
-        <v>20.190000000000001</v>
+        <v>20.79</v>
       </c>
       <c r="M5">
-        <v>100926.88</v>
+        <v>103964.65</v>
       </c>
       <c r="N5">
-        <v>10476828.1</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>232035.12</v>
+        <v>45392.71</v>
       </c>
       <c r="P5">
-        <v>298799.45</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +873,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>36894151.130000003</v>
+        <v>43577506.859999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>38369917.18</v>
+        <v>43577506.859999999</v>
       </c>
       <c r="L6">
-        <v>84.33</v>
+        <v>95.77</v>
       </c>
       <c r="M6">
-        <v>1475766.05</v>
+        <v>1676057.96</v>
       </c>
       <c r="N6">
-        <v>8605848.8699999992</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>8542243.3300000001</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>430029.14</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +926,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>91050594.319999993</v>
+        <v>102650740.70999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>94692618.090000004</v>
+        <v>102650740.70999999</v>
       </c>
       <c r="L7">
-        <v>104.06</v>
+        <v>112.8</v>
       </c>
       <c r="M7">
-        <v>3642023.77</v>
+        <v>3948105.41</v>
       </c>
       <c r="N7">
-        <v>-50594.32</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>1876005.11</v>
+        <v>25191700.300000001</v>
       </c>
       <c r="P7">
-        <v>1770110.6</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,22 +985,22 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>49451892.960000001</v>
+        <v>47549897.07</v>
       </c>
       <c r="L8">
-        <v>108.69</v>
+        <v>104.51</v>
       </c>
       <c r="M8">
-        <v>1901995.88</v>
+        <v>1828842.2</v>
       </c>
       <c r="N8">
-        <v>-2049897.07</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>6935218.1799999997</v>
+        <v>5367028.63</v>
       </c>
       <c r="P8">
-        <v>1258722.1299999999</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1104,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1156,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1182,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>10.6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1208,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1286,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-03_2023 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B083E9F-DEA2-4106-816F-4657E255DA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EC62B8B-3347-443F-8D53-8B9FFA0AA191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="48">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -111,12 +111,21 @@
     <t>GAMBINO NADIA</t>
   </si>
   <si>
+    <t>3RAS MARCAS</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>LUDUEÑA JULIANA</t>
+  </si>
+  <si>
     <t>10</t>
   </si>
   <si>
@@ -127,6 +136,12 @@
   </si>
   <si>
     <t>PEYRONEL ANDREA</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>VERGARA MARIA JOSE</t>
   </si>
   <si>
     <t>SupervisorId</t>
@@ -200,8 +215,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q13">
+  <autoFilter ref="A1:Q13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -564,7 +579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -572,9 +587,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -661,28 +675,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>3969767.17</v>
+        <v>33720.54</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3969767.17</v>
+        <v>438367.05</v>
       </c>
       <c r="L2">
-        <v>40.26</v>
+        <v>4.45</v>
       </c>
       <c r="M2">
-        <v>152683.35</v>
+        <v>16860.27</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>409428.31</v>
       </c>
       <c r="O2">
-        <v>14900.13</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>-394674.33</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,28 +728,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>49393373</v>
+        <v>461764.55</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49393373</v>
+        <v>6002939.0999999996</v>
       </c>
       <c r="L3">
-        <v>102.6</v>
+        <v>12.47</v>
       </c>
       <c r="M3">
-        <v>1899745.12</v>
+        <v>230882.27</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>1986593.14</v>
       </c>
       <c r="O3">
-        <v>74417</v>
+        <v>1588733.49</v>
       </c>
       <c r="P3">
-        <v>321498.46000000002</v>
+        <v>1010554.6</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +781,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>105794987.53</v>
+        <v>3480243.36</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>105794987.53</v>
+        <v>45243163.710000001</v>
       </c>
       <c r="L4">
-        <v>81.38</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="M4">
-        <v>4069037.98</v>
+        <v>1740121.68</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>5271656.53</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>1786614.14</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>3927221.77</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -811,37 +825,37 @@
         <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="H5">
-        <v>13000000</v>
+        <v>6000000</v>
       </c>
       <c r="I5">
-        <v>2703081.01</v>
+        <v>536177.49</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2703081.01</v>
+        <v>6970307.3300000001</v>
       </c>
       <c r="L5">
-        <v>20.79</v>
+        <v>116.17</v>
       </c>
       <c r="M5">
-        <v>103964.65</v>
+        <v>268088.74</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>227659.27</v>
       </c>
       <c r="O5">
-        <v>45392.71</v>
+        <v>95103</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>185990.13</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -855,13 +869,13 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>105004</v>
+        <v>105003</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -870,31 +884,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>45500000</v>
+        <v>13000000</v>
       </c>
       <c r="I6">
-        <v>43577506.859999999</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>43577506.859999999</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>95.77</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>1676057.96</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>541666.67000000004</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>35188.85</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>190441.46</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -908,46 +922,46 @@
         <v>26</v>
       </c>
       <c r="C7">
-        <v>120041</v>
+        <v>105004</v>
       </c>
       <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="H7">
-        <v>91000000</v>
+        <v>6300000</v>
       </c>
       <c r="I7">
-        <v>102650740.70999999</v>
+        <v>488226.57</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>102650740.70999999</v>
+        <v>6346945.3600000003</v>
       </c>
       <c r="L7">
-        <v>112.8</v>
+        <v>100.75</v>
       </c>
       <c r="M7">
-        <v>3948105.41</v>
+        <v>244113.28</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>242157.23</v>
       </c>
       <c r="O7">
-        <v>25191700.300000001</v>
+        <v>241252.22</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>73314.98</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -961,13 +975,13 @@
         <v>26</v>
       </c>
       <c r="C8">
-        <v>105006</v>
+        <v>105004</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
         <v>21</v>
@@ -979,30 +993,295 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>47549897.07</v>
+        <v>437609.08</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>47549897.07</v>
+        <v>5688918.0099999998</v>
       </c>
       <c r="L8">
-        <v>104.51</v>
+        <v>12.5</v>
       </c>
       <c r="M8">
-        <v>1828842.2</v>
+        <v>218804.54</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>1877599.62</v>
       </c>
       <c r="O8">
-        <v>5367028.63</v>
+        <v>22217494.219999999</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>475032.11</v>
       </c>
       <c r="Q8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9">
+        <v>105002</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9">
+        <v>7800000</v>
+      </c>
+      <c r="I9">
+        <v>371092.41</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>4824201.3</v>
+      </c>
+      <c r="L9">
+        <v>61.85</v>
+      </c>
+      <c r="M9">
+        <v>185546.2</v>
+      </c>
+      <c r="N9">
+        <v>309537.82</v>
+      </c>
+      <c r="O9">
+        <v>349662.44</v>
+      </c>
+      <c r="P9">
+        <v>224076.95</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10">
+        <v>120041</v>
+      </c>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10">
+        <v>91000000</v>
+      </c>
+      <c r="I10">
+        <v>2914790.26</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>37892273.409999996</v>
+      </c>
+      <c r="L10">
+        <v>41.64</v>
+      </c>
+      <c r="M10">
+        <v>1457395.13</v>
+      </c>
+      <c r="N10">
+        <v>3670217.07</v>
+      </c>
+      <c r="O10">
+        <v>7377664.7000000002</v>
+      </c>
+      <c r="P10">
+        <v>18165977.399999999</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>105006</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11">
+        <v>7200000</v>
+      </c>
+      <c r="I11">
+        <v>682706.99</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>8875190.8200000003</v>
+      </c>
+      <c r="L11">
+        <v>123.27</v>
+      </c>
+      <c r="M11">
+        <v>341353.49</v>
+      </c>
+      <c r="N11">
+        <v>271553.88</v>
+      </c>
+      <c r="O11">
+        <v>356741.6</v>
+      </c>
+      <c r="P11">
+        <v>402824.54</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12">
+        <v>105006</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12">
+        <v>45500000</v>
+      </c>
+      <c r="I12">
+        <v>1302420.53</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>16931466.940000001</v>
+      </c>
+      <c r="L12">
+        <v>37.21</v>
+      </c>
+      <c r="M12">
+        <v>651210.27</v>
+      </c>
+      <c r="N12">
+        <v>1841565.81</v>
+      </c>
+      <c r="O12">
+        <v>6224776.5899999999</v>
+      </c>
+      <c r="P12">
+        <v>2380322</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13">
+        <v>120008</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13">
+        <v>2700000</v>
+      </c>
+      <c r="I13">
+        <v>54140.22</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>703822.81</v>
+      </c>
+      <c r="L13">
+        <v>26.07</v>
+      </c>
+      <c r="M13">
+        <v>27070.11</v>
+      </c>
+      <c r="N13">
+        <v>110244.16</v>
+      </c>
+      <c r="O13">
+        <v>35566.769999999997</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
         <v>0</v>
       </c>
     </row>
@@ -1031,7 +1310,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1049,10 +1328,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1069,16 +1348,16 @@
         <v>105006</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1095,16 +1374,16 @@
         <v>105004</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1127,10 +1406,10 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H4">
-        <v>2.2000000000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1153,10 +1432,10 @@
         <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H5">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1179,10 +1458,10 @@
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H6">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1205,10 +1484,10 @@
         <v>28</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H7">
-        <v>2.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1225,16 +1504,16 @@
         <v>120041</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H8">
-        <v>1.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1254,13 +1533,13 @@
         <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H9">
-        <v>1.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1280,13 +1559,13 @@
         <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="H10">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-04_2026 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EC62B8B-3347-443F-8D53-8B9FFA0AA191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97848D8C-760F-424B-AFCA-5F8EBED4FD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -111,21 +111,12 @@
     <t>GAMBINO NADIA</t>
   </si>
   <si>
-    <t>3RAS MARCAS</t>
-  </si>
-  <si>
     <t>4</t>
   </si>
   <si>
     <t>GRIBAUDO ANGEL</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>LUDUEÑA JULIANA</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
@@ -136,12 +127,6 @@
   </si>
   <si>
     <t>PEYRONEL ANDREA</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>VERGARA MARIA JOSE</t>
   </si>
   <si>
     <t>SupervisorId</t>
@@ -215,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q13">
-  <autoFilter ref="A1:Q13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -579,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -681,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>438367.05</v>
+        <v>281004.52</v>
       </c>
       <c r="L2">
-        <v>4.45</v>
+        <v>2.85</v>
       </c>
       <c r="M2">
-        <v>16860.27</v>
+        <v>11240.18</v>
       </c>
       <c r="N2">
-        <v>409428.31</v>
+        <v>446649.07</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>-394674.33</v>
+        <v>256415.72</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -728,28 +713,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>461764.55</v>
+        <v>1663101.49</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>6002939.0999999996</v>
+        <v>13859179.050000001</v>
       </c>
       <c r="L3">
-        <v>12.47</v>
+        <v>28.79</v>
       </c>
       <c r="M3">
-        <v>230882.27</v>
+        <v>554367.16</v>
       </c>
       <c r="N3">
-        <v>1986593.14</v>
+        <v>2112586.2999999998</v>
       </c>
       <c r="O3">
-        <v>1588733.49</v>
+        <v>358889.2</v>
       </c>
       <c r="P3">
-        <v>1010554.6</v>
+        <v>2592173.73</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -781,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>3480243.36</v>
+        <v>4677721.93</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>45243163.710000001</v>
+        <v>38981016.07</v>
       </c>
       <c r="L4">
-        <v>34.799999999999997</v>
+        <v>29.99</v>
       </c>
       <c r="M4">
-        <v>1740121.68</v>
+        <v>1559240.64</v>
       </c>
       <c r="N4">
-        <v>5271656.53</v>
+        <v>5696467.1900000004</v>
       </c>
       <c r="O4">
-        <v>1786614.14</v>
+        <v>1344521.79</v>
       </c>
       <c r="P4">
-        <v>3927221.77</v>
+        <v>2241268.9900000002</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,37 +810,37 @@
         <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H5">
-        <v>6000000</v>
+        <v>13000000</v>
       </c>
       <c r="I5">
-        <v>536177.49</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6970307.3300000001</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>116.17</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>268088.74</v>
+        <v>0</v>
       </c>
       <c r="N5">
-        <v>227659.27</v>
+        <v>590909.09</v>
       </c>
       <c r="O5">
-        <v>95103</v>
+        <v>328805.12</v>
       </c>
       <c r="P5">
-        <v>185990.13</v>
+        <v>179761.44</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -869,13 +854,13 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>105003</v>
+        <v>105004</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -884,31 +869,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>13000000</v>
+        <v>45500000</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>475459.38</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>3962161.48</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>8.7100000000000009</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>158486.46</v>
       </c>
       <c r="N6">
-        <v>541666.67000000004</v>
+        <v>2046570.03</v>
       </c>
       <c r="O6">
-        <v>35188.85</v>
+        <v>545512.85</v>
       </c>
       <c r="P6">
-        <v>190441.46</v>
+        <v>256882.82</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -922,46 +907,46 @@
         <v>26</v>
       </c>
       <c r="C7">
-        <v>105004</v>
+        <v>120041</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="H7">
-        <v>6300000</v>
+        <v>91000000</v>
       </c>
       <c r="I7">
-        <v>488226.57</v>
+        <v>4707949.79</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>6346945.3600000003</v>
+        <v>39232914.920000002</v>
       </c>
       <c r="L7">
-        <v>100.75</v>
+        <v>43.11</v>
       </c>
       <c r="M7">
-        <v>244113.28</v>
+        <v>1569316.6</v>
       </c>
       <c r="N7">
-        <v>242157.23</v>
+        <v>3922365.92</v>
       </c>
       <c r="O7">
-        <v>241252.22</v>
+        <v>69152.259999999995</v>
       </c>
       <c r="P7">
-        <v>73314.98</v>
+        <v>717048.65</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -975,13 +960,13 @@
         <v>26</v>
       </c>
       <c r="C8">
-        <v>105004</v>
+        <v>105006</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
         <v>21</v>
@@ -993,295 +978,30 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>437609.08</v>
+        <v>2237272.21</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>5688918.0099999998</v>
+        <v>18643935.109999999</v>
       </c>
       <c r="L8">
-        <v>12.5</v>
+        <v>40.98</v>
       </c>
       <c r="M8">
-        <v>218804.54</v>
+        <v>745757.4</v>
       </c>
       <c r="N8">
-        <v>1877599.62</v>
+        <v>1966487.63</v>
       </c>
       <c r="O8">
-        <v>22217494.219999999</v>
+        <v>10765841.289999999</v>
       </c>
       <c r="P8">
-        <v>475032.11</v>
+        <v>452518.64</v>
       </c>
       <c r="Q8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9">
-        <v>105002</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>35</v>
-      </c>
-      <c r="F9" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9">
-        <v>7800000</v>
-      </c>
-      <c r="I9">
-        <v>371092.41</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>4824201.3</v>
-      </c>
-      <c r="L9">
-        <v>61.85</v>
-      </c>
-      <c r="M9">
-        <v>185546.2</v>
-      </c>
-      <c r="N9">
-        <v>309537.82</v>
-      </c>
-      <c r="O9">
-        <v>349662.44</v>
-      </c>
-      <c r="P9">
-        <v>224076.95</v>
-      </c>
-      <c r="Q9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10">
-        <v>120041</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10">
-        <v>91000000</v>
-      </c>
-      <c r="I10">
-        <v>2914790.26</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>37892273.409999996</v>
-      </c>
-      <c r="L10">
-        <v>41.64</v>
-      </c>
-      <c r="M10">
-        <v>1457395.13</v>
-      </c>
-      <c r="N10">
-        <v>3670217.07</v>
-      </c>
-      <c r="O10">
-        <v>7377664.7000000002</v>
-      </c>
-      <c r="P10">
-        <v>18165977.399999999</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11">
-        <v>105006</v>
-      </c>
-      <c r="D11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11">
-        <v>7200000</v>
-      </c>
-      <c r="I11">
-        <v>682706.99</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <v>8875190.8200000003</v>
-      </c>
-      <c r="L11">
-        <v>123.27</v>
-      </c>
-      <c r="M11">
-        <v>341353.49</v>
-      </c>
-      <c r="N11">
-        <v>271553.88</v>
-      </c>
-      <c r="O11">
-        <v>356741.6</v>
-      </c>
-      <c r="P11">
-        <v>402824.54</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12">
-        <v>105006</v>
-      </c>
-      <c r="D12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12">
-        <v>45500000</v>
-      </c>
-      <c r="I12">
-        <v>1302420.53</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>16931466.940000001</v>
-      </c>
-      <c r="L12">
-        <v>37.21</v>
-      </c>
-      <c r="M12">
-        <v>651210.27</v>
-      </c>
-      <c r="N12">
-        <v>1841565.81</v>
-      </c>
-      <c r="O12">
-        <v>6224776.5899999999</v>
-      </c>
-      <c r="P12">
-        <v>2380322</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13">
-        <v>120008</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" t="s">
-        <v>31</v>
-      </c>
-      <c r="G13" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13">
-        <v>2700000</v>
-      </c>
-      <c r="I13">
-        <v>54140.22</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>703822.81</v>
-      </c>
-      <c r="L13">
-        <v>26.07</v>
-      </c>
-      <c r="M13">
-        <v>27070.11</v>
-      </c>
-      <c r="N13">
-        <v>110244.16</v>
-      </c>
-      <c r="O13">
-        <v>35566.769999999997</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
         <v>0</v>
       </c>
     </row>
@@ -1310,7 +1030,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1328,10 +1048,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1348,13 +1068,13 @@
         <v>105006</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1374,13 +1094,13 @@
         <v>105004</v>
       </c>
       <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
         <v>32</v>
       </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1406,7 +1126,7 @@
         <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -1432,7 +1152,7 @@
         <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1458,7 +1178,7 @@
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1484,7 +1204,7 @@
         <v>28</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1504,13 +1224,13 @@
         <v>120041</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1533,10 +1253,10 @@
         <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1559,10 +1279,10 @@
         <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G10" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H10">
         <v>0</v>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-05_2157 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97848D8C-760F-424B-AFCA-5F8EBED4FD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E0695A8-B020-4856-886A-832B367DDE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>9860000</v>
       </c>
       <c r="I2">
-        <v>33720.54</v>
+        <v>63520.81</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>281004.52</v>
+        <v>397005.06</v>
       </c>
       <c r="L2">
-        <v>2.85</v>
+        <v>4.03</v>
       </c>
       <c r="M2">
-        <v>11240.18</v>
+        <v>15880.2</v>
       </c>
       <c r="N2">
-        <v>446649.07</v>
+        <v>466499.01</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>237687.56</v>
       </c>
       <c r="P2">
-        <v>256415.72</v>
+        <v>565344.55000000005</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>48140000</v>
       </c>
       <c r="I3">
-        <v>1663101.49</v>
+        <v>1996096.77</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>13859179.050000001</v>
+        <v>12475604.82</v>
       </c>
       <c r="L3">
-        <v>28.79</v>
+        <v>25.92</v>
       </c>
       <c r="M3">
-        <v>554367.16</v>
+        <v>499024.19</v>
       </c>
       <c r="N3">
-        <v>2112586.2999999998</v>
+        <v>2197328.73</v>
       </c>
       <c r="O3">
-        <v>358889.2</v>
+        <v>8011270.4000000004</v>
       </c>
       <c r="P3">
-        <v>2592173.73</v>
+        <v>1138797.95</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>4677721.93</v>
+        <v>6675303.1100000003</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>38981016.07</v>
+        <v>41720644.439999998</v>
       </c>
       <c r="L4">
-        <v>29.99</v>
+        <v>32.090000000000003</v>
       </c>
       <c r="M4">
-        <v>1559240.64</v>
+        <v>1668825.78</v>
       </c>
       <c r="N4">
-        <v>5696467.1900000004</v>
+        <v>5872604.6100000003</v>
       </c>
       <c r="O4">
-        <v>1344521.79</v>
+        <v>29938609.420000002</v>
       </c>
       <c r="P4">
-        <v>2241268.9900000002</v>
+        <v>2374567.2999999998</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>13000000</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>93063.61</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>581647.53</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>4.47</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>23265.9</v>
       </c>
       <c r="N5">
-        <v>590909.09</v>
+        <v>614616.02</v>
       </c>
       <c r="O5">
-        <v>328805.12</v>
+        <v>135315.26</v>
       </c>
       <c r="P5">
-        <v>179761.44</v>
+        <v>85473.35</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>45500000</v>
       </c>
       <c r="I6">
-        <v>475459.38</v>
+        <v>562361.39</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3962161.48</v>
+        <v>3514758.66</v>
       </c>
       <c r="L6">
-        <v>8.7100000000000009</v>
+        <v>7.72</v>
       </c>
       <c r="M6">
-        <v>158486.46</v>
+        <v>140590.35</v>
       </c>
       <c r="N6">
-        <v>2046570.03</v>
+        <v>2139887.5499999998</v>
       </c>
       <c r="O6">
-        <v>545512.85</v>
+        <v>277796.40999999997</v>
       </c>
       <c r="P6">
-        <v>256882.82</v>
+        <v>846819.87</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>91000000</v>
       </c>
       <c r="I7">
-        <v>4707949.79</v>
+        <v>4987244.8099999996</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>39232914.920000002</v>
+        <v>31170280.079999998</v>
       </c>
       <c r="L7">
-        <v>43.11</v>
+        <v>34.25</v>
       </c>
       <c r="M7">
-        <v>1569316.6</v>
+        <v>1246811.2</v>
       </c>
       <c r="N7">
-        <v>3922365.92</v>
+        <v>4095845.49</v>
       </c>
       <c r="O7">
-        <v>69152.259999999995</v>
+        <v>5025737.67</v>
       </c>
       <c r="P7">
-        <v>717048.65</v>
+        <v>2099915.04</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>45500000</v>
       </c>
       <c r="I8">
-        <v>2237272.21</v>
+        <v>2614771.27</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>18643935.109999999</v>
+        <v>16342320.42</v>
       </c>
       <c r="L8">
-        <v>40.98</v>
+        <v>35.92</v>
       </c>
       <c r="M8">
-        <v>745757.4</v>
+        <v>653692.81999999995</v>
       </c>
       <c r="N8">
-        <v>1966487.63</v>
+        <v>2042153.75</v>
       </c>
       <c r="O8">
-        <v>10765841.289999999</v>
+        <v>129767.6</v>
       </c>
       <c r="P8">
-        <v>452518.64</v>
+        <v>1023984.12</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-06_2058 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E0695A8-B020-4856-886A-832B367DDE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BD88F17-1CBA-4082-83EF-76629E69D24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -657,31 +657,31 @@
         <v>22</v>
       </c>
       <c r="H2">
-        <v>9860000</v>
+        <v>6500000</v>
       </c>
       <c r="I2">
-        <v>63520.81</v>
+        <v>468727.96</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>397005.06</v>
+        <v>2343639.7799999998</v>
       </c>
       <c r="L2">
-        <v>4.03</v>
+        <v>36.06</v>
       </c>
       <c r="M2">
-        <v>15880.2</v>
+        <v>93745.59</v>
       </c>
       <c r="N2">
-        <v>466499.01</v>
+        <v>301563.59999999998</v>
       </c>
       <c r="O2">
-        <v>237687.56</v>
+        <v>-14900.13</v>
       </c>
       <c r="P2">
-        <v>565344.55000000005</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -710,31 +710,31 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>48140000</v>
+        <v>58500000</v>
       </c>
       <c r="I3">
-        <v>1996096.77</v>
+        <v>3206464.92</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>12475604.82</v>
+        <v>16032324.619999999</v>
       </c>
       <c r="L3">
-        <v>25.92</v>
+        <v>27.41</v>
       </c>
       <c r="M3">
-        <v>499024.19</v>
+        <v>641292.98</v>
       </c>
       <c r="N3">
-        <v>2197328.73</v>
+        <v>2764676.75</v>
       </c>
       <c r="O3">
-        <v>8011270.4000000004</v>
+        <v>897345.98</v>
       </c>
       <c r="P3">
-        <v>1138797.95</v>
+        <v>2261239.6</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -763,31 +763,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>130000000</v>
+        <v>117000000</v>
       </c>
       <c r="I4">
-        <v>6675303.1100000003</v>
+        <v>7555451.7300000004</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>41720644.439999998</v>
+        <v>37777258.630000003</v>
       </c>
       <c r="L4">
-        <v>32.090000000000003</v>
+        <v>32.29</v>
       </c>
       <c r="M4">
-        <v>1668825.78</v>
+        <v>1511090.35</v>
       </c>
       <c r="N4">
-        <v>5872604.6100000003</v>
+        <v>5472227.4100000001</v>
       </c>
       <c r="O4">
-        <v>29938609.420000002</v>
+        <v>14730910.1</v>
       </c>
       <c r="P4">
-        <v>2374567.2999999998</v>
+        <v>7017019.2000000002</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -816,31 +816,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>13000000</v>
+        <v>3250000</v>
       </c>
       <c r="I5">
-        <v>93063.61</v>
+        <v>157389.93</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>581647.53</v>
+        <v>786949.67</v>
       </c>
       <c r="L5">
-        <v>4.47</v>
+        <v>24.21</v>
       </c>
       <c r="M5">
-        <v>23265.9</v>
+        <v>31477.99</v>
       </c>
       <c r="N5">
-        <v>614616.02</v>
+        <v>154630.5</v>
       </c>
       <c r="O5">
-        <v>135315.26</v>
+        <v>179909.12</v>
       </c>
       <c r="P5">
-        <v>85473.35</v>
+        <v>232035.12</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -869,31 +869,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>45500000</v>
+        <v>48750000</v>
       </c>
       <c r="I6">
-        <v>562361.39</v>
+        <v>836560.44</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3514758.66</v>
+        <v>4182802.21</v>
       </c>
       <c r="L6">
-        <v>7.72</v>
+        <v>8.58</v>
       </c>
       <c r="M6">
-        <v>140590.35</v>
+        <v>167312.09</v>
       </c>
       <c r="N6">
-        <v>2139887.5499999998</v>
+        <v>2395671.98</v>
       </c>
       <c r="O6">
-        <v>277796.40999999997</v>
+        <v>7046464.1299999999</v>
       </c>
       <c r="P6">
-        <v>846819.87</v>
+        <v>8542243.3300000001</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -922,31 +922,31 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>91000000</v>
+        <v>107250000</v>
       </c>
       <c r="I7">
-        <v>4987244.8099999996</v>
+        <v>5641231.7300000004</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>31170280.079999998</v>
+        <v>28206158.66</v>
       </c>
       <c r="L7">
-        <v>34.25</v>
+        <v>26.3</v>
       </c>
       <c r="M7">
-        <v>1246811.2</v>
+        <v>1128246.3500000001</v>
       </c>
       <c r="N7">
-        <v>4095845.49</v>
+        <v>5080438.41</v>
       </c>
       <c r="O7">
-        <v>5025737.67</v>
+        <v>12632251.619999999</v>
       </c>
       <c r="P7">
-        <v>2099915.04</v>
+        <v>1876005.11</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -975,31 +975,31 @@
         <v>22</v>
       </c>
       <c r="H8">
-        <v>45500000</v>
+        <v>48750000</v>
       </c>
       <c r="I8">
-        <v>2614771.27</v>
+        <v>3302621.44</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>16342320.42</v>
+        <v>16513107.199999999</v>
       </c>
       <c r="L8">
-        <v>35.92</v>
+        <v>33.869999999999997</v>
       </c>
       <c r="M8">
-        <v>653692.81999999995</v>
+        <v>660524.29</v>
       </c>
       <c r="N8">
-        <v>2042153.75</v>
+        <v>2272368.9300000002</v>
       </c>
       <c r="O8">
-        <v>129767.6</v>
+        <v>693863.67</v>
       </c>
       <c r="P8">
-        <v>1023984.12</v>
+        <v>6935218.1799999997</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-08_2049 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BD88F17-1CBA-4082-83EF-76629E69D24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B8A874A-2E53-482B-B0F8-5EC753FFC9DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>468727.96</v>
+        <v>730863.96</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2343639.7799999998</v>
+        <v>2714637.58</v>
       </c>
       <c r="L2">
-        <v>36.06</v>
+        <v>41.76</v>
       </c>
       <c r="M2">
-        <v>93745.59</v>
+        <v>104409.14</v>
       </c>
       <c r="N2">
-        <v>301563.59999999998</v>
+        <v>303638.74</v>
       </c>
       <c r="O2">
-        <v>-14900.13</v>
+        <v>33720.54</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>424275.25</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>3206464.92</v>
+        <v>7682123.1500000004</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>16032324.619999999</v>
+        <v>28533600.260000002</v>
       </c>
       <c r="L3">
-        <v>27.41</v>
+        <v>48.78</v>
       </c>
       <c r="M3">
-        <v>641292.98</v>
+        <v>1097446.1599999999</v>
       </c>
       <c r="N3">
-        <v>2764676.75</v>
+        <v>2674625.1</v>
       </c>
       <c r="O3">
-        <v>897345.98</v>
+        <v>49288.92</v>
       </c>
       <c r="P3">
-        <v>2261239.6</v>
+        <v>464048.79</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>7555451.7300000004</v>
+        <v>7630655.4000000004</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>37777258.630000003</v>
+        <v>28342434.34</v>
       </c>
       <c r="L4">
-        <v>32.29</v>
+        <v>24.22</v>
       </c>
       <c r="M4">
-        <v>1511090.35</v>
+        <v>1090093.6299999999</v>
       </c>
       <c r="N4">
-        <v>5472227.4100000001</v>
+        <v>5756281.29</v>
       </c>
       <c r="O4">
-        <v>14730910.1</v>
+        <v>3103671.85</v>
       </c>
       <c r="P4">
-        <v>7017019.2000000002</v>
+        <v>9713048.1600000001</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>157389.93</v>
+        <v>373126.43</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>786949.67</v>
+        <v>1385898.16</v>
       </c>
       <c r="L5">
-        <v>24.21</v>
+        <v>42.64</v>
       </c>
       <c r="M5">
-        <v>31477.99</v>
+        <v>53303.78</v>
       </c>
       <c r="N5">
-        <v>154630.5</v>
+        <v>151414.39999999999</v>
       </c>
       <c r="O5">
-        <v>179909.12</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>232035.12</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>836560.44</v>
+        <v>1034894.2</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4182802.21</v>
+        <v>3843892.73</v>
       </c>
       <c r="L6">
-        <v>8.58</v>
+        <v>7.88</v>
       </c>
       <c r="M6">
-        <v>167312.09</v>
+        <v>147842.03</v>
       </c>
       <c r="N6">
-        <v>2395671.98</v>
+        <v>2511321.36</v>
       </c>
       <c r="O6">
-        <v>7046464.1299999999</v>
+        <v>14900.13</v>
       </c>
       <c r="P6">
-        <v>8542243.3300000001</v>
+        <v>850958.91</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>5641231.7300000004</v>
+        <v>7476805.7000000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>28206158.66</v>
+        <v>27770992.600000001</v>
       </c>
       <c r="L7">
-        <v>26.3</v>
+        <v>25.89</v>
       </c>
       <c r="M7">
-        <v>1128246.3500000001</v>
+        <v>1068115.1000000001</v>
       </c>
       <c r="N7">
-        <v>5080438.41</v>
+        <v>5251220.75</v>
       </c>
       <c r="O7">
-        <v>12632251.619999999</v>
+        <v>448578.24</v>
       </c>
       <c r="P7">
-        <v>1876005.11</v>
+        <v>831740.63</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>3302621.44</v>
+        <v>3723279.82</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>16513107.199999999</v>
+        <v>13829325.039999999</v>
       </c>
       <c r="L8">
-        <v>33.869999999999997</v>
+        <v>28.37</v>
       </c>
       <c r="M8">
-        <v>660524.29</v>
+        <v>531897.12</v>
       </c>
       <c r="N8">
-        <v>2272368.9300000002</v>
+        <v>2369827.38</v>
       </c>
       <c r="O8">
-        <v>693863.67</v>
+        <v>543685.03</v>
       </c>
       <c r="P8">
-        <v>6935218.1799999997</v>
+        <v>903677.88</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.3</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-10_1713 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B8A874A-2E53-482B-B0F8-5EC753FFC9DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDD4F8E3-7380-4142-AFD9-B5BEB9113E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -660,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>730863.96</v>
+        <v>812391.15</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2714637.58</v>
+        <v>2538722.33</v>
       </c>
       <c r="L2">
-        <v>41.76</v>
+        <v>39.06</v>
       </c>
       <c r="M2">
-        <v>104409.14</v>
+        <v>101548.89</v>
       </c>
       <c r="N2">
-        <v>303638.74</v>
+        <v>334565.23</v>
       </c>
       <c r="O2">
-        <v>33720.54</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>424275.25</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>7682123.1500000004</v>
+        <v>7968879.8499999996</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>28533600.260000002</v>
+        <v>24902749.52</v>
       </c>
       <c r="L3">
-        <v>48.78</v>
+        <v>42.57</v>
       </c>
       <c r="M3">
-        <v>1097446.1599999999</v>
+        <v>996109.98</v>
       </c>
       <c r="N3">
-        <v>2674625.1</v>
+        <v>2972418.83</v>
       </c>
       <c r="O3">
-        <v>49288.92</v>
+        <v>1251447.3500000001</v>
       </c>
       <c r="P3">
-        <v>464048.79</v>
+        <v>1588733.49</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>7630655.4000000004</v>
+        <v>14894643.66</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>28342434.34</v>
+        <v>46545761.450000003</v>
       </c>
       <c r="L4">
-        <v>24.22</v>
+        <v>39.78</v>
       </c>
       <c r="M4">
-        <v>1090093.6299999999</v>
+        <v>1861830.46</v>
       </c>
       <c r="N4">
-        <v>5756281.29</v>
+        <v>6006197.4299999997</v>
       </c>
       <c r="O4">
-        <v>3103671.85</v>
+        <v>1197478.57</v>
       </c>
       <c r="P4">
-        <v>9713048.1600000001</v>
+        <v>1786614.14</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1385898.16</v>
+        <v>1166020.0900000001</v>
       </c>
       <c r="L5">
-        <v>42.64</v>
+        <v>35.880000000000003</v>
       </c>
       <c r="M5">
-        <v>53303.78</v>
+        <v>46640.800000000003</v>
       </c>
       <c r="N5">
-        <v>151414.39999999999</v>
+        <v>169227.86</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>35188.85</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>1034894.2</v>
+        <v>1210333.6000000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3843892.73</v>
+        <v>3782292.51</v>
       </c>
       <c r="L6">
-        <v>7.88</v>
+        <v>7.76</v>
       </c>
       <c r="M6">
-        <v>147842.03</v>
+        <v>151291.70000000001</v>
       </c>
       <c r="N6">
-        <v>2511321.36</v>
+        <v>2796450.96</v>
       </c>
       <c r="O6">
-        <v>14900.13</v>
+        <v>37850.300000000003</v>
       </c>
       <c r="P6">
-        <v>850958.91</v>
+        <v>22217494.219999999</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>7476805.7000000002</v>
+        <v>8072911.9800000004</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>27770992.600000001</v>
+        <v>25227849.949999999</v>
       </c>
       <c r="L7">
-        <v>25.89</v>
+        <v>23.52</v>
       </c>
       <c r="M7">
-        <v>1068115.1000000001</v>
+        <v>1009114</v>
       </c>
       <c r="N7">
-        <v>5251220.75</v>
+        <v>5833946.3499999996</v>
       </c>
       <c r="O7">
-        <v>448578.24</v>
+        <v>1793159.53</v>
       </c>
       <c r="P7">
-        <v>831740.63</v>
+        <v>7377664.7000000002</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>3723279.82</v>
+        <v>7011542.3700000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>13829325.039999999</v>
+        <v>21911069.91</v>
       </c>
       <c r="L8">
-        <v>28.37</v>
+        <v>44.95</v>
       </c>
       <c r="M8">
-        <v>531897.12</v>
+        <v>876442.8</v>
       </c>
       <c r="N8">
-        <v>2369827.38</v>
+        <v>2455203.39</v>
       </c>
       <c r="O8">
-        <v>543685.03</v>
+        <v>934851.68</v>
       </c>
       <c r="P8">
-        <v>903677.88</v>
+        <v>6224776.5899999999</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>5.6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-11_1741 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDD4F8E3-7380-4142-AFD9-B5BEB9113E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CA3F435-7424-468A-BEF1-CB274EE46555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,7 +201,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="3RAS MARCAS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -572,7 +578,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -633,7 +640,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -659,25 +666,25 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>812391.15</v>
+        <v>4296544.54</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2538722.33</v>
+        <v>11934845.939999999</v>
       </c>
       <c r="L2">
-        <v>39.06</v>
+        <v>183.61</v>
       </c>
       <c r="M2">
-        <v>101548.89</v>
+        <v>477393.84</v>
       </c>
       <c r="N2">
-        <v>334565.23</v>
+        <v>137715.97</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>29800.27</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -686,7 +693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -712,34 +719,34 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>7968879.8499999996</v>
+        <v>8674882.8900000006</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>24902749.52</v>
+        <v>24096896.93</v>
       </c>
       <c r="L3">
-        <v>42.57</v>
+        <v>41.19</v>
       </c>
       <c r="M3">
-        <v>996109.98</v>
+        <v>963875.88</v>
       </c>
       <c r="N3">
-        <v>2972418.83</v>
+        <v>3114069.82</v>
       </c>
       <c r="O3">
-        <v>1251447.3500000001</v>
+        <v>303859.36</v>
       </c>
       <c r="P3">
-        <v>1588733.49</v>
+        <v>358889.2</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -765,34 +772,34 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>14894643.66</v>
+        <v>16186593.300000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>46545761.450000003</v>
+        <v>44962759.159999996</v>
       </c>
       <c r="L4">
-        <v>39.78</v>
+        <v>38.43</v>
       </c>
       <c r="M4">
-        <v>1861830.46</v>
+        <v>1798510.37</v>
       </c>
       <c r="N4">
-        <v>6006197.4299999997</v>
+        <v>6300837.9199999999</v>
       </c>
       <c r="O4">
-        <v>1197478.57</v>
+        <v>1997581.18</v>
       </c>
       <c r="P4">
-        <v>1786614.14</v>
+        <v>1344521.79</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -824,28 +831,28 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1166020.0900000001</v>
+        <v>1036462.3</v>
       </c>
       <c r="L5">
-        <v>35.880000000000003</v>
+        <v>31.89</v>
       </c>
       <c r="M5">
-        <v>46640.800000000003</v>
+        <v>41458.49</v>
       </c>
       <c r="N5">
-        <v>169227.86</v>
+        <v>179804.6</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>93063.61</v>
       </c>
       <c r="P5">
-        <v>35188.85</v>
+        <v>328805.12</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -871,34 +878,34 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>1210333.6000000001</v>
+        <v>1630568.93</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3782292.51</v>
+        <v>4529358.1399999997</v>
       </c>
       <c r="L6">
-        <v>7.76</v>
+        <v>9.2899999999999991</v>
       </c>
       <c r="M6">
-        <v>151291.70000000001</v>
+        <v>181174.33</v>
       </c>
       <c r="N6">
-        <v>2796450.96</v>
+        <v>2944964.44</v>
       </c>
       <c r="O6">
-        <v>37850.300000000003</v>
+        <v>86902.01</v>
       </c>
       <c r="P6">
-        <v>22217494.219999999</v>
+        <v>545512.85</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -924,34 +931,34 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>8072911.9800000004</v>
+        <v>9279635.3399999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25227849.949999999</v>
+        <v>25776764.84</v>
       </c>
       <c r="L7">
-        <v>23.52</v>
+        <v>24.03</v>
       </c>
       <c r="M7">
-        <v>1009114</v>
+        <v>1031070.59</v>
       </c>
       <c r="N7">
-        <v>5833946.3499999996</v>
+        <v>6123147.79</v>
       </c>
       <c r="O7">
-        <v>1793159.53</v>
+        <v>279295.02</v>
       </c>
       <c r="P7">
-        <v>7377664.7000000002</v>
+        <v>69152.259999999995</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -977,28 +984,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>7011542.3700000001</v>
+        <v>7356289.0700000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>21911069.91</v>
+        <v>20434136.300000001</v>
       </c>
       <c r="L8">
-        <v>44.95</v>
+        <v>41.92</v>
       </c>
       <c r="M8">
-        <v>876442.8</v>
+        <v>817365.45</v>
       </c>
       <c r="N8">
-        <v>2455203.39</v>
+        <v>2587106.9300000002</v>
       </c>
       <c r="O8">
-        <v>934851.68</v>
+        <v>377499.05</v>
       </c>
       <c r="P8">
-        <v>6224776.5899999999</v>
+        <v>10765841.289999999</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1128,7 +1135,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1213,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1239,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1265,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-12_1746 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CA3F435-7424-468A-BEF1-CB274EE46555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65200830-3060-4186-9A84-F784430A1B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,13 +201,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="3RAS MARCAS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -578,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -640,7 +633,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -672,28 +665,28 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>11934845.939999999</v>
+        <v>10741361.35</v>
       </c>
       <c r="L2">
-        <v>183.61</v>
+        <v>165.25</v>
       </c>
       <c r="M2">
-        <v>477393.84</v>
+        <v>429654.45</v>
       </c>
       <c r="N2">
-        <v>137715.97</v>
+        <v>146897.03</v>
       </c>
       <c r="O2">
-        <v>29800.27</v>
+        <v>405207.15</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>237687.56</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -719,34 +712,34 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>8674882.8900000006</v>
+        <v>8886973.1699999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>24096896.93</v>
+        <v>22217432.920000002</v>
       </c>
       <c r="L3">
-        <v>41.19</v>
+        <v>37.979999999999997</v>
       </c>
       <c r="M3">
-        <v>963875.88</v>
+        <v>888697.32</v>
       </c>
       <c r="N3">
-        <v>3114069.82</v>
+        <v>3307535.12</v>
       </c>
       <c r="O3">
-        <v>303859.36</v>
+        <v>1146277.48</v>
       </c>
       <c r="P3">
-        <v>358889.2</v>
+        <v>8011270.4000000004</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -772,34 +765,34 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>16186593.300000001</v>
+        <v>16999678.370000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>44962759.159999996</v>
+        <v>42499195.920000002</v>
       </c>
       <c r="L4">
-        <v>38.43</v>
+        <v>36.32</v>
       </c>
       <c r="M4">
-        <v>1798510.37</v>
+        <v>1699967.84</v>
       </c>
       <c r="N4">
-        <v>6300837.9199999999</v>
+        <v>6666688.1100000003</v>
       </c>
       <c r="O4">
-        <v>1997581.18</v>
+        <v>880148.62</v>
       </c>
       <c r="P4">
-        <v>1344521.79</v>
+        <v>29938609.420000002</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -825,34 +818,34 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>373126.43</v>
+        <v>388473.56</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1036462.3</v>
+        <v>971183.9</v>
       </c>
       <c r="L5">
-        <v>31.89</v>
+        <v>29.88</v>
       </c>
       <c r="M5">
-        <v>41458.49</v>
+        <v>38847.360000000001</v>
       </c>
       <c r="N5">
-        <v>179804.6</v>
+        <v>190768.43</v>
       </c>
       <c r="O5">
-        <v>93063.61</v>
+        <v>64326.33</v>
       </c>
       <c r="P5">
-        <v>328805.12</v>
+        <v>135315.26</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -878,34 +871,34 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>1630568.93</v>
+        <v>2011511.4</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4529358.1399999997</v>
+        <v>5028778.51</v>
       </c>
       <c r="L6">
-        <v>9.2899999999999991</v>
+        <v>10.32</v>
       </c>
       <c r="M6">
-        <v>181174.33</v>
+        <v>201151.14</v>
       </c>
       <c r="N6">
-        <v>2944964.44</v>
+        <v>3115899.24</v>
       </c>
       <c r="O6">
-        <v>86902.01</v>
+        <v>274199.06</v>
       </c>
       <c r="P6">
-        <v>545512.85</v>
+        <v>277796.40999999997</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -931,34 +924,34 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>9279635.3399999999</v>
+        <v>9348043.7400000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25776764.84</v>
+        <v>23370109.350000001</v>
       </c>
       <c r="L7">
-        <v>24.03</v>
+        <v>21.79</v>
       </c>
       <c r="M7">
-        <v>1031070.59</v>
+        <v>934804.37</v>
       </c>
       <c r="N7">
-        <v>6123147.79</v>
+        <v>6526797.0800000001</v>
       </c>
       <c r="O7">
-        <v>279295.02</v>
+        <v>653986.92000000004</v>
       </c>
       <c r="P7">
-        <v>69152.259999999995</v>
+        <v>5025737.67</v>
       </c>
       <c r="Q7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -984,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>7356289.0700000003</v>
+        <v>7704276.3300000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20434136.300000001</v>
+        <v>19260690.829999998</v>
       </c>
       <c r="L8">
-        <v>41.92</v>
+        <v>39.51</v>
       </c>
       <c r="M8">
-        <v>817365.45</v>
+        <v>770427.63</v>
       </c>
       <c r="N8">
-        <v>2587106.9300000002</v>
+        <v>2736381.58</v>
       </c>
       <c r="O8">
-        <v>377499.05</v>
+        <v>685366.82</v>
       </c>
       <c r="P8">
-        <v>10765841.289999999</v>
+        <v>129767.6</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1083,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1109,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1213,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1239,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1265,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-13_2112 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65200830-3060-4186-9A84-F784430A1B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB658E86-A871-47D0-B34D-5E802B81356F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>4296544.54</v>
+        <v>4521327.6500000004</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>10741361.35</v>
+        <v>10275744.65</v>
       </c>
       <c r="L2">
-        <v>165.25</v>
+        <v>158.09</v>
       </c>
       <c r="M2">
-        <v>429654.45</v>
+        <v>411029.79</v>
       </c>
       <c r="N2">
-        <v>146897.03</v>
+        <v>141333.74</v>
       </c>
       <c r="O2">
-        <v>405207.15</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>237687.56</v>
+        <v>-14900.13</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>8886973.1699999999</v>
+        <v>9912558.5399999991</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>22217432.920000002</v>
+        <v>22528542.140000001</v>
       </c>
       <c r="L3">
-        <v>37.979999999999997</v>
+        <v>38.51</v>
       </c>
       <c r="M3">
-        <v>888697.32</v>
+        <v>901141.69</v>
       </c>
       <c r="N3">
-        <v>3307535.12</v>
+        <v>3470531.53</v>
       </c>
       <c r="O3">
-        <v>1146277.48</v>
+        <v>4586483.28</v>
       </c>
       <c r="P3">
-        <v>8011270.4000000004</v>
+        <v>897345.98</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>16999678.370000001</v>
+        <v>14434816.08</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>42499195.920000002</v>
+        <v>32806400.170000002</v>
       </c>
       <c r="L4">
-        <v>36.32</v>
+        <v>28.04</v>
       </c>
       <c r="M4">
-        <v>1699967.84</v>
+        <v>1312256.01</v>
       </c>
       <c r="N4">
-        <v>6666688.1100000003</v>
+        <v>7326084.5700000003</v>
       </c>
       <c r="O4">
-        <v>880148.62</v>
+        <v>127759.73</v>
       </c>
       <c r="P4">
-        <v>29938609.420000002</v>
+        <v>14730910.1</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>388473.56</v>
+        <v>928741.61</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>971183.9</v>
+        <v>2110776.39</v>
       </c>
       <c r="L5">
-        <v>29.88</v>
+        <v>64.95</v>
       </c>
       <c r="M5">
-        <v>38847.360000000001</v>
+        <v>84431.06</v>
       </c>
       <c r="N5">
-        <v>190768.43</v>
+        <v>165804.17000000001</v>
       </c>
       <c r="O5">
-        <v>64326.33</v>
+        <v>215736.49</v>
       </c>
       <c r="P5">
-        <v>135315.26</v>
+        <v>179909.12</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>2011511.4</v>
+        <v>1994506.38</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>5028778.51</v>
+        <v>4532969.04</v>
       </c>
       <c r="L6">
-        <v>10.32</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="M6">
-        <v>201151.14</v>
+        <v>181318.76</v>
       </c>
       <c r="N6">
-        <v>3115899.24</v>
+        <v>3339678.12</v>
       </c>
       <c r="O6">
-        <v>274199.06</v>
+        <v>198333.75</v>
       </c>
       <c r="P6">
-        <v>277796.40999999997</v>
+        <v>7046464.1299999999</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>9348043.7400000002</v>
+        <v>16404322.060000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>23370109.350000001</v>
+        <v>37282550.140000001</v>
       </c>
       <c r="L7">
-        <v>21.79</v>
+        <v>34.76</v>
       </c>
       <c r="M7">
-        <v>934804.37</v>
+        <v>1491302.01</v>
       </c>
       <c r="N7">
-        <v>6526797.0800000001</v>
+        <v>6488977</v>
       </c>
       <c r="O7">
-        <v>653986.92000000004</v>
+        <v>2217958.38</v>
       </c>
       <c r="P7">
-        <v>5025737.67</v>
+        <v>12632251.619999999</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>7704276.3300000001</v>
+        <v>8302730.5199999996</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>19260690.829999998</v>
+        <v>18869842.09</v>
       </c>
       <c r="L8">
-        <v>39.51</v>
+        <v>38.71</v>
       </c>
       <c r="M8">
-        <v>770427.63</v>
+        <v>754793.68</v>
       </c>
       <c r="N8">
-        <v>2736381.58</v>
+        <v>2889090.68</v>
       </c>
       <c r="O8">
-        <v>685366.82</v>
+        <v>423141.73</v>
       </c>
       <c r="P8">
-        <v>129767.6</v>
+        <v>693863.67</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>4.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-14_1749 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB658E86-A871-47D0-B34D-5E802B81356F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{33869295-2D3B-4E57-982E-F5754F276064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>4521327.6500000004</v>
+        <v>4395230.93</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>10275744.65</v>
+        <v>9156731.0999999996</v>
       </c>
       <c r="L2">
-        <v>158.09</v>
+        <v>140.87</v>
       </c>
       <c r="M2">
-        <v>411029.79</v>
+        <v>366269.24</v>
       </c>
       <c r="N2">
-        <v>141333.74</v>
+        <v>161905.31</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>262136.01</v>
       </c>
       <c r="P2">
-        <v>-14900.13</v>
+        <v>-186387.74</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>9912558.5399999991</v>
+        <v>10562434.369999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>22528542.140000001</v>
+        <v>22005071.609999999</v>
       </c>
       <c r="L3">
-        <v>38.51</v>
+        <v>37.619999999999997</v>
       </c>
       <c r="M3">
-        <v>901141.69</v>
+        <v>880202.86</v>
       </c>
       <c r="N3">
-        <v>3470531.53</v>
+        <v>3687505.05</v>
       </c>
       <c r="O3">
-        <v>4586483.28</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>897345.98</v>
+        <v>213763.74</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>14434816.08</v>
+        <v>28281532.170000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>32806400.170000002</v>
+        <v>58919858.689999998</v>
       </c>
       <c r="L4">
-        <v>28.04</v>
+        <v>50.36</v>
       </c>
       <c r="M4">
-        <v>1312256.01</v>
+        <v>2356794.35</v>
       </c>
       <c r="N4">
-        <v>7326084.5700000003</v>
+        <v>6824497.5300000003</v>
       </c>
       <c r="O4">
-        <v>127759.73</v>
+        <v>-52556.05</v>
       </c>
       <c r="P4">
-        <v>14730910.1</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2110776.39</v>
+        <v>1934878.36</v>
       </c>
       <c r="L5">
-        <v>64.95</v>
+        <v>59.53</v>
       </c>
       <c r="M5">
-        <v>84431.06</v>
+        <v>77395.13</v>
       </c>
       <c r="N5">
-        <v>165804.17000000001</v>
+        <v>178558.34</v>
       </c>
       <c r="O5">
-        <v>215736.49</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>179909.12</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>1994506.38</v>
+        <v>2524103.14</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4532969.04</v>
+        <v>5258548.21</v>
       </c>
       <c r="L6">
-        <v>9.3000000000000007</v>
+        <v>10.79</v>
       </c>
       <c r="M6">
-        <v>181318.76</v>
+        <v>210341.93</v>
       </c>
       <c r="N6">
-        <v>3339678.12</v>
+        <v>3555838.22</v>
       </c>
       <c r="O6">
-        <v>198333.75</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>7046464.1299999999</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>16404322.060000001</v>
+        <v>17252698.440000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>37282550.140000001</v>
+        <v>35943121.740000002</v>
       </c>
       <c r="L7">
-        <v>34.76</v>
+        <v>33.51</v>
       </c>
       <c r="M7">
-        <v>1491302.01</v>
+        <v>1437724.87</v>
       </c>
       <c r="N7">
-        <v>6488977</v>
+        <v>6922869.3499999996</v>
       </c>
       <c r="O7">
-        <v>2217958.38</v>
+        <v>-382384.42</v>
       </c>
       <c r="P7">
-        <v>12632251.619999999</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>8302730.5199999996</v>
+        <v>8425507.5700000003</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>18869842.09</v>
+        <v>17553140.780000001</v>
       </c>
       <c r="L8">
-        <v>38.71</v>
+        <v>36.01</v>
       </c>
       <c r="M8">
-        <v>754793.68</v>
+        <v>702125.63</v>
       </c>
       <c r="N8">
-        <v>2889090.68</v>
+        <v>3101884.03</v>
       </c>
       <c r="O8">
-        <v>423141.73</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>693863.67</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>24.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-18_1847 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EA01C04-F567-4001-8001-E14265EF75C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{854DB308-9B45-401A-95FB-FB411A9BAFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>4444697.0599999996</v>
+        <v>4732701.83</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>8547494.3499999996</v>
+        <v>8451253.2799999993</v>
       </c>
       <c r="L2">
-        <v>131.5</v>
+        <v>130.02000000000001</v>
       </c>
       <c r="M2">
-        <v>341899.77</v>
+        <v>338050.13</v>
       </c>
       <c r="N2">
-        <v>171275.24</v>
+        <v>160663.47</v>
       </c>
       <c r="O2">
-        <v>3484153.39</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>29800.27</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>10368242.369999999</v>
+        <v>12065008.83</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>19938927.629999999</v>
+        <v>21544658.629999999</v>
       </c>
       <c r="L3">
-        <v>34.08</v>
+        <v>36.83</v>
       </c>
       <c r="M3">
-        <v>797557.11</v>
+        <v>861786.35</v>
       </c>
       <c r="N3">
-        <v>4010979.8</v>
+        <v>4221362.83</v>
       </c>
       <c r="O3">
-        <v>706003.05</v>
+        <v>212090.27</v>
       </c>
       <c r="P3">
-        <v>1251447.3500000001</v>
+        <v>303859.36</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>31896377.280000001</v>
+        <v>36781540.729999997</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>61339187.07</v>
+        <v>65681322.740000002</v>
       </c>
       <c r="L4">
-        <v>52.43</v>
+        <v>56.14</v>
       </c>
       <c r="M4">
-        <v>2453567.48</v>
+        <v>2627252.91</v>
       </c>
       <c r="N4">
-        <v>7091968.5599999996</v>
+        <v>7292587.21</v>
       </c>
       <c r="O4">
-        <v>1291949.6299999999</v>
+        <v>813085.07</v>
       </c>
       <c r="P4">
-        <v>1197478.57</v>
+        <v>1997581.18</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>953654.06</v>
+        <v>6352663.7000000002</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1833950.12</v>
+        <v>11344042.33</v>
       </c>
       <c r="L5">
-        <v>56.43</v>
+        <v>349.05</v>
       </c>
       <c r="M5">
-        <v>73358</v>
+        <v>453761.69</v>
       </c>
       <c r="N5">
-        <v>191362.16</v>
+        <v>-282060.34000000003</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>15347.13</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>93063.61</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>2524103.14</v>
+        <v>2772890.56</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4854044.5</v>
+        <v>4951590.29</v>
       </c>
       <c r="L6">
-        <v>9.9600000000000009</v>
+        <v>10.16</v>
       </c>
       <c r="M6">
-        <v>194161.78</v>
+        <v>198063.61</v>
       </c>
       <c r="N6">
-        <v>3852158.07</v>
+        <v>4179737.22</v>
       </c>
       <c r="O6">
-        <v>399093.13</v>
+        <v>402084.67</v>
       </c>
       <c r="P6">
-        <v>37850.300000000003</v>
+        <v>86902.01</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>17488971.879999999</v>
+        <v>18062208.100000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>33632638.219999999</v>
+        <v>32253943.039999999</v>
       </c>
       <c r="L7">
-        <v>31.36</v>
+        <v>30.07</v>
       </c>
       <c r="M7">
-        <v>1345305.53</v>
+        <v>1290157.72</v>
       </c>
       <c r="N7">
-        <v>7480085.6799999997</v>
+        <v>8107981.0800000001</v>
       </c>
       <c r="O7">
-        <v>1130660.6299999999</v>
+        <v>144471.13</v>
       </c>
       <c r="P7">
-        <v>1793159.53</v>
+        <v>279295.02</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>9016485.25</v>
+        <v>9454887.4000000004</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>17339394.710000001</v>
+        <v>16883727.489999998</v>
       </c>
       <c r="L8">
-        <v>35.57</v>
+        <v>34.630000000000003</v>
       </c>
       <c r="M8">
-        <v>693575.79</v>
+        <v>675349.1</v>
       </c>
       <c r="N8">
-        <v>3311126.23</v>
+        <v>3572282.96</v>
       </c>
       <c r="O8">
-        <v>344746.7</v>
+        <v>347987.26</v>
       </c>
       <c r="P8">
-        <v>934851.68</v>
+        <v>377499.05</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0.3</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>11</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.5</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-19_1634 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{854DB308-9B45-401A-95FB-FB411A9BAFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65DFCFA9-A743-40EE-8101-AD1557D24C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>4732701.83</v>
+        <v>4808898.96</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>8451253.2799999993</v>
+        <v>8014831.5999999996</v>
       </c>
       <c r="L2">
-        <v>130.02000000000001</v>
+        <v>123.31</v>
       </c>
       <c r="M2">
-        <v>338050.13</v>
+        <v>320593.26</v>
       </c>
       <c r="N2">
-        <v>160663.47</v>
+        <v>169110.1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>224783.11</v>
       </c>
       <c r="P2">
-        <v>29800.27</v>
+        <v>405207.15</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>12065008.83</v>
+        <v>12269164.09</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>21544658.629999999</v>
+        <v>20448606.809999999</v>
       </c>
       <c r="L3">
-        <v>36.83</v>
+        <v>34.950000000000003</v>
       </c>
       <c r="M3">
-        <v>861786.35</v>
+        <v>817944.27</v>
       </c>
       <c r="N3">
-        <v>4221362.83</v>
+        <v>4623083.59</v>
       </c>
       <c r="O3">
-        <v>212090.27</v>
+        <v>1025585.37</v>
       </c>
       <c r="P3">
-        <v>303859.36</v>
+        <v>1146277.48</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>36781540.729999997</v>
+        <v>37927400.549999997</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>65681322.740000002</v>
+        <v>63212334.259999998</v>
       </c>
       <c r="L4">
-        <v>56.14</v>
+        <v>54.03</v>
       </c>
       <c r="M4">
-        <v>2627252.91</v>
+        <v>2528493.37</v>
       </c>
       <c r="N4">
-        <v>7292587.21</v>
+        <v>7907259.9400000004</v>
       </c>
       <c r="O4">
-        <v>813085.07</v>
+        <v>-2564862.29</v>
       </c>
       <c r="P4">
-        <v>1997581.18</v>
+        <v>880148.62</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>6352663.7000000002</v>
+        <v>6391397.3499999996</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>11344042.33</v>
+        <v>10652328.92</v>
       </c>
       <c r="L5">
-        <v>349.05</v>
+        <v>327.76</v>
       </c>
       <c r="M5">
-        <v>453761.69</v>
+        <v>426093.16</v>
       </c>
       <c r="N5">
-        <v>-282060.34000000003</v>
+        <v>-314139.74</v>
       </c>
       <c r="O5">
-        <v>15347.13</v>
+        <v>540268.05000000005</v>
       </c>
       <c r="P5">
-        <v>93063.61</v>
+        <v>64326.33</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>2772890.56</v>
+        <v>2821154.39</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4951590.29</v>
+        <v>4701923.99</v>
       </c>
       <c r="L6">
-        <v>10.16</v>
+        <v>9.64</v>
       </c>
       <c r="M6">
-        <v>198063.61</v>
+        <v>188076.96</v>
       </c>
       <c r="N6">
-        <v>4179737.22</v>
+        <v>4592884.5599999996</v>
       </c>
       <c r="O6">
-        <v>402084.67</v>
+        <v>-17005.03</v>
       </c>
       <c r="P6">
-        <v>86902.01</v>
+        <v>274199.06</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>18062208.100000001</v>
+        <v>18423278.690000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>32253943.039999999</v>
+        <v>30705464.48</v>
       </c>
       <c r="L7">
-        <v>30.07</v>
+        <v>28.63</v>
       </c>
       <c r="M7">
-        <v>1290157.72</v>
+        <v>1228218.58</v>
       </c>
       <c r="N7">
-        <v>8107981.0800000001</v>
+        <v>8882672.1300000008</v>
       </c>
       <c r="O7">
-        <v>144471.13</v>
+        <v>7056278.3200000003</v>
       </c>
       <c r="P7">
-        <v>279295.02</v>
+        <v>653986.92000000004</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>9454887.4000000004</v>
+        <v>9791515.2400000002</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>16883727.489999998</v>
+        <v>16319192.060000001</v>
       </c>
       <c r="L8">
-        <v>34.630000000000003</v>
+        <v>33.479999999999997</v>
       </c>
       <c r="M8">
-        <v>675349.1</v>
+        <v>652767.68000000005</v>
       </c>
       <c r="N8">
-        <v>3572282.96</v>
+        <v>3895848.48</v>
       </c>
       <c r="O8">
-        <v>347987.26</v>
+        <v>598454.18999999994</v>
       </c>
       <c r="P8">
-        <v>377499.05</v>
+        <v>685366.82</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.1000000000000001</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>9.5</v>
+        <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.2000000000000002</v>
+        <v>2.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-20_1720 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65DFCFA9-A743-40EE-8101-AD1557D24C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45490D17-FD6B-4933-8502-641E0D69286C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>4808898.96</v>
+        <v>5273416.07</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>8014831.5999999996</v>
+        <v>8239712.5999999996</v>
       </c>
       <c r="L2">
-        <v>123.31</v>
+        <v>126.76</v>
       </c>
       <c r="M2">
-        <v>320593.26</v>
+        <v>329588.5</v>
       </c>
       <c r="N2">
-        <v>169110.1</v>
+        <v>136287.1</v>
       </c>
       <c r="O2">
-        <v>224783.11</v>
+        <v>-126096.72</v>
       </c>
       <c r="P2">
-        <v>405207.15</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>12269164.09</v>
+        <v>13168788.060000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>20448606.809999999</v>
+        <v>20576231.34</v>
       </c>
       <c r="L3">
-        <v>34.950000000000003</v>
+        <v>35.17</v>
       </c>
       <c r="M3">
-        <v>817944.27</v>
+        <v>823049.25</v>
       </c>
       <c r="N3">
-        <v>4623083.59</v>
+        <v>5036801.33</v>
       </c>
       <c r="O3">
-        <v>1025585.37</v>
+        <v>455683.83</v>
       </c>
       <c r="P3">
-        <v>1146277.48</v>
+        <v>4586483.28</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>37927400.549999997</v>
+        <v>39105432.119999997</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>63212334.259999998</v>
+        <v>61102237.689999998</v>
       </c>
       <c r="L4">
-        <v>54.03</v>
+        <v>52.22</v>
       </c>
       <c r="M4">
-        <v>2528493.37</v>
+        <v>2444089.5099999998</v>
       </c>
       <c r="N4">
-        <v>7907259.9400000004</v>
+        <v>8654951.9900000002</v>
       </c>
       <c r="O4">
-        <v>-2564862.29</v>
+        <v>17461561.199999999</v>
       </c>
       <c r="P4">
-        <v>880148.62</v>
+        <v>127759.73</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>6391397.3499999996</v>
+        <v>6801750.6299999999</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10652328.92</v>
+        <v>10627735.369999999</v>
       </c>
       <c r="L5">
-        <v>327.76</v>
+        <v>327.01</v>
       </c>
       <c r="M5">
-        <v>426093.16</v>
+        <v>425109.41</v>
       </c>
       <c r="N5">
-        <v>-314139.74</v>
+        <v>-394638.96</v>
       </c>
       <c r="O5">
-        <v>540268.05000000005</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>64326.33</v>
+        <v>215736.49</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>2821154.39</v>
+        <v>5503370.6600000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>4701923.99</v>
+        <v>8599016.6600000001</v>
       </c>
       <c r="L6">
-        <v>9.64</v>
+        <v>17.64</v>
       </c>
       <c r="M6">
-        <v>188076.96</v>
+        <v>343960.67</v>
       </c>
       <c r="N6">
-        <v>4592884.5599999996</v>
+        <v>4805181.04</v>
       </c>
       <c r="O6">
-        <v>-17005.03</v>
+        <v>529596.76</v>
       </c>
       <c r="P6">
-        <v>274199.06</v>
+        <v>198333.75</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>18423278.690000001</v>
+        <v>27554822.359999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>30705464.48</v>
+        <v>43054409.939999998</v>
       </c>
       <c r="L7">
-        <v>28.63</v>
+        <v>40.14</v>
       </c>
       <c r="M7">
-        <v>1228218.58</v>
+        <v>1722176.4</v>
       </c>
       <c r="N7">
-        <v>8882672.1300000008</v>
+        <v>8855019.7400000002</v>
       </c>
       <c r="O7">
-        <v>7056278.3200000003</v>
+        <v>848376.38</v>
       </c>
       <c r="P7">
-        <v>653986.92000000004</v>
+        <v>2217958.38</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>9791515.2400000002</v>
+        <v>10893175.27</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>16319192.060000001</v>
+        <v>17020586.359999999</v>
       </c>
       <c r="L8">
-        <v>33.479999999999997</v>
+        <v>34.909999999999997</v>
       </c>
       <c r="M8">
-        <v>652767.68000000005</v>
+        <v>680823.45</v>
       </c>
       <c r="N8">
-        <v>3895848.48</v>
+        <v>4206313.8600000003</v>
       </c>
       <c r="O8">
-        <v>598454.18999999994</v>
+        <v>713754.73</v>
       </c>
       <c r="P8">
-        <v>685366.82</v>
+        <v>423141.73</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>9.1999999999999993</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-21_1637 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45490D17-FD6B-4933-8502-641E0D69286C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA208A18-1C89-4037-804A-B7EAC3454B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>5273416.07</v>
+        <v>5299015.6399999997</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>8239712.5999999996</v>
+        <v>7792670.0499999998</v>
       </c>
       <c r="L2">
-        <v>126.76</v>
+        <v>119.89</v>
       </c>
       <c r="M2">
-        <v>329588.5</v>
+        <v>311706.8</v>
       </c>
       <c r="N2">
-        <v>136287.1</v>
+        <v>150123.04999999999</v>
       </c>
       <c r="O2">
-        <v>-126096.72</v>
+        <v>49466.14</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>262136.01</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>13168788.060000001</v>
+        <v>15634014.630000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>20576231.34</v>
+        <v>22991197.98</v>
       </c>
       <c r="L3">
-        <v>35.17</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="M3">
-        <v>823049.25</v>
+        <v>919647.92</v>
       </c>
       <c r="N3">
-        <v>5036801.33</v>
+        <v>5358248.17</v>
       </c>
       <c r="O3">
-        <v>455683.83</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>4586483.28</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>39105432.119999997</v>
+        <v>39789871</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>61102237.689999998</v>
+        <v>58514516.170000002</v>
       </c>
       <c r="L4">
-        <v>52.22</v>
+        <v>50.01</v>
       </c>
       <c r="M4">
-        <v>2444089.5099999998</v>
+        <v>2340580.65</v>
       </c>
       <c r="N4">
-        <v>8654951.9900000002</v>
+        <v>9651266.1300000008</v>
       </c>
       <c r="O4">
-        <v>17461561.199999999</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>127759.73</v>
+        <v>-52556.05</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10627735.369999999</v>
+        <v>10002574.460000001</v>
       </c>
       <c r="L5">
-        <v>327.01</v>
+        <v>307.77</v>
       </c>
       <c r="M5">
-        <v>425109.41</v>
+        <v>400102.98</v>
       </c>
       <c r="N5">
-        <v>-394638.96</v>
+        <v>-443968.83</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>24912.45</v>
       </c>
       <c r="P5">
-        <v>215736.49</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>5503370.6600000001</v>
+        <v>5700229.2199999997</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>8599016.6600000001</v>
+        <v>8382690.0300000003</v>
       </c>
       <c r="L6">
-        <v>17.64</v>
+        <v>17.2</v>
       </c>
       <c r="M6">
-        <v>343960.67</v>
+        <v>335307.59999999998</v>
       </c>
       <c r="N6">
-        <v>4805181.04</v>
+        <v>5381221.3499999996</v>
       </c>
       <c r="O6">
-        <v>529596.76</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>198333.75</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>27554822.359999999</v>
+        <v>28493598.73</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>43054409.939999998</v>
+        <v>41902351.079999998</v>
       </c>
       <c r="L7">
-        <v>40.14</v>
+        <v>39.07</v>
       </c>
       <c r="M7">
-        <v>1722176.4</v>
+        <v>1676094.04</v>
       </c>
       <c r="N7">
-        <v>8855019.7400000002</v>
+        <v>9844550.1600000001</v>
       </c>
       <c r="O7">
-        <v>848376.38</v>
+        <v>236273.44</v>
       </c>
       <c r="P7">
-        <v>2217958.38</v>
+        <v>-382384.42</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>10893175.27</v>
+        <v>12348020.119999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>17020586.359999999</v>
+        <v>18158853.109999999</v>
       </c>
       <c r="L8">
-        <v>34.909999999999997</v>
+        <v>37.25</v>
       </c>
       <c r="M8">
-        <v>680823.45</v>
+        <v>726354.12</v>
       </c>
       <c r="N8">
-        <v>4206313.8600000003</v>
+        <v>4550247.49</v>
       </c>
       <c r="O8">
-        <v>713754.73</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>423141.73</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>9.1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.6</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-22_1224 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA208A18-1C89-4037-804A-B7EAC3454B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F57EF116-7A11-43E0-A5AC-C4ADAE8FDAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>5299015.6399999997</v>
+        <v>5413122.71</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>7792670.0499999998</v>
+        <v>7518225.9800000004</v>
       </c>
       <c r="L2">
-        <v>119.89</v>
+        <v>115.67</v>
       </c>
       <c r="M2">
-        <v>311706.8</v>
+        <v>300729.03999999998</v>
       </c>
       <c r="N2">
-        <v>150123.04999999999</v>
+        <v>155268.18</v>
       </c>
       <c r="O2">
-        <v>49466.14</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>262136.01</v>
+        <v>81527.179999999993</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>15634014.630000001</v>
+        <v>15703295.23</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>22991197.98</v>
+        <v>21810132.27</v>
       </c>
       <c r="L3">
-        <v>39.299999999999997</v>
+        <v>37.28</v>
       </c>
       <c r="M3">
-        <v>919647.92</v>
+        <v>872405.29</v>
       </c>
       <c r="N3">
-        <v>5358248.17</v>
+        <v>6113814.9699999997</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>286756.7</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -771,22 +771,22 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>58514516.170000002</v>
+        <v>55263709.719999999</v>
       </c>
       <c r="L4">
-        <v>50.01</v>
+        <v>47.23</v>
       </c>
       <c r="M4">
-        <v>2340580.65</v>
+        <v>2210548.39</v>
       </c>
       <c r="N4">
-        <v>9651266.1300000008</v>
+        <v>11030018.43</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>-52556.05</v>
+        <v>7263988.2699999996</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,19 +824,19 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10002574.460000001</v>
+        <v>9446875.8800000008</v>
       </c>
       <c r="L5">
-        <v>307.77</v>
+        <v>290.67</v>
       </c>
       <c r="M5">
-        <v>400102.98</v>
+        <v>377875.04</v>
       </c>
       <c r="N5">
-        <v>-443968.83</v>
+        <v>-507392.95</v>
       </c>
       <c r="O5">
-        <v>24912.45</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -877,22 +877,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>8382690.0300000003</v>
+        <v>7916985.0300000003</v>
       </c>
       <c r="L6">
-        <v>17.2</v>
+        <v>16.239999999999998</v>
       </c>
       <c r="M6">
-        <v>335307.59999999998</v>
+        <v>316679.40000000002</v>
       </c>
       <c r="N6">
-        <v>5381221.3499999996</v>
+        <v>6149967.25</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>175439.41</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -930,22 +930,22 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>41902351.079999998</v>
+        <v>39574442.689999998</v>
       </c>
       <c r="L7">
-        <v>39.07</v>
+        <v>36.9</v>
       </c>
       <c r="M7">
-        <v>1676094.04</v>
+        <v>1582977.71</v>
       </c>
       <c r="N7">
-        <v>9844550.1600000001</v>
+        <v>11250914.470000001</v>
       </c>
       <c r="O7">
-        <v>236273.44</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>-382384.42</v>
+        <v>596106.28</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,22 +983,22 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>18158853.109999999</v>
+        <v>17150027.940000001</v>
       </c>
       <c r="L8">
-        <v>37.25</v>
+        <v>35.18</v>
       </c>
       <c r="M8">
-        <v>726354.12</v>
+        <v>686001.12</v>
       </c>
       <c r="N8">
-        <v>4550247.49</v>
+        <v>5200282.84</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>3288262.55</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-24_1659 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F57EF116-7A11-43E0-A5AC-C4ADAE8FDAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5863F07-8761-4B18-BBB9-13A2DB169A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>5413122.71</v>
+        <v>5732701.9100000001</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>7518225.9800000004</v>
+        <v>7543028.8200000003</v>
       </c>
       <c r="L2">
-        <v>115.67</v>
+        <v>116.05</v>
       </c>
       <c r="M2">
-        <v>300729.03999999998</v>
+        <v>301721.15000000002</v>
       </c>
       <c r="N2">
-        <v>155268.18</v>
+        <v>127883.02</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>288004.77</v>
       </c>
       <c r="P2">
-        <v>81527.179999999993</v>
+        <v>3484153.39</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>15703295.23</v>
+        <v>16548995.24</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>21810132.27</v>
+        <v>21774993.73</v>
       </c>
       <c r="L3">
-        <v>37.28</v>
+        <v>37.22</v>
       </c>
       <c r="M3">
-        <v>872405.29</v>
+        <v>870999.75</v>
       </c>
       <c r="N3">
-        <v>6113814.9699999997</v>
+        <v>6991834.1299999999</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>1800174.78</v>
       </c>
       <c r="P3">
-        <v>286756.7</v>
+        <v>706003.05</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>39789871</v>
+        <v>52056300.240000002</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>55263709.719999999</v>
+        <v>68495131.900000006</v>
       </c>
       <c r="L4">
-        <v>47.23</v>
+        <v>58.54</v>
       </c>
       <c r="M4">
-        <v>2210548.39</v>
+        <v>2739805.28</v>
       </c>
       <c r="N4">
-        <v>11030018.43</v>
+        <v>10823949.960000001</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>4885163.46</v>
       </c>
       <c r="P4">
-        <v>7263988.2699999996</v>
+        <v>1291949.6299999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,25 +818,25 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>6801750.6299999999</v>
+        <v>6825893.8300000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>9446875.8800000008</v>
+        <v>8981439.25</v>
       </c>
       <c r="L5">
-        <v>290.67</v>
+        <v>276.35000000000002</v>
       </c>
       <c r="M5">
-        <v>377875.04</v>
+        <v>359257.57</v>
       </c>
       <c r="N5">
-        <v>-507392.95</v>
+        <v>-595982.30000000005</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>5399009.6399999997</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>5700229.2199999997</v>
+        <v>5899015.5800000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>7916985.0300000003</v>
+        <v>7761862.6100000003</v>
       </c>
       <c r="L6">
-        <v>16.239999999999998</v>
+        <v>15.92</v>
       </c>
       <c r="M6">
-        <v>316679.40000000002</v>
+        <v>310474.5</v>
       </c>
       <c r="N6">
-        <v>6149967.25</v>
+        <v>7141830.7400000002</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>248787.42</v>
       </c>
       <c r="P6">
-        <v>175439.41</v>
+        <v>399093.13</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>28493598.73</v>
+        <v>29190550.059999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>39574442.689999998</v>
+        <v>38408618.5</v>
       </c>
       <c r="L7">
-        <v>36.9</v>
+        <v>35.81</v>
       </c>
       <c r="M7">
-        <v>1582977.71</v>
+        <v>1536344.74</v>
       </c>
       <c r="N7">
-        <v>11250914.470000001</v>
+        <v>13009908.32</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>774446.28</v>
       </c>
       <c r="P7">
-        <v>596106.28</v>
+        <v>1130660.6299999999</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>12348020.119999999</v>
+        <v>16203950.109999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>17150027.940000001</v>
+        <v>21320986.989999998</v>
       </c>
       <c r="L8">
-        <v>35.18</v>
+        <v>43.74</v>
       </c>
       <c r="M8">
-        <v>686001.12</v>
+        <v>852839.48</v>
       </c>
       <c r="N8">
-        <v>5200282.84</v>
+        <v>5424341.6500000004</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>438402.15</v>
       </c>
       <c r="P8">
-        <v>3288262.55</v>
+        <v>344746.7</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.5999999999999996</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.5</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.2999999999999998</v>
+        <v>2.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-25_1727 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5863F07-8761-4B18-BBB9-13A2DB169A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{27A979C6-7674-484B-BA5B-D50A9FED6EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -200,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q7">
+  <autoFilter ref="A1:Q7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -564,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>7543028.8200000003</v>
+        <v>7165877.3799999999</v>
       </c>
       <c r="L2">
-        <v>116.05</v>
+        <v>110.24</v>
       </c>
       <c r="M2">
-        <v>301721.15000000002</v>
+        <v>286635.09999999998</v>
       </c>
       <c r="N2">
-        <v>127883.02</v>
+        <v>153459.62</v>
       </c>
       <c r="O2">
-        <v>288004.77</v>
+        <v>62422</v>
       </c>
       <c r="P2">
-        <v>3484153.39</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>16548995.24</v>
+        <v>16983694.489999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>21774993.73</v>
+        <v>21229618.109999999</v>
       </c>
       <c r="L3">
-        <v>37.22</v>
+        <v>36.29</v>
       </c>
       <c r="M3">
-        <v>870999.75</v>
+        <v>849184.72</v>
       </c>
       <c r="N3">
-        <v>6991834.1299999999</v>
+        <v>8303261.0999999996</v>
       </c>
       <c r="O3">
-        <v>1800174.78</v>
+        <v>100746.94</v>
       </c>
       <c r="P3">
-        <v>706003.05</v>
+        <v>212090.27</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -747,13 +747,13 @@
         <v>26</v>
       </c>
       <c r="C4">
-        <v>105008</v>
+        <v>105003</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
         <v>21</v>
@@ -762,31 +762,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>117000000</v>
+        <v>3250000</v>
       </c>
       <c r="I4">
-        <v>52056300.240000002</v>
+        <v>6825893.8300000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>68495131.900000006</v>
+        <v>8532367.2899999991</v>
       </c>
       <c r="L4">
-        <v>58.54</v>
+        <v>262.52999999999997</v>
       </c>
       <c r="M4">
-        <v>2739805.28</v>
+        <v>341294.69</v>
       </c>
       <c r="N4">
-        <v>10823949.960000001</v>
+        <v>-715178.77</v>
       </c>
       <c r="O4">
-        <v>4885163.46</v>
+        <v>38733.65</v>
       </c>
       <c r="P4">
-        <v>1291949.6299999999</v>
+        <v>15347.13</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -800,13 +800,13 @@
         <v>26</v>
       </c>
       <c r="C5">
-        <v>105003</v>
+        <v>105004</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
         <v>21</v>
@@ -815,31 +815,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>3250000</v>
+        <v>48750000</v>
       </c>
       <c r="I5">
-        <v>6825893.8300000001</v>
+        <v>6448427.8300000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>8981439.25</v>
+        <v>8060534.7800000003</v>
       </c>
       <c r="L5">
-        <v>276.35000000000002</v>
+        <v>16.53</v>
       </c>
       <c r="M5">
-        <v>359257.57</v>
+        <v>322421.39</v>
       </c>
       <c r="N5">
-        <v>-595982.30000000005</v>
+        <v>8460314.4299999997</v>
       </c>
       <c r="O5">
-        <v>5399009.6399999997</v>
+        <v>2594646.59</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>402084.67</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -853,13 +853,13 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>105004</v>
+        <v>120041</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -868,31 +868,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>48750000</v>
+        <v>107250000</v>
       </c>
       <c r="I6">
-        <v>5899015.5800000001</v>
+        <v>37612240.210000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>7761862.6100000003</v>
+        <v>47015300.259999998</v>
       </c>
       <c r="L6">
-        <v>15.92</v>
+        <v>43.84</v>
       </c>
       <c r="M6">
-        <v>310474.5</v>
+        <v>1880612.01</v>
       </c>
       <c r="N6">
-        <v>7141830.7400000002</v>
+        <v>13927551.960000001</v>
       </c>
       <c r="O6">
-        <v>248787.42</v>
+        <v>1227454.22</v>
       </c>
       <c r="P6">
-        <v>399093.13</v>
+        <v>144471.13</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -906,13 +906,13 @@
         <v>26</v>
       </c>
       <c r="C7">
-        <v>120041</v>
+        <v>105006</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
         <v>21</v>
@@ -921,86 +921,33 @@
         <v>22</v>
       </c>
       <c r="H7">
-        <v>107250000</v>
+        <v>48750000</v>
       </c>
       <c r="I7">
-        <v>29190550.059999999</v>
+        <v>16966099.329999998</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>38408618.5</v>
+        <v>21207624.16</v>
       </c>
       <c r="L7">
-        <v>35.81</v>
+        <v>43.5</v>
       </c>
       <c r="M7">
-        <v>1536344.74</v>
+        <v>848304.97</v>
       </c>
       <c r="N7">
-        <v>13009908.32</v>
+        <v>6356780.1299999999</v>
       </c>
       <c r="O7">
-        <v>774446.28</v>
+        <v>1265039.8500000001</v>
       </c>
       <c r="P7">
-        <v>1130660.6299999999</v>
+        <v>347987.26</v>
       </c>
       <c r="Q7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8">
-        <v>105006</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H8">
-        <v>48750000</v>
-      </c>
-      <c r="I8">
-        <v>16203950.109999999</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>21320986.989999998</v>
-      </c>
-      <c r="L8">
-        <v>43.74</v>
-      </c>
-      <c r="M8">
-        <v>852839.48</v>
-      </c>
-      <c r="N8">
-        <v>5424341.6500000004</v>
-      </c>
-      <c r="O8">
-        <v>438402.15</v>
-      </c>
-      <c r="P8">
-        <v>344746.7</v>
-      </c>
-      <c r="Q8">
         <v>0</v>
       </c>
     </row>
@@ -1076,7 +1023,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1075,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1101,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1153,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1205,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-26_1738 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27A979C6-7674-484B-BA5B-D50A9FED6EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06505ADF-3A6E-4F38-9371-A49542FD0928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,22 +665,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>7165877.3799999999</v>
+        <v>6824645.1299999999</v>
       </c>
       <c r="L2">
-        <v>110.24</v>
+        <v>104.99</v>
       </c>
       <c r="M2">
-        <v>286635.09999999998</v>
+        <v>272985.81</v>
       </c>
       <c r="N2">
-        <v>153459.62</v>
+        <v>191824.52</v>
       </c>
       <c r="O2">
-        <v>62422</v>
+        <v>478292.23</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>224783.11</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>16983694.489999998</v>
+        <v>17742036.629999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>21229618.109999999</v>
+        <v>21121472.18</v>
       </c>
       <c r="L3">
-        <v>36.29</v>
+        <v>36.11</v>
       </c>
       <c r="M3">
-        <v>849184.72</v>
+        <v>844858.89</v>
       </c>
       <c r="N3">
-        <v>8303261.0999999996</v>
+        <v>10189490.84</v>
       </c>
       <c r="O3">
-        <v>100746.94</v>
+        <v>899623.97</v>
       </c>
       <c r="P3">
-        <v>212090.27</v>
+        <v>1025585.37</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>3250000</v>
       </c>
       <c r="I4">
-        <v>6825893.8300000001</v>
+        <v>6935675.8300000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>8532367.2899999991</v>
+        <v>8256756.9400000004</v>
       </c>
       <c r="L4">
-        <v>262.52999999999997</v>
+        <v>254.05</v>
       </c>
       <c r="M4">
-        <v>341294.69</v>
+        <v>330270.28000000003</v>
       </c>
       <c r="N4">
-        <v>-715178.77</v>
+        <v>-921418.96</v>
       </c>
       <c r="O4">
-        <v>38733.65</v>
+        <v>410353.28</v>
       </c>
       <c r="P4">
-        <v>15347.13</v>
+        <v>540268.05000000005</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>48750000</v>
       </c>
       <c r="I5">
-        <v>6448427.8300000001</v>
+        <v>7503935.4299999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>8060534.7800000003</v>
+        <v>8933256.4700000007</v>
       </c>
       <c r="L5">
-        <v>16.53</v>
+        <v>18.32</v>
       </c>
       <c r="M5">
-        <v>322421.39</v>
+        <v>357330.26</v>
       </c>
       <c r="N5">
-        <v>8460314.4299999997</v>
+        <v>10311516.140000001</v>
       </c>
       <c r="O5">
-        <v>2594646.59</v>
+        <v>135833.51</v>
       </c>
       <c r="P5">
-        <v>402084.67</v>
+        <v>-17005.03</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>107250000</v>
       </c>
       <c r="I6">
-        <v>37612240.210000001</v>
+        <v>37761968.789999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>47015300.259999998</v>
+        <v>44954724.75</v>
       </c>
       <c r="L6">
-        <v>43.84</v>
+        <v>41.92</v>
       </c>
       <c r="M6">
-        <v>1880612.01</v>
+        <v>1798188.99</v>
       </c>
       <c r="N6">
-        <v>13927551.960000001</v>
+        <v>17372007.800000001</v>
       </c>
       <c r="O6">
-        <v>1227454.22</v>
+        <v>8063949.9900000002</v>
       </c>
       <c r="P6">
-        <v>144471.13</v>
+        <v>7056278.3200000003</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>48750000</v>
       </c>
       <c r="I7">
-        <v>16966099.329999998</v>
+        <v>17688718.059999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>21207624.16</v>
+        <v>21057997.690000001</v>
       </c>
       <c r="L7">
-        <v>43.5</v>
+        <v>43.2</v>
       </c>
       <c r="M7">
-        <v>848304.97</v>
+        <v>842319.91</v>
       </c>
       <c r="N7">
-        <v>6356780.1299999999</v>
+        <v>7765320.4800000004</v>
       </c>
       <c r="O7">
-        <v>1265039.8500000001</v>
+        <v>173248.02</v>
       </c>
       <c r="P7">
-        <v>347987.26</v>
+        <v>598454.18999999994</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -1023,7 +1023,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1075,7 +1075,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1153,7 +1153,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1179,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1205,7 +1205,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2000000000000002</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1231,7 +1231,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-27_0741 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06505ADF-3A6E-4F38-9371-A49542FD0928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2A34CB1-F789-43FA-B4CB-77E7BC1FA8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -200,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q7">
-  <autoFilter ref="A1:Q7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
+  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
@@ -564,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -665,16 +665,16 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6824645.1299999999</v>
+        <v>6514433.9800000004</v>
       </c>
       <c r="L2">
-        <v>104.99</v>
+        <v>100.22</v>
       </c>
       <c r="M2">
-        <v>272985.81</v>
+        <v>260577.36</v>
       </c>
       <c r="N2">
-        <v>191824.52</v>
+        <v>255766.03</v>
       </c>
       <c r="O2">
         <v>478292.23</v>
@@ -712,22 +712,22 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>17742036.629999999</v>
+        <v>17751929.84</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>21121472.18</v>
+        <v>20172647.550000001</v>
       </c>
       <c r="L3">
-        <v>36.11</v>
+        <v>34.479999999999997</v>
       </c>
       <c r="M3">
-        <v>844858.89</v>
+        <v>806905.9</v>
       </c>
       <c r="N3">
-        <v>10189490.84</v>
+        <v>13582690.050000001</v>
       </c>
       <c r="O3">
         <v>899623.97</v>
@@ -747,13 +747,13 @@
         <v>26</v>
       </c>
       <c r="C4">
-        <v>105003</v>
+        <v>105008</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
         <v>21</v>
@@ -762,31 +762,31 @@
         <v>22</v>
       </c>
       <c r="H4">
-        <v>3250000</v>
+        <v>117000000</v>
       </c>
       <c r="I4">
-        <v>6935675.8300000001</v>
+        <v>68908854.430000007</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>8256756.9400000004</v>
+        <v>78305516.390000001</v>
       </c>
       <c r="L4">
-        <v>254.05</v>
+        <v>66.930000000000007</v>
       </c>
       <c r="M4">
-        <v>330270.28000000003</v>
+        <v>3132220.66</v>
       </c>
       <c r="N4">
-        <v>-921418.96</v>
+        <v>16030381.859999999</v>
       </c>
       <c r="O4">
-        <v>410353.28</v>
+        <v>688957</v>
       </c>
       <c r="P4">
-        <v>540268.05000000005</v>
+        <v>-2564862.29</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -800,13 +800,13 @@
         <v>26</v>
       </c>
       <c r="C5">
-        <v>105004</v>
+        <v>105003</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
         <v>21</v>
@@ -815,31 +815,31 @@
         <v>22</v>
       </c>
       <c r="H5">
-        <v>48750000</v>
+        <v>3250000</v>
       </c>
       <c r="I5">
-        <v>7503935.4299999997</v>
+        <v>6935675.8300000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>8933256.4700000007</v>
+        <v>7881449.8099999996</v>
       </c>
       <c r="L5">
-        <v>18.32</v>
+        <v>242.51</v>
       </c>
       <c r="M5">
-        <v>357330.26</v>
+        <v>315257.99</v>
       </c>
       <c r="N5">
-        <v>10311516.140000001</v>
+        <v>-1228558.6100000001</v>
       </c>
       <c r="O5">
-        <v>135833.51</v>
+        <v>410353.28</v>
       </c>
       <c r="P5">
-        <v>-17005.03</v>
+        <v>540268.05000000005</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -853,13 +853,13 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>120041</v>
+        <v>105004</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
         <v>21</v>
@@ -868,31 +868,31 @@
         <v>22</v>
       </c>
       <c r="H6">
-        <v>107250000</v>
+        <v>48750000</v>
       </c>
       <c r="I6">
-        <v>37761968.789999999</v>
+        <v>7503935.4299999997</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>44954724.75</v>
+        <v>8527199.3499999996</v>
       </c>
       <c r="L6">
-        <v>41.92</v>
+        <v>17.489999999999998</v>
       </c>
       <c r="M6">
-        <v>1798188.99</v>
+        <v>341087.97</v>
       </c>
       <c r="N6">
-        <v>17372007.800000001</v>
+        <v>13748688.189999999</v>
       </c>
       <c r="O6">
-        <v>8063949.9900000002</v>
+        <v>135833.51</v>
       </c>
       <c r="P6">
-        <v>7056278.3200000003</v>
+        <v>-17005.03</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -906,13 +906,13 @@
         <v>26</v>
       </c>
       <c r="C7">
-        <v>105006</v>
+        <v>120041</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
         <v>21</v>
@@ -921,33 +921,86 @@
         <v>22</v>
       </c>
       <c r="H7">
+        <v>107250000</v>
+      </c>
+      <c r="I7">
+        <v>54248754.390000001</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>61646311.810000002</v>
+      </c>
+      <c r="L7">
+        <v>57.48</v>
+      </c>
+      <c r="M7">
+        <v>2465852.4700000002</v>
+      </c>
+      <c r="N7">
+        <v>17667081.870000001</v>
+      </c>
+      <c r="O7">
+        <v>8063949.9900000002</v>
+      </c>
+      <c r="P7">
+        <v>7056278.3200000003</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>105006</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8">
         <v>48750000</v>
       </c>
-      <c r="I7">
+      <c r="I8">
         <v>17688718.059999999</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>21057997.690000001</v>
-      </c>
-      <c r="L7">
-        <v>43.2</v>
-      </c>
-      <c r="M7">
-        <v>842319.91</v>
-      </c>
-      <c r="N7">
-        <v>7765320.4800000004</v>
-      </c>
-      <c r="O7">
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>20100815.98</v>
+      </c>
+      <c r="L8">
+        <v>41.23</v>
+      </c>
+      <c r="M8">
+        <v>804032.64</v>
+      </c>
+      <c r="N8">
+        <v>10353760.65</v>
+      </c>
+      <c r="O8">
         <v>173248.02</v>
       </c>
-      <c r="P7">
+      <c r="P8">
         <v>598454.18999999994</v>
       </c>
-      <c r="Q7">
+      <c r="Q8">
         <v>0</v>
       </c>
     </row>
@@ -1153,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1179,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1205,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.2999999999999998</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-08-27_1652 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2A34CB1-F789-43FA-B4CB-77E7BC1FA8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D32BD91-6D88-43FE-A70B-85E9B7A1FE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>5732701.9100000001</v>
+        <v>6090086.6699999999</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6514433.9800000004</v>
+        <v>6619659.4199999999</v>
       </c>
       <c r="L2">
-        <v>100.22</v>
+        <v>101.84</v>
       </c>
       <c r="M2">
-        <v>260577.36</v>
+        <v>264786.38</v>
       </c>
       <c r="N2">
-        <v>255766.03</v>
+        <v>204956.66</v>
       </c>
       <c r="O2">
-        <v>478292.23</v>
+        <v>25599.57</v>
       </c>
       <c r="P2">
-        <v>224783.11</v>
+        <v>-126096.72</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>17751929.84</v>
+        <v>19184686.079999998</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>20172647.550000001</v>
+        <v>20852919.649999999</v>
       </c>
       <c r="L3">
-        <v>34.479999999999997</v>
+        <v>35.65</v>
       </c>
       <c r="M3">
-        <v>806905.9</v>
+        <v>834116.79</v>
       </c>
       <c r="N3">
-        <v>13582690.050000001</v>
+        <v>19657656.960000001</v>
       </c>
       <c r="O3">
-        <v>899623.97</v>
+        <v>2415401.67</v>
       </c>
       <c r="P3">
-        <v>1025585.37</v>
+        <v>455683.83</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>68908854.430000007</v>
+        <v>69287552.159999996</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>78305516.390000001</v>
+        <v>75312556.689999998</v>
       </c>
       <c r="L4">
-        <v>66.930000000000007</v>
+        <v>64.37</v>
       </c>
       <c r="M4">
-        <v>3132220.66</v>
+        <v>3012502.27</v>
       </c>
       <c r="N4">
-        <v>16030381.859999999</v>
+        <v>23856223.920000002</v>
       </c>
       <c r="O4">
-        <v>688957</v>
+        <v>684438.87</v>
       </c>
       <c r="P4">
-        <v>-2564862.29</v>
+        <v>17461561.199999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>6935675.8300000001</v>
+        <v>7169388.7999999998</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>7881449.8099999996</v>
+        <v>7792813.9199999999</v>
       </c>
       <c r="L5">
-        <v>242.51</v>
+        <v>239.78</v>
       </c>
       <c r="M5">
-        <v>315257.99</v>
+        <v>311712.56</v>
       </c>
       <c r="N5">
-        <v>-1228558.6100000001</v>
+        <v>-1959694.4</v>
       </c>
       <c r="O5">
-        <v>410353.28</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>540268.05000000005</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>7503935.4299999997</v>
+        <v>9780250.6999999993</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>8527199.3499999996</v>
+        <v>10630707.289999999</v>
       </c>
       <c r="L6">
-        <v>17.489999999999998</v>
+        <v>21.81</v>
       </c>
       <c r="M6">
-        <v>341087.97</v>
+        <v>425228.29</v>
       </c>
       <c r="N6">
-        <v>13748688.189999999</v>
+        <v>19484874.649999999</v>
       </c>
       <c r="O6">
-        <v>135833.51</v>
+        <v>196858.56</v>
       </c>
       <c r="P6">
-        <v>-17005.03</v>
+        <v>529596.76</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>54248754.390000001</v>
+        <v>54952004.100000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>61646311.810000002</v>
+        <v>59730439.240000002</v>
       </c>
       <c r="L7">
-        <v>57.48</v>
+        <v>55.69</v>
       </c>
       <c r="M7">
-        <v>2465852.4700000002</v>
+        <v>2389217.5699999998</v>
       </c>
       <c r="N7">
-        <v>17667081.870000001</v>
+        <v>26148997.949999999</v>
       </c>
       <c r="O7">
-        <v>8063949.9900000002</v>
+        <v>938776.37</v>
       </c>
       <c r="P7">
-        <v>7056278.3200000003</v>
+        <v>848376.38</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>17688718.059999999</v>
+        <v>21212091.16</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20100815.98</v>
+        <v>23056620.829999998</v>
       </c>
       <c r="L8">
-        <v>41.23</v>
+        <v>47.3</v>
       </c>
       <c r="M8">
-        <v>804032.64</v>
+        <v>922264.83</v>
       </c>
       <c r="N8">
-        <v>10353760.65</v>
+        <v>13768954.42</v>
       </c>
       <c r="O8">
-        <v>173248.02</v>
+        <v>1454844.85</v>
       </c>
       <c r="P8">
-        <v>598454.18999999994</v>
+        <v>713754.73</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>4.4000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-28_1739 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D32BD91-6D88-43FE-A70B-85E9B7A1FE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC1F40D5-4829-4295-BED9-74043E87204A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>6090086.6699999999</v>
+        <v>6092577.2800000003</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6619659.4199999999</v>
+        <v>6346434.6699999999</v>
       </c>
       <c r="L2">
-        <v>101.84</v>
+        <v>97.64</v>
       </c>
       <c r="M2">
-        <v>264786.38</v>
+        <v>253857.39</v>
       </c>
       <c r="N2">
-        <v>204956.66</v>
+        <v>407422.71999999997</v>
       </c>
       <c r="O2">
-        <v>25599.57</v>
+        <v>114107.07</v>
       </c>
       <c r="P2">
-        <v>-126096.72</v>
+        <v>49466.14</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +712,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>19184686.079999998</v>
+        <v>39225178.530000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>20852919.649999999</v>
+        <v>40859560.969999999</v>
       </c>
       <c r="L3">
-        <v>35.65</v>
+        <v>69.849999999999994</v>
       </c>
       <c r="M3">
-        <v>834116.79</v>
+        <v>1634382.44</v>
       </c>
       <c r="N3">
-        <v>19657656.960000001</v>
+        <v>19274821.469999999</v>
       </c>
       <c r="O3">
-        <v>2415401.67</v>
+        <v>55505.48</v>
       </c>
       <c r="P3">
-        <v>455683.83</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +765,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>69287552.159999996</v>
+        <v>82978204.579999998</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>75312556.689999998</v>
+        <v>86435629.769999996</v>
       </c>
       <c r="L4">
-        <v>64.37</v>
+        <v>73.88</v>
       </c>
       <c r="M4">
-        <v>3012502.27</v>
+        <v>3457425.19</v>
       </c>
       <c r="N4">
-        <v>23856223.920000002</v>
+        <v>34021795.420000002</v>
       </c>
       <c r="O4">
-        <v>684438.87</v>
+        <v>7287391.9100000001</v>
       </c>
       <c r="P4">
-        <v>17461561.199999999</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +818,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>7169388.7999999998</v>
+        <v>7366508.0199999996</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>7792813.9199999999</v>
+        <v>7673445.8600000003</v>
       </c>
       <c r="L5">
-        <v>239.78</v>
+        <v>236.11</v>
       </c>
       <c r="M5">
-        <v>311712.56</v>
+        <v>306937.83</v>
       </c>
       <c r="N5">
-        <v>-1959694.4</v>
+        <v>-4116508.02</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>24143.200000000001</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>24912.45</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +871,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>9780250.6999999993</v>
+        <v>10017730.210000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10630707.289999999</v>
+        <v>10435135.630000001</v>
       </c>
       <c r="L6">
-        <v>21.81</v>
+        <v>21.41</v>
       </c>
       <c r="M6">
-        <v>425228.29</v>
+        <v>417405.43</v>
       </c>
       <c r="N6">
-        <v>19484874.649999999</v>
+        <v>38732269.789999999</v>
       </c>
       <c r="O6">
-        <v>196858.56</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>529596.76</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>54952004.100000001</v>
+        <v>67549693.489999995</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>59730439.240000002</v>
+        <v>70364264.049999997</v>
       </c>
       <c r="L7">
-        <v>55.69</v>
+        <v>65.61</v>
       </c>
       <c r="M7">
-        <v>2389217.5699999998</v>
+        <v>2814570.56</v>
       </c>
       <c r="N7">
-        <v>26148997.949999999</v>
+        <v>39700306.509999998</v>
       </c>
       <c r="O7">
-        <v>938776.37</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <v>848376.38</v>
+        <v>236273.44</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +977,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>21212091.16</v>
+        <v>22144335.98</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23056620.829999998</v>
+        <v>23067016.640000001</v>
       </c>
       <c r="L8">
-        <v>47.3</v>
+        <v>47.32</v>
       </c>
       <c r="M8">
-        <v>922264.83</v>
+        <v>922680.67</v>
       </c>
       <c r="N8">
-        <v>13768954.42</v>
+        <v>26605664.02</v>
       </c>
       <c r="O8">
-        <v>1454844.85</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>713754.73</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.0999999999999996</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>5.3</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.4</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>2.2999999999999998</v>
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-08-29_1337 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC1F40D5-4829-4295-BED9-74043E87204A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BB540A2-DF11-43CA-A860-6B87FED578E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -659,28 +659,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>6092577.2800000003</v>
+        <v>6220187.6200000001</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6346434.6699999999</v>
+        <v>6479362.0999999996</v>
       </c>
       <c r="L2">
-        <v>97.64</v>
+        <v>99.68</v>
       </c>
       <c r="M2">
-        <v>253857.39</v>
+        <v>259174.48</v>
       </c>
       <c r="N2">
-        <v>407422.71999999997</v>
+        <v>279812.38</v>
       </c>
       <c r="O2">
-        <v>114107.07</v>
+        <v>319579.2</v>
       </c>
       <c r="P2">
-        <v>49466.14</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,25 +712,25 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>39225178.530000001</v>
+        <v>44544262.229999997</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>40859560.969999999</v>
+        <v>46400273.149999999</v>
       </c>
       <c r="L3">
-        <v>69.849999999999994</v>
+        <v>79.319999999999993</v>
       </c>
       <c r="M3">
-        <v>1634382.44</v>
+        <v>1856010.93</v>
       </c>
       <c r="N3">
-        <v>19274821.469999999</v>
+        <v>13955737.77</v>
       </c>
       <c r="O3">
-        <v>55505.48</v>
+        <v>789240.23</v>
       </c>
       <c r="P3">
         <v>0</v>
@@ -765,25 +765,25 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>82978204.579999998</v>
+        <v>83250178.450000003</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>86435629.769999996</v>
+        <v>86718935.879999995</v>
       </c>
       <c r="L4">
-        <v>73.88</v>
+        <v>74.12</v>
       </c>
       <c r="M4">
-        <v>3457425.19</v>
+        <v>3468757.44</v>
       </c>
       <c r="N4">
-        <v>34021795.420000002</v>
+        <v>33749821.549999997</v>
       </c>
       <c r="O4">
-        <v>7287391.9100000001</v>
+        <v>4979037.34</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -836,10 +836,10 @@
         <v>-4116508.02</v>
       </c>
       <c r="O5">
-        <v>24143.200000000001</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>24912.45</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,25 +871,25 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>10017730.210000001</v>
+        <v>9982357.7200000007</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10435135.630000001</v>
+        <v>10398289.289999999</v>
       </c>
       <c r="L6">
-        <v>21.41</v>
+        <v>21.33</v>
       </c>
       <c r="M6">
-        <v>417405.43</v>
+        <v>415931.57</v>
       </c>
       <c r="N6">
-        <v>38732269.789999999</v>
+        <v>38767642.280000001</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>198786.36</v>
       </c>
       <c r="P6">
         <v>0</v>
@@ -924,28 +924,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>67549693.489999995</v>
+        <v>68063064.379999995</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>70364264.049999997</v>
+        <v>70899025.400000006</v>
       </c>
       <c r="L7">
-        <v>65.61</v>
+        <v>66.11</v>
       </c>
       <c r="M7">
-        <v>2814570.56</v>
+        <v>2835961.02</v>
       </c>
       <c r="N7">
-        <v>39700306.509999998</v>
+        <v>39186935.619999997</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>696951.33</v>
       </c>
       <c r="P7">
-        <v>236273.44</v>
+        <v>0</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,25 +977,25 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>22144335.98</v>
+        <v>21922768.469999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23067016.640000001</v>
+        <v>22836217.149999999</v>
       </c>
       <c r="L8">
-        <v>47.32</v>
+        <v>46.84</v>
       </c>
       <c r="M8">
-        <v>922680.67</v>
+        <v>913448.69</v>
       </c>
       <c r="N8">
-        <v>26605664.02</v>
+        <v>26827231.530000001</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>3855929.99</v>
       </c>
       <c r="P8">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-01_1718 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3912EB8F-AAD0-49DD-9379-43EEF192BE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45FE5210-8DD2-4A24-9F6B-3BD0EBF84813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,10 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="17" customWidth="1"/>
@@ -659,28 +661,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>6220187.6200000001</v>
+        <v>89033.12</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6220187.6200000001</v>
+        <v>2314861.2000000002</v>
       </c>
       <c r="L2">
-        <v>95.7</v>
+        <v>35.61</v>
       </c>
       <c r="M2">
-        <v>248807.5</v>
+        <v>89033.12</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>256438.68</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>288004.77</v>
+        <v>62422</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +714,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>44544262.229999997</v>
+        <v>7635712.5300000003</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>44544262.229999997</v>
+        <v>198528525.78999999</v>
       </c>
       <c r="L3">
-        <v>76.14</v>
+        <v>339.37</v>
       </c>
       <c r="M3">
-        <v>1781770.49</v>
+        <v>7635712.5300000003</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>2034571.5</v>
       </c>
       <c r="O3">
-        <v>554759.04</v>
+        <v>734455.9</v>
       </c>
       <c r="P3">
-        <v>1800174.78</v>
+        <v>100746.94</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +767,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>82889180.920000002</v>
+        <v>12984756.84</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>82889180.920000002</v>
+        <v>337603677.89999998</v>
       </c>
       <c r="L4">
-        <v>70.849999999999994</v>
+        <v>288.55</v>
       </c>
       <c r="M4">
-        <v>3315567.24</v>
+        <v>12984756.84</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>4160609.73</v>
       </c>
       <c r="O4">
-        <v>1268157.78</v>
+        <v>15584396.4</v>
       </c>
       <c r="P4">
-        <v>4885163.46</v>
+        <v>1634934.39</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -818,28 +820,28 @@
         <v>3250000</v>
       </c>
       <c r="I5">
-        <v>7755549.1799999997</v>
+        <v>21094.7</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>7755549.1799999997</v>
+        <v>548462.18999999994</v>
       </c>
       <c r="L5">
-        <v>238.63</v>
+        <v>16.88</v>
       </c>
       <c r="M5">
-        <v>310221.96999999997</v>
+        <v>21094.7</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>129156.21</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>109782</v>
       </c>
       <c r="P5">
-        <v>5399009.6399999997</v>
+        <v>38733.65</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -871,28 +873,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>10155362.300000001</v>
+        <v>4453446.84</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10155362.300000001</v>
+        <v>115789617.87</v>
       </c>
       <c r="L6">
-        <v>20.83</v>
+        <v>237.52</v>
       </c>
       <c r="M6">
-        <v>406214.49</v>
+        <v>4453446.84</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>1771862.13</v>
       </c>
       <c r="O6">
-        <v>549412.25</v>
+        <v>1055507.6000000001</v>
       </c>
       <c r="P6">
-        <v>248787.42</v>
+        <v>2594646.59</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +926,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>68179043.670000002</v>
+        <v>2171261.9300000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>68179043.670000002</v>
+        <v>56452810.259999998</v>
       </c>
       <c r="L7">
-        <v>63.57</v>
+        <v>52.64</v>
       </c>
       <c r="M7">
-        <v>2727161.75</v>
+        <v>2171261.9300000002</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>4203149.5199999996</v>
       </c>
       <c r="O7">
-        <v>8393371.9900000002</v>
+        <v>16664832.34</v>
       </c>
       <c r="P7">
-        <v>774446.28</v>
+        <v>1227454.22</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +979,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>22097968.920000002</v>
+        <v>767067.6</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>22097968.920000002</v>
+        <v>19943757.670000002</v>
       </c>
       <c r="L8">
-        <v>45.33</v>
+        <v>40.909999999999997</v>
       </c>
       <c r="M8">
-        <v>883918.76</v>
+        <v>767067.6</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>1919317.3</v>
       </c>
       <c r="O8">
-        <v>732484.06</v>
+        <v>722618.73</v>
       </c>
       <c r="P8">
-        <v>438402.15</v>
+        <v>1265039.8500000001</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1104,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1130,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1154,7 +1156,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1182,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>5.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1206,7 +1208,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>4.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1286,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>1.3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-03_1728 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2357C0C2-2890-4EE8-B7B2-11ED6A82BD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C5EA489-3F4C-436E-A722-34D26706818B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -660,28 +660,28 @@
         <v>6500000</v>
       </c>
       <c r="I2">
-        <v>86186.58</v>
+        <v>524469.71</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1077332.25</v>
+        <v>4545404.12</v>
       </c>
       <c r="L2">
-        <v>16.57</v>
+        <v>69.930000000000007</v>
       </c>
       <c r="M2">
-        <v>43093.29</v>
+        <v>174823.24</v>
       </c>
       <c r="N2">
-        <v>278861.45</v>
+        <v>259805.66</v>
       </c>
       <c r="O2">
-        <v>331006.88</v>
+        <v>141131.70000000001</v>
       </c>
       <c r="P2">
-        <v>478292.23</v>
+        <v>25599.57</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>58500000</v>
       </c>
       <c r="I3">
-        <v>9837360.6799999997</v>
+        <v>12058075.369999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>122967008.44</v>
+        <v>104503319.84999999</v>
       </c>
       <c r="L3">
-        <v>210.2</v>
+        <v>178.64</v>
       </c>
       <c r="M3">
-        <v>4918680.34</v>
+        <v>4019358.46</v>
       </c>
       <c r="N3">
-        <v>2115766.9300000002</v>
+        <v>2019214.11</v>
       </c>
       <c r="O3">
-        <v>1417167.38</v>
+        <v>20222919.98</v>
       </c>
       <c r="P3">
-        <v>899623.97</v>
+        <v>2415401.67</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>117000000</v>
       </c>
       <c r="I4">
-        <v>14666202.99</v>
+        <v>15293474.52</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>183327537.41</v>
+        <v>132543445.84</v>
       </c>
       <c r="L4">
-        <v>156.69</v>
+        <v>113.28</v>
       </c>
       <c r="M4">
-        <v>7333101.5</v>
+        <v>5097824.84</v>
       </c>
       <c r="N4">
-        <v>4449295.5199999996</v>
+        <v>4422022.8499999996</v>
       </c>
       <c r="O4">
-        <v>10110967.859999999</v>
+        <v>4205985.53</v>
       </c>
       <c r="P4">
-        <v>688957</v>
+        <v>684438.87</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3827187.11</v>
+        <v>2653516.39</v>
       </c>
       <c r="L5">
-        <v>117.76</v>
+        <v>81.650000000000006</v>
       </c>
       <c r="M5">
-        <v>153087.48000000001</v>
+        <v>102058.32</v>
       </c>
       <c r="N5">
         <v>127992.39</v>
       </c>
       <c r="O5">
-        <v>233712.97</v>
+        <v>197119.22</v>
       </c>
       <c r="P5">
-        <v>410353.28</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>48750000</v>
       </c>
       <c r="I6">
-        <v>4910547.93</v>
+        <v>4941242.1900000004</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>61381849.079999998</v>
+        <v>42824098.979999997</v>
       </c>
       <c r="L6">
-        <v>125.91</v>
+        <v>87.84</v>
       </c>
       <c r="M6">
-        <v>2455273.96</v>
+        <v>1647080.73</v>
       </c>
       <c r="N6">
-        <v>1906063.13</v>
+        <v>1904728.6</v>
       </c>
       <c r="O6">
-        <v>2276315.27</v>
+        <v>202107.02</v>
       </c>
       <c r="P6">
-        <v>135833.51</v>
+        <v>196858.56</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>107250000</v>
       </c>
       <c r="I7">
-        <v>2532338.9300000002</v>
+        <v>3091469.42</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>31654236.66</v>
+        <v>26792734.940000001</v>
       </c>
       <c r="L7">
-        <v>29.51</v>
+        <v>24.98</v>
       </c>
       <c r="M7">
-        <v>1266169.47</v>
+        <v>1030489.81</v>
       </c>
       <c r="N7">
-        <v>4552941.79</v>
+        <v>4528631.76</v>
       </c>
       <c r="O7">
-        <v>11745242.85</v>
+        <v>2298353.0699999998</v>
       </c>
       <c r="P7">
-        <v>8063949.9900000002</v>
+        <v>938776.37</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>48750000</v>
       </c>
       <c r="I8">
-        <v>1002482.67</v>
+        <v>1141531.68</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>12531033.41</v>
+        <v>9893274.5800000001</v>
       </c>
       <c r="L8">
-        <v>25.7</v>
+        <v>20.29</v>
       </c>
       <c r="M8">
-        <v>501241.34</v>
+        <v>380510.56</v>
       </c>
       <c r="N8">
-        <v>2075979.01</v>
+        <v>2069933.41</v>
       </c>
       <c r="O8">
-        <v>3553038.26</v>
+        <v>710677.3</v>
       </c>
       <c r="P8">
-        <v>173248.02</v>
+        <v>1454844.85</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>39.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-07_1728 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBE98E2D-FAA0-41F6-A6CA-CAF586BD6415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E109CE96-4B85-4A0B-B8D2-A689A807CC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -659,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>544961.92000000004</v>
+        <v>577912.55000000005</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2724809.59</v>
+        <v>2407968.96</v>
       </c>
       <c r="L2">
-        <v>31.39</v>
+        <v>27.74</v>
       </c>
       <c r="M2">
-        <v>108992.38</v>
+        <v>96318.76</v>
       </c>
       <c r="N2">
-        <v>406751.9</v>
+        <v>426425.66</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>40005.5</v>
       </c>
       <c r="P2">
-        <v>319579.2</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>12402055.24</v>
+        <v>13648237.82</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>62010276.210000001</v>
+        <v>56867657.600000001</v>
       </c>
       <c r="L3">
-        <v>101.13</v>
+        <v>92.74</v>
       </c>
       <c r="M3">
-        <v>2480411.0499999998</v>
+        <v>2274706.2999999998</v>
       </c>
       <c r="N3">
-        <v>2445897.2400000002</v>
+        <v>2509040.11</v>
       </c>
       <c r="O3">
-        <v>2419878.06</v>
+        <v>5163141.7699999996</v>
       </c>
       <c r="P3">
-        <v>789240.23</v>
+        <v>554759.04</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>16932880.120000001</v>
+        <v>25319468.550000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>84664400.590000004</v>
+        <v>105497785.62</v>
       </c>
       <c r="L4">
-        <v>65.13</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="M4">
-        <v>3386576.02</v>
+        <v>4219911.42</v>
       </c>
       <c r="N4">
-        <v>5653355.9900000002</v>
+        <v>5509501.6600000001</v>
       </c>
       <c r="O4">
-        <v>10429780.050000001</v>
+        <v>2218349.9</v>
       </c>
       <c r="P4">
-        <v>4979037.34</v>
+        <v>1268157.78</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,19 +825,19 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2012763.72</v>
+        <v>1677303.1</v>
       </c>
       <c r="L5">
-        <v>20.64</v>
+        <v>17.2</v>
       </c>
       <c r="M5">
-        <v>80510.55</v>
+        <v>67092.12</v>
       </c>
       <c r="N5">
-        <v>467372.36</v>
+        <v>491970.91</v>
       </c>
       <c r="O5">
-        <v>389041.16</v>
+        <v>21094.7</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -871,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>5152447.1500000004</v>
+        <v>5298112.41</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>25762235.760000002</v>
+        <v>22075468.370000001</v>
       </c>
       <c r="L6">
-        <v>79.27</v>
+        <v>67.92</v>
       </c>
       <c r="M6">
-        <v>1030489.43</v>
+        <v>883018.73</v>
       </c>
       <c r="N6">
-        <v>1367377.64</v>
+        <v>1431678.29</v>
       </c>
       <c r="O6">
-        <v>329124.67</v>
+        <v>4297326.75</v>
       </c>
       <c r="P6">
-        <v>198786.36</v>
+        <v>549412.25</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>6014847.8899999997</v>
+        <v>6781439.6600000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>30074239.469999999</v>
+        <v>28255998.59</v>
       </c>
       <c r="L7">
-        <v>26.44</v>
+        <v>24.84</v>
       </c>
       <c r="M7">
-        <v>1202969.58</v>
+        <v>1130239.94</v>
       </c>
       <c r="N7">
-        <v>5386757.6100000003</v>
+        <v>5629924.2300000004</v>
       </c>
       <c r="O7">
-        <v>242815.89</v>
+        <v>658011.37</v>
       </c>
       <c r="P7">
-        <v>696951.33</v>
+        <v>8393371.9900000002</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -977,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>1604564.57</v>
+        <v>1546882.92</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>8022822.8300000001</v>
+        <v>6445345.5099999998</v>
       </c>
       <c r="L8">
-        <v>20.57</v>
+        <v>16.53</v>
       </c>
       <c r="M8">
-        <v>320912.90999999997</v>
+        <v>257813.82</v>
       </c>
       <c r="N8">
-        <v>1869771.77</v>
+        <v>1971216.69</v>
       </c>
       <c r="O8">
-        <v>519079.97</v>
+        <v>407749.33</v>
       </c>
       <c r="P8">
-        <v>3855929.99</v>
+        <v>732484.06</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1102,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1128,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1180,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-08_1713 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E109CE96-4B85-4A0B-B8D2-A689A807CC7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{84A65529-9B02-4326-9D5F-4A2CD9316D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -666,19 +665,19 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2407968.96</v>
+        <v>2063973.39</v>
       </c>
       <c r="L2">
-        <v>27.74</v>
+        <v>23.78</v>
       </c>
       <c r="M2">
-        <v>96318.76</v>
+        <v>82558.94</v>
       </c>
       <c r="N2">
-        <v>426425.66</v>
+        <v>450115.97</v>
       </c>
       <c r="O2">
-        <v>40005.5</v>
+        <v>-2846.54</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>13648237.82</v>
+        <v>19297599.25</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>56867657.600000001</v>
+        <v>68919997.310000002</v>
       </c>
       <c r="L3">
-        <v>92.74</v>
+        <v>112.39</v>
       </c>
       <c r="M3">
-        <v>2274706.2999999998</v>
+        <v>2756799.89</v>
       </c>
       <c r="N3">
-        <v>2509040.11</v>
+        <v>2334577.8199999998</v>
       </c>
       <c r="O3">
-        <v>5163141.7699999996</v>
+        <v>251569.42</v>
       </c>
       <c r="P3">
-        <v>554759.04</v>
+        <v>734455.9</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>25319468.550000001</v>
+        <v>26932540.640000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>105497785.62</v>
+        <v>96187645.150000006</v>
       </c>
       <c r="L4">
-        <v>81.150000000000006</v>
+        <v>73.989999999999995</v>
       </c>
       <c r="M4">
-        <v>4219911.42</v>
+        <v>3847505.81</v>
       </c>
       <c r="N4">
-        <v>5509501.6600000001</v>
+        <v>5725969.96</v>
       </c>
       <c r="O4">
-        <v>2218349.9</v>
+        <v>1681446.15</v>
       </c>
       <c r="P4">
-        <v>1268157.78</v>
+        <v>15584396.4</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +824,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1677303.1</v>
+        <v>1437688.37</v>
       </c>
       <c r="L5">
-        <v>17.2</v>
+        <v>14.75</v>
       </c>
       <c r="M5">
-        <v>67092.12</v>
+        <v>57507.53</v>
       </c>
       <c r="N5">
-        <v>491970.91</v>
+        <v>519302.63</v>
       </c>
       <c r="O5">
-        <v>21094.7</v>
+        <v>285080.27</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>109782</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>5298112.41</v>
+        <v>5435906.0099999998</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>22075468.370000001</v>
+        <v>19413950.039999999</v>
       </c>
       <c r="L6">
-        <v>67.92</v>
+        <v>59.74</v>
       </c>
       <c r="M6">
-        <v>883018.73</v>
+        <v>776558</v>
       </c>
       <c r="N6">
-        <v>1431678.29</v>
+        <v>1503560.78</v>
       </c>
       <c r="O6">
-        <v>4297326.75</v>
+        <v>457101.09</v>
       </c>
       <c r="P6">
-        <v>549412.25</v>
+        <v>1055507.6000000001</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>6781439.6600000001</v>
+        <v>7374265.7999999998</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>28255998.59</v>
+        <v>26336663.57</v>
       </c>
       <c r="L7">
-        <v>24.84</v>
+        <v>23.15</v>
       </c>
       <c r="M7">
-        <v>1130239.94</v>
+        <v>1053466.54</v>
       </c>
       <c r="N7">
-        <v>5629924.2300000004</v>
+        <v>5909763.0099999998</v>
       </c>
       <c r="O7">
-        <v>658011.37</v>
+        <v>404109.01</v>
       </c>
       <c r="P7">
-        <v>8393371.9900000002</v>
+        <v>16664832.34</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>1546882.92</v>
+        <v>1945742.48</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>6445345.5099999998</v>
+        <v>6949080.2800000003</v>
       </c>
       <c r="L8">
-        <v>16.53</v>
+        <v>17.82</v>
       </c>
       <c r="M8">
-        <v>257813.82</v>
+        <v>277963.21000000002</v>
       </c>
       <c r="N8">
-        <v>1971216.69</v>
+        <v>2058569.86</v>
       </c>
       <c r="O8">
-        <v>407749.33</v>
+        <v>219976.32000000001</v>
       </c>
       <c r="P8">
-        <v>732484.06</v>
+        <v>722618.73</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1154,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>0.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-11_1802 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24851FF7-3457-4042-8173-4687DF2120B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFC5FE34-825F-4C20-A4E0-3433DE441431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,8 +572,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="9" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -660,28 +659,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2281048.87</v>
+        <v>2255628.77</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>6336246.8499999996</v>
+        <v>5639071.9199999999</v>
       </c>
       <c r="L2">
-        <v>73</v>
+        <v>64.97</v>
       </c>
       <c r="M2">
-        <v>253449.87</v>
+        <v>225562.88</v>
       </c>
       <c r="N2">
-        <v>399934.45</v>
+        <v>428291.42</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>73717.86</v>
       </c>
       <c r="P2">
-        <v>141131.70000000001</v>
+        <v>49027.62</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +712,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>21151641.390000001</v>
+        <v>21461811.100000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>58754559.420000002</v>
+        <v>53654527.759999998</v>
       </c>
       <c r="L3">
-        <v>95.82</v>
+        <v>87.5</v>
       </c>
       <c r="M3">
-        <v>2350182.38</v>
+        <v>2146181.11</v>
       </c>
       <c r="N3">
-        <v>2510522.41</v>
+        <v>2657212.59</v>
       </c>
       <c r="O3">
-        <v>343979.88</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>20222919.98</v>
+        <v>6482530.5899999999</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +765,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>55640813.560000002</v>
+        <v>57835761.200000003</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>154557815.44</v>
+        <v>144589403</v>
       </c>
       <c r="L4">
-        <v>118.89</v>
+        <v>111.22</v>
       </c>
       <c r="M4">
-        <v>6182312.6200000001</v>
+        <v>5783576.1200000001</v>
       </c>
       <c r="N4">
-        <v>4647449.1500000004</v>
+        <v>4810949.25</v>
       </c>
       <c r="O4">
-        <v>1335695.71</v>
+        <v>303709.89</v>
       </c>
       <c r="P4">
-        <v>4205985.53</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +818,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>452021.63</v>
+        <v>2228327.59</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1255615.6399999999</v>
+        <v>5570818.9800000004</v>
       </c>
       <c r="L5">
-        <v>12.88</v>
+        <v>57.14</v>
       </c>
       <c r="M5">
-        <v>50224.63</v>
+        <v>222832.76</v>
       </c>
       <c r="N5">
-        <v>581123.65</v>
+        <v>501444.83</v>
       </c>
       <c r="O5">
-        <v>68302.98</v>
+        <v>28074.79</v>
       </c>
       <c r="P5">
-        <v>197119.22</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +871,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>7015589.8700000001</v>
+        <v>9116071.0199999996</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>19487749.649999999</v>
+        <v>22790177.550000001</v>
       </c>
       <c r="L6">
-        <v>59.96</v>
+        <v>70.12</v>
       </c>
       <c r="M6">
-        <v>779509.99</v>
+        <v>911607.1</v>
       </c>
       <c r="N6">
-        <v>1592775.63</v>
+        <v>1558928.6</v>
       </c>
       <c r="O6">
-        <v>127705.67</v>
+        <v>22110.77</v>
       </c>
       <c r="P6">
-        <v>202107.02</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +924,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>9678965.5299999993</v>
+        <v>10307300.060000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>26886015.370000001</v>
+        <v>25768250.149999999</v>
       </c>
       <c r="L7">
-        <v>23.64</v>
+        <v>22.65</v>
       </c>
       <c r="M7">
-        <v>1075440.6100000001</v>
+        <v>1030730.01</v>
       </c>
       <c r="N7">
-        <v>6504439.6500000004</v>
+        <v>6896180</v>
       </c>
       <c r="O7">
-        <v>708960.31</v>
+        <v>2214418.16</v>
       </c>
       <c r="P7">
-        <v>2298353.0699999998</v>
+        <v>535067.81000000006</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +977,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>4424528.7</v>
+        <v>7996391.0599999996</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>12290357.51</v>
+        <v>19990977.649999999</v>
       </c>
       <c r="L8">
-        <v>31.51</v>
+        <v>51.26</v>
       </c>
       <c r="M8">
-        <v>491614.3</v>
+        <v>799639.11</v>
       </c>
       <c r="N8">
-        <v>2160966.96</v>
+        <v>2066907.26</v>
       </c>
       <c r="O8">
-        <v>463032.88</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>710677.3</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1076,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1102,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1128,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1180,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>24.1</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1284,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>